<commit_message>
add data, script testing
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/Desktop/reading/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/Desktop/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C114A0FF-60C5-084E-A959-E2A36EC0F53E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FFFF06F-71AA-D14F-8EA5-0BEFF77FF6F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15120" yWindow="680" windowWidth="15120" windowHeight="16880" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="-20" yWindow="680" windowWidth="15140" windowHeight="16880" activeTab="1" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="82">
   <si>
     <t>book_id</t>
   </si>
@@ -239,15 +239,58 @@
   </si>
   <si>
     <t>full</t>
+  </si>
+  <si>
+    <t>date_started</t>
+  </si>
+  <si>
+    <t>date_finished</t>
+  </si>
+  <si>
+    <t>The Stone Door</t>
+  </si>
+  <si>
+    <t>A Month in the Country</t>
+  </si>
+  <si>
+    <t>Leonora Carrington</t>
+  </si>
+  <si>
+    <t>J.L. Carr</t>
+  </si>
+  <si>
+    <t>Miguel de Cervantes</t>
+  </si>
+  <si>
+    <t>classics</t>
+  </si>
+  <si>
+    <t>untimed</t>
+  </si>
+  <si>
+    <t>Don Quixote II</t>
+  </si>
+  <si>
+    <t>The Tolkien Reader</t>
+  </si>
+  <si>
+    <t>J.R.R. Tolkien</t>
+  </si>
+  <si>
+    <t>fantasy</t>
+  </si>
+  <si>
+    <t>no-curve</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm\ "/>
     <numFmt numFmtId="165" formatCode="[mm]:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -292,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -300,7 +343,8 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -635,19 +679,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -675,93 +722,262 @@
       <c r="I1" s="1" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J1" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2">
         <f>ROW() - 1</f>
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>70</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="E2">
-        <v>1982</v>
+        <v>1977</v>
       </c>
       <c r="F2" t="s">
         <v>16</v>
       </c>
       <c r="G2">
-        <v>449</v>
+        <v>136</v>
       </c>
       <c r="H2">
-        <v>136496</v>
+        <v>38544</v>
       </c>
       <c r="I2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+      <c r="J2" s="7">
+        <v>46019</v>
+      </c>
+      <c r="K2" s="7">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
+        <f t="shared" ref="A3:A4" si="0">ROW() - 1</f>
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>73</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="E3">
-        <v>1986</v>
+        <v>1980</v>
       </c>
       <c r="F3" t="s">
         <v>16</v>
       </c>
       <c r="G3">
-        <v>499</v>
+        <v>160</v>
       </c>
       <c r="H3">
-        <v>142714</v>
+        <v>36949</v>
       </c>
       <c r="I3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+      <c r="J3" s="7">
+        <v>46024</v>
+      </c>
+      <c r="K3" s="7">
+        <v>46026</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="D4" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="E4">
-        <v>1978</v>
+        <v>1615</v>
       </c>
       <c r="F4" t="s">
         <v>16</v>
       </c>
       <c r="G4">
+        <v>487</v>
+      </c>
+      <c r="H4">
+        <v>205432</v>
+      </c>
+      <c r="I4" t="s">
+        <v>76</v>
+      </c>
+      <c r="J4" s="7">
+        <v>46027</v>
+      </c>
+      <c r="K4" s="7">
+        <v>46032</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <f>ROW() - 1</f>
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5">
+        <v>1982</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5">
+        <v>449</v>
+      </c>
+      <c r="H5">
+        <v>136496</v>
+      </c>
+      <c r="I5" t="s">
+        <v>67</v>
+      </c>
+      <c r="J5" s="7">
+        <v>46035</v>
+      </c>
+      <c r="K5" s="7">
+        <v>46045</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <f t="shared" ref="A6:A7" si="1">ROW() - 1</f>
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6">
+        <v>1986</v>
+      </c>
+      <c r="F6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6">
+        <v>499</v>
+      </c>
+      <c r="H6">
+        <v>142714</v>
+      </c>
+      <c r="I6" t="s">
+        <v>67</v>
+      </c>
+      <c r="J6" s="7">
+        <v>46047</v>
+      </c>
+      <c r="K6" s="7">
+        <v>46055</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7">
+        <v>1978</v>
+      </c>
+      <c r="F7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7">
         <v>210</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H7">
         <v>53760</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I7" t="s">
         <v>67</v>
+      </c>
+      <c r="J7" s="7">
+        <v>46058</v>
+      </c>
+      <c r="K7" s="7">
+        <v>46064</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E8">
+        <v>1966</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8">
+        <v>266</v>
+      </c>
+      <c r="H8" t="s">
+        <v>63</v>
+      </c>
+      <c r="I8" t="s">
+        <v>81</v>
+      </c>
+      <c r="J8" s="7">
+        <v>46067</v>
+      </c>
+      <c r="K8" s="7">
+        <v>46085</v>
       </c>
     </row>
   </sheetData>
@@ -771,7 +987,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -809,7 +1025,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C2" s="3">
         <v>46035.930555555555</v>
@@ -826,11 +1042,11 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3">
-        <f t="shared" ref="A3:A33" si="0">ROW() - 1</f>
+        <f t="shared" ref="A3:A51" si="0">ROW() - 1</f>
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C3" s="4">
         <v>46036.619444444441</v>
@@ -851,7 +1067,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C4" s="4">
         <v>46037.911111111112</v>
@@ -872,7 +1088,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C5" s="4">
         <v>46038.941666666666</v>
@@ -893,7 +1109,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C6" s="4">
         <v>46039.911111111112</v>
@@ -914,7 +1130,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C7" s="4">
         <v>46040.961805555555</v>
@@ -935,7 +1151,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C8" s="4">
         <v>46041.897916666669</v>
@@ -956,7 +1172,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C9" s="3">
         <v>46042.923611111109</v>
@@ -977,7 +1193,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C10" s="3">
         <v>46043.914583333331</v>
@@ -998,7 +1214,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C11" s="3">
         <v>46044.347222222219</v>
@@ -1019,7 +1235,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C12" s="3">
         <v>46044.919444444444</v>
@@ -1040,7 +1256,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C13" s="3">
         <v>46045.881944444445</v>
@@ -1061,7 +1277,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C14" s="3">
         <v>46047.862500000003</v>
@@ -1082,7 +1298,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C15" s="3">
         <v>46048.916666666664</v>
@@ -1103,7 +1319,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C16" s="3">
         <v>46049.9375</v>
@@ -1124,7 +1340,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C17" s="3">
         <v>46050.935416666667</v>
@@ -1145,7 +1361,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C18" s="3">
         <v>46051.929166666669</v>
@@ -1166,7 +1382,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C19" s="3">
         <v>46052.620138888888</v>
@@ -1187,7 +1403,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C20" s="3">
         <v>46053.595833333333</v>
@@ -1208,7 +1424,7 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C21" s="3">
         <v>46053.922222222223</v>
@@ -1229,7 +1445,7 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C22" s="4">
         <v>46054.505555555559</v>
@@ -1250,7 +1466,7 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C23" s="3">
         <v>46054.92083333333</v>
@@ -1271,7 +1487,7 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C24" s="3">
         <v>46055.686111111114</v>
@@ -1292,7 +1508,7 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C25" s="3">
         <v>46055.761805555558</v>
@@ -1313,7 +1529,7 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C26" s="3">
         <v>46059.930555555555</v>
@@ -1334,7 +1550,7 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C27" s="3">
         <v>46060.914583333331</v>
@@ -1355,7 +1571,7 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C28" s="3">
         <v>46061.722916666666</v>
@@ -1376,7 +1592,7 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C29" s="3">
         <v>46061.982638888891</v>
@@ -1397,7 +1613,7 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C30" s="3">
         <v>46062.960416666669</v>
@@ -1418,7 +1634,7 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C31" s="3">
         <v>46063.956250000003</v>
@@ -1439,7 +1655,7 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C32" s="3">
         <v>46063.956250000003</v>
@@ -1460,7 +1676,7 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C33" s="4">
         <v>46064.916666666664</v>
@@ -1473,6 +1689,321 @@
       </c>
       <c r="F33" s="6">
         <v>1.0208333333333333E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>7</v>
+      </c>
+      <c r="C34" s="3">
+        <v>46067.939583333333</v>
+      </c>
+      <c r="D34" t="s">
+        <v>63</v>
+      </c>
+      <c r="E34" t="s">
+        <v>63</v>
+      </c>
+      <c r="F34" s="6">
+        <v>1.5613425925925926E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>7</v>
+      </c>
+      <c r="C35" s="3">
+        <v>46072.52847222222</v>
+      </c>
+      <c r="D35" t="s">
+        <v>63</v>
+      </c>
+      <c r="E35" t="s">
+        <v>63</v>
+      </c>
+      <c r="F35" s="6">
+        <v>1.8240740740740741E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>7</v>
+      </c>
+      <c r="C36" s="3">
+        <v>46072.940972222219</v>
+      </c>
+      <c r="D36" t="s">
+        <v>63</v>
+      </c>
+      <c r="E36" t="s">
+        <v>63</v>
+      </c>
+      <c r="F36" s="6">
+        <v>1.4039351851851851E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>7</v>
+      </c>
+      <c r="C37" s="3">
+        <v>46073.943055555559</v>
+      </c>
+      <c r="D37" t="s">
+        <v>63</v>
+      </c>
+      <c r="E37" t="s">
+        <v>63</v>
+      </c>
+      <c r="F37" s="6">
+        <v>1.1493055555555555E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>7</v>
+      </c>
+      <c r="C38" s="3">
+        <v>46074.601388888892</v>
+      </c>
+      <c r="D38" t="s">
+        <v>63</v>
+      </c>
+      <c r="E38" t="s">
+        <v>63</v>
+      </c>
+      <c r="F38" s="6">
+        <v>1.3171296296296296E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>7</v>
+      </c>
+      <c r="C39" s="3">
+        <v>46075.9375</v>
+      </c>
+      <c r="D39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E39" t="s">
+        <v>63</v>
+      </c>
+      <c r="F39" s="6">
+        <v>2.1435185185185186E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>7</v>
+      </c>
+      <c r="C40" s="3">
+        <v>46076.821527777778</v>
+      </c>
+      <c r="D40" t="s">
+        <v>63</v>
+      </c>
+      <c r="E40" t="s">
+        <v>63</v>
+      </c>
+      <c r="F40" s="6">
+        <v>1.224537037037037E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>7</v>
+      </c>
+      <c r="C41" s="3">
+        <v>46077.96597222222</v>
+      </c>
+      <c r="D41" t="s">
+        <v>63</v>
+      </c>
+      <c r="E41" t="s">
+        <v>63</v>
+      </c>
+      <c r="F41" s="6">
+        <v>3.9351851851851848E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>7</v>
+      </c>
+      <c r="C42" s="3">
+        <v>46079.945138888892</v>
+      </c>
+      <c r="D42" t="s">
+        <v>63</v>
+      </c>
+      <c r="E42" t="s">
+        <v>63</v>
+      </c>
+      <c r="F42" s="6">
+        <v>1.0694444444444444E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>7</v>
+      </c>
+      <c r="C43" s="3">
+        <v>46080.617361111108</v>
+      </c>
+      <c r="D43" t="s">
+        <v>63</v>
+      </c>
+      <c r="E43" t="s">
+        <v>63</v>
+      </c>
+      <c r="F43" s="6">
+        <v>1.9085648148148147E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>7</v>
+      </c>
+      <c r="C44" s="3">
+        <v>46080.921527777777</v>
+      </c>
+      <c r="D44" t="s">
+        <v>63</v>
+      </c>
+      <c r="E44" t="s">
+        <v>63</v>
+      </c>
+      <c r="F44" s="6">
+        <v>1.2314814814814815E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>7</v>
+      </c>
+      <c r="C45" s="3">
+        <v>46081.799305555556</v>
+      </c>
+      <c r="D45" t="s">
+        <v>63</v>
+      </c>
+      <c r="E45" t="s">
+        <v>63</v>
+      </c>
+      <c r="F45" s="6">
+        <v>7.3032407407407404E-3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>7</v>
+      </c>
+      <c r="C46" s="3">
+        <v>46081.947222222225</v>
+      </c>
+      <c r="D46" t="s">
+        <v>63</v>
+      </c>
+      <c r="E46" t="s">
+        <v>63</v>
+      </c>
+      <c r="F46" s="6">
+        <v>8.5879629629629622E-3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>7</v>
+      </c>
+      <c r="C47" s="3">
+        <v>46084.95</v>
+      </c>
+      <c r="D47" t="s">
+        <v>63</v>
+      </c>
+      <c r="E47" t="s">
+        <v>63</v>
+      </c>
+      <c r="F47" s="6">
+        <v>7.4999999999999997E-3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>7</v>
+      </c>
+      <c r="C48" s="3">
+        <v>46085.945833333331</v>
+      </c>
+      <c r="D48" t="s">
+        <v>63</v>
+      </c>
+      <c r="E48" t="s">
+        <v>63</v>
+      </c>
+      <c r="F48" s="6">
+        <v>1.1516203703703704E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1515,7 +2046,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -1533,7 +2064,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -1551,7 +2082,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -1569,7 +2100,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -1587,7 +2118,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C6">
         <v>5</v>
@@ -1605,7 +2136,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C7">
         <v>6</v>
@@ -1623,7 +2154,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C8">
         <v>7</v>
@@ -1641,7 +2172,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C9">
         <v>8</v>
@@ -1659,7 +2190,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C10">
         <v>9</v>
@@ -1677,7 +2208,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C11">
         <v>10</v>
@@ -1695,7 +2226,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C12">
         <v>11</v>
@@ -1713,7 +2244,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C13">
         <v>12</v>
@@ -1731,7 +2262,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C14">
         <v>13</v>
@@ -1749,7 +2280,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C15">
         <v>14</v>
@@ -1767,7 +2298,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C16">
         <v>15</v>
@@ -1785,7 +2316,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C17">
         <v>16</v>
@@ -1803,7 +2334,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C18">
         <v>17</v>
@@ -1821,7 +2352,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C19">
         <v>18</v>
@@ -1839,7 +2370,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C20">
         <v>19</v>
@@ -1857,7 +2388,7 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C21">
         <v>20</v>
@@ -1875,7 +2406,7 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -1893,7 +2424,7 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C23">
         <v>2</v>
@@ -1911,7 +2442,7 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C24">
         <v>3</v>
@@ -1929,7 +2460,7 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C25">
         <v>4</v>
@@ -1947,7 +2478,7 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C26">
         <v>5</v>
@@ -1965,7 +2496,7 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C27">
         <v>6</v>
@@ -1983,7 +2514,7 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C28">
         <v>7</v>
@@ -2001,7 +2532,7 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C29">
         <v>8</v>
@@ -2019,7 +2550,7 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C30">
         <v>9</v>
@@ -2037,7 +2568,7 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C31">
         <v>10</v>
@@ -2055,7 +2586,7 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C32">
         <v>11</v>
@@ -2073,7 +2604,7 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C33">
         <v>12</v>
@@ -2091,7 +2622,7 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C34">
         <v>13</v>
@@ -2109,7 +2640,7 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C35">
         <v>14</v>
@@ -2127,7 +2658,7 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C36">
         <v>15</v>
@@ -2145,7 +2676,7 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C37">
         <v>16</v>
@@ -2163,7 +2694,7 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C38">
         <v>17</v>
@@ -2181,7 +2712,7 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C39">
         <v>18</v>
@@ -2199,7 +2730,7 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C40">
         <v>19</v>
@@ -2217,7 +2748,7 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C41">
         <v>20</v>
@@ -2235,7 +2766,7 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C42">
         <v>21</v>
@@ -2253,7 +2784,7 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -2272,7 +2803,7 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C44">
         <v>2</v>
@@ -2291,7 +2822,7 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C45">
         <v>3</v>
@@ -2310,7 +2841,7 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C46">
         <v>4</v>
@@ -2329,7 +2860,7 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C47">
         <v>5</v>
@@ -2348,7 +2879,7 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C48">
         <v>6</v>
@@ -2367,7 +2898,7 @@
         <v>48</v>
       </c>
       <c r="B49">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C49">
         <v>7</v>
@@ -2386,7 +2917,7 @@
         <v>49</v>
       </c>
       <c r="B50">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C50">
         <v>8</v>
@@ -2405,7 +2936,7 @@
         <v>50</v>
       </c>
       <c r="B51">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C51">
         <v>9</v>
@@ -2424,7 +2955,7 @@
         <v>51</v>
       </c>
       <c r="B52">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C52">
         <v>10</v>
@@ -2443,7 +2974,7 @@
         <v>52</v>
       </c>
       <c r="B53">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C53">
         <v>11</v>
@@ -2462,7 +2993,7 @@
         <v>53</v>
       </c>
       <c r="B54">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C54">
         <v>12</v>
@@ -2481,7 +3012,7 @@
         <v>54</v>
       </c>
       <c r="B55">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C55">
         <v>13</v>
@@ -2500,7 +3031,7 @@
         <v>55</v>
       </c>
       <c r="B56">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C56">
         <v>14</v>
@@ -2519,7 +3050,7 @@
         <v>56</v>
       </c>
       <c r="B57">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C57">
         <v>15</v>
@@ -2538,7 +3069,7 @@
         <v>57</v>
       </c>
       <c r="B58">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C58">
         <v>16</v>
@@ -2557,7 +3088,7 @@
         <v>58</v>
       </c>
       <c r="B59">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C59">
         <v>17</v>
@@ -2576,7 +3107,7 @@
         <v>59</v>
       </c>
       <c r="B60">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C60">
         <v>18</v>
@@ -2595,7 +3126,7 @@
         <v>60</v>
       </c>
       <c r="B61">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C61">
         <v>19</v>
@@ -2614,7 +3145,7 @@
         <v>61</v>
       </c>
       <c r="B62">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C62">
         <v>20</v>
@@ -2633,7 +3164,7 @@
         <v>62</v>
       </c>
       <c r="B63">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C63">
         <v>21</v>
@@ -2652,7 +3183,7 @@
         <v>63</v>
       </c>
       <c r="B64">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C64">
         <v>22</v>
@@ -2671,7 +3202,7 @@
         <v>64</v>
       </c>
       <c r="B65">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C65">
         <v>23</v>
@@ -2690,7 +3221,7 @@
         <v>65</v>
       </c>
       <c r="B66">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C66">
         <v>24</v>
@@ -2709,7 +3240,7 @@
         <v>66</v>
       </c>
       <c r="B67">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C67">
         <v>25</v>

</xml_diff>

<commit_message>
update log (baby driver)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/Desktop/reading-analysis/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/Stuff/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7395A5A3-04FE-4744-92AF-F4D04E25D084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B986209A-4126-B448-80E0-6553C44A0A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="15140" windowHeight="16880" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="-20" yWindow="680" windowWidth="15040" windowHeight="18980" activeTab="2" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="108">
   <si>
     <t>book_id</t>
   </si>
@@ -290,6 +290,75 @@
   </si>
   <si>
     <t>11 (Epilogue)</t>
+  </si>
+  <si>
+    <t>Edward Johnston</t>
+  </si>
+  <si>
+    <t>Priscilla Johnston</t>
+  </si>
+  <si>
+    <t>biography</t>
+  </si>
+  <si>
+    <t>Portrait</t>
+  </si>
+  <si>
+    <t>Ancestry</t>
+  </si>
+  <si>
+    <t>Childhood</t>
+  </si>
+  <si>
+    <t>Interlude</t>
+  </si>
+  <si>
+    <t>The Beginning, 1898</t>
+  </si>
+  <si>
+    <t>The First Class, 1898-1901</t>
+  </si>
+  <si>
+    <t>Greta, 1901</t>
+  </si>
+  <si>
+    <t>Lincoln's Inn, 1902-1903</t>
+  </si>
+  <si>
+    <t>Gray's Inn, 1903-1905</t>
+  </si>
+  <si>
+    <t>Hammersmith, 1905-1912</t>
+  </si>
+  <si>
+    <t>Ditchling, 1912-1916</t>
+  </si>
+  <si>
+    <t>Halletts, 1916-1919</t>
+  </si>
+  <si>
+    <t>Cleves, 1920-1927</t>
+  </si>
+  <si>
+    <t>Late Working Years, 1928-1935</t>
+  </si>
+  <si>
+    <t>The Hermit, 1936-1944</t>
+  </si>
+  <si>
+    <t>word_count_type</t>
+  </si>
+  <si>
+    <t>exact</t>
+  </si>
+  <si>
+    <t>estimate</t>
+  </si>
+  <si>
+    <t>Baby Driver</t>
+  </si>
+  <si>
+    <t>Jan Kerouac</t>
   </si>
 </sst>
 </file>
@@ -344,7 +413,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -355,6 +424,8 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -689,7 +760,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -699,12 +770,13 @@
     <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.33203125" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -730,16 +802,19 @@
         <v>65</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="L1" s="8" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2">
         <f>ROW() - 1</f>
         <v>1</v>
@@ -766,16 +841,19 @@
         <v>38544</v>
       </c>
       <c r="I2" t="s">
+        <v>104</v>
+      </c>
+      <c r="J2" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="7">
+      <c r="K2" s="7">
         <v>46019</v>
       </c>
-      <c r="K2" s="7">
+      <c r="L2" s="7">
         <v>46023</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3">
         <f t="shared" ref="A3:A4" si="0">ROW() - 1</f>
         <v>2</v>
@@ -802,16 +880,19 @@
         <v>36949</v>
       </c>
       <c r="I3" t="s">
+        <v>104</v>
+      </c>
+      <c r="J3" t="s">
         <v>76</v>
       </c>
-      <c r="J3" s="7">
+      <c r="K3" s="7">
         <v>46024</v>
       </c>
-      <c r="K3" s="7">
+      <c r="L3" s="7">
         <v>46026</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -838,16 +919,19 @@
         <v>205432</v>
       </c>
       <c r="I4" t="s">
+        <v>104</v>
+      </c>
+      <c r="J4" t="s">
         <v>76</v>
       </c>
-      <c r="J4" s="7">
+      <c r="K4" s="7">
         <v>46027</v>
       </c>
-      <c r="K4" s="7">
+      <c r="L4" s="7">
         <v>46032</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5">
         <f>ROW() - 1</f>
         <v>4</v>
@@ -874,16 +958,19 @@
         <v>136496</v>
       </c>
       <c r="I5" t="s">
+        <v>104</v>
+      </c>
+      <c r="J5" t="s">
         <v>67</v>
       </c>
-      <c r="J5" s="7">
+      <c r="K5" s="7">
         <v>46035</v>
       </c>
-      <c r="K5" s="7">
+      <c r="L5" s="7">
         <v>46045</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6">
         <f t="shared" ref="A6:A7" si="1">ROW() - 1</f>
         <v>5</v>
@@ -910,16 +997,19 @@
         <v>142714</v>
       </c>
       <c r="I6" t="s">
+        <v>104</v>
+      </c>
+      <c r="J6" t="s">
         <v>67</v>
       </c>
-      <c r="J6" s="7">
+      <c r="K6" s="7">
         <v>46047</v>
       </c>
-      <c r="K6" s="7">
+      <c r="L6" s="7">
         <v>46055</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7">
         <f t="shared" si="1"/>
         <v>6</v>
@@ -946,16 +1036,19 @@
         <v>53760</v>
       </c>
       <c r="I7" t="s">
+        <v>104</v>
+      </c>
+      <c r="J7" t="s">
         <v>67</v>
       </c>
-      <c r="J7" s="7">
+      <c r="K7" s="7">
         <v>46058</v>
       </c>
-      <c r="K7" s="7">
+      <c r="L7" s="7">
         <v>46064</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -981,16 +1074,19 @@
         <v>63</v>
       </c>
       <c r="I8" t="s">
+        <v>63</v>
+      </c>
+      <c r="J8" t="s">
         <v>81</v>
       </c>
-      <c r="J8" s="7">
+      <c r="K8" s="7">
         <v>46067</v>
       </c>
-      <c r="K8" s="7">
+      <c r="L8" s="7">
         <v>46085</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1012,17 +1108,96 @@
       <c r="G9">
         <v>261</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9">
         <v>105626</v>
       </c>
       <c r="I9" t="s">
+        <v>104</v>
+      </c>
+      <c r="J9" t="s">
         <v>67</v>
       </c>
-      <c r="J9" s="7">
+      <c r="K9" s="7">
         <v>46089</v>
       </c>
-      <c r="K9" s="7">
+      <c r="L9" s="7">
         <v>46106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10">
+        <v>1959</v>
+      </c>
+      <c r="F10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10">
+        <v>310</v>
+      </c>
+      <c r="H10">
+        <v>105413</v>
+      </c>
+      <c r="I10" t="s">
+        <v>105</v>
+      </c>
+      <c r="J10" t="s">
+        <v>67</v>
+      </c>
+      <c r="K10" s="7">
+        <v>46107</v>
+      </c>
+      <c r="L10" s="7">
+        <v>46131</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" t="s">
+        <v>107</v>
+      </c>
+      <c r="D11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E11">
+        <v>1981</v>
+      </c>
+      <c r="F11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11">
+        <v>244</v>
+      </c>
+      <c r="H11">
+        <v>90974</v>
+      </c>
+      <c r="I11" t="s">
+        <v>104</v>
+      </c>
+      <c r="J11" t="s">
+        <v>67</v>
+      </c>
+      <c r="K11" s="7">
+        <v>46135</v>
+      </c>
+      <c r="L11" s="7">
+        <v>46147</v>
       </c>
     </row>
   </sheetData>
@@ -1032,7 +1207,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I102"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -1087,7 +1262,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3">
-        <f t="shared" ref="A3:A65" si="0">ROW() - 1</f>
+        <f t="shared" ref="A3:A66" si="0">ROW() - 1</f>
         <v>2</v>
       </c>
       <c r="B3">
@@ -2407,6 +2582,703 @@
       <c r="F65" s="6">
         <v>1.1122685185185185E-2</v>
       </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+      <c r="B66">
+        <v>9</v>
+      </c>
+      <c r="C66" s="3">
+        <v>46107.823611111111</v>
+      </c>
+      <c r="D66">
+        <v>15</v>
+      </c>
+      <c r="E66">
+        <v>24</v>
+      </c>
+      <c r="F66" s="6">
+        <v>9.1087962962962971E-3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <f t="shared" ref="A67:A98" si="1">ROW() - 1</f>
+        <v>66</v>
+      </c>
+      <c r="B67">
+        <v>9</v>
+      </c>
+      <c r="C67" s="3">
+        <v>46108.624305555553</v>
+      </c>
+      <c r="D67">
+        <v>24</v>
+      </c>
+      <c r="E67">
+        <v>41</v>
+      </c>
+      <c r="F67" s="6">
+        <v>1.5694444444444445E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <f t="shared" si="1"/>
+        <v>67</v>
+      </c>
+      <c r="B68">
+        <v>9</v>
+      </c>
+      <c r="C68" s="3">
+        <v>46111.502083333333</v>
+      </c>
+      <c r="D68">
+        <v>41</v>
+      </c>
+      <c r="E68">
+        <v>54</v>
+      </c>
+      <c r="F68" s="6">
+        <v>1.0208333333333333E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <f t="shared" si="1"/>
+        <v>68</v>
+      </c>
+      <c r="B69">
+        <v>9</v>
+      </c>
+      <c r="C69" s="3">
+        <v>46112.541666666664</v>
+      </c>
+      <c r="D69">
+        <v>54</v>
+      </c>
+      <c r="E69">
+        <v>66</v>
+      </c>
+      <c r="F69" s="6">
+        <v>1.1238425925925926E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <f t="shared" si="1"/>
+        <v>69</v>
+      </c>
+      <c r="B70">
+        <v>9</v>
+      </c>
+      <c r="C70" s="3">
+        <v>46112.820138888892</v>
+      </c>
+      <c r="D70">
+        <v>66</v>
+      </c>
+      <c r="E70">
+        <v>79</v>
+      </c>
+      <c r="F70" s="6">
+        <v>1.1388888888888889E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <f t="shared" si="1"/>
+        <v>70</v>
+      </c>
+      <c r="B71">
+        <v>9</v>
+      </c>
+      <c r="C71" s="3">
+        <v>46112.960416666669</v>
+      </c>
+      <c r="D71">
+        <v>79</v>
+      </c>
+      <c r="E71">
+        <v>98</v>
+      </c>
+      <c r="F71" s="6">
+        <v>1.8888888888888889E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <f t="shared" si="1"/>
+        <v>71</v>
+      </c>
+      <c r="B72">
+        <v>9</v>
+      </c>
+      <c r="C72" s="3">
+        <v>46114.463888888888</v>
+      </c>
+      <c r="D72">
+        <v>98</v>
+      </c>
+      <c r="E72">
+        <v>111</v>
+      </c>
+      <c r="F72" s="6">
+        <v>9.0277777777777769E-3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <f t="shared" si="1"/>
+        <v>72</v>
+      </c>
+      <c r="B73">
+        <v>9</v>
+      </c>
+      <c r="C73" s="3">
+        <v>46116.780555555553</v>
+      </c>
+      <c r="D73">
+        <v>111</v>
+      </c>
+      <c r="E73">
+        <v>129</v>
+      </c>
+      <c r="F73" s="6">
+        <v>1.8449074074074073E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <f t="shared" si="1"/>
+        <v>73</v>
+      </c>
+      <c r="B74">
+        <v>9</v>
+      </c>
+      <c r="C74" s="3">
+        <v>46117.963194444441</v>
+      </c>
+      <c r="D74">
+        <v>129</v>
+      </c>
+      <c r="E74">
+        <v>146</v>
+      </c>
+      <c r="F74" s="6">
+        <v>1.7743055555555557E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A75">
+        <f t="shared" si="1"/>
+        <v>74</v>
+      </c>
+      <c r="B75">
+        <v>9</v>
+      </c>
+      <c r="C75" s="3">
+        <v>46121.458333333336</v>
+      </c>
+      <c r="D75">
+        <v>146</v>
+      </c>
+      <c r="E75">
+        <v>167</v>
+      </c>
+      <c r="F75" s="6">
+        <v>1.7453703703703704E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A76">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+      <c r="B76">
+        <v>9</v>
+      </c>
+      <c r="C76" s="3">
+        <v>46121.991666666669</v>
+      </c>
+      <c r="D76">
+        <v>167</v>
+      </c>
+      <c r="E76">
+        <v>182</v>
+      </c>
+      <c r="F76" s="6">
+        <v>1.3159722222222222E-2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A77">
+        <f t="shared" si="1"/>
+        <v>76</v>
+      </c>
+      <c r="B77">
+        <v>9</v>
+      </c>
+      <c r="C77" s="3">
+        <v>46125.981944444444</v>
+      </c>
+      <c r="D77">
+        <v>182</v>
+      </c>
+      <c r="E77">
+        <v>198</v>
+      </c>
+      <c r="F77" s="6">
+        <v>1.5196759259259259E-2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A78">
+        <f t="shared" si="1"/>
+        <v>77</v>
+      </c>
+      <c r="B78">
+        <v>9</v>
+      </c>
+      <c r="C78" s="3">
+        <v>46126.959027777775</v>
+      </c>
+      <c r="D78">
+        <v>198</v>
+      </c>
+      <c r="E78">
+        <v>211</v>
+      </c>
+      <c r="F78" s="6">
+        <v>1.5150462962962963E-2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A79">
+        <f t="shared" si="1"/>
+        <v>78</v>
+      </c>
+      <c r="B79">
+        <v>9</v>
+      </c>
+      <c r="C79" s="3">
+        <v>46127.956250000003</v>
+      </c>
+      <c r="D79">
+        <v>211</v>
+      </c>
+      <c r="E79">
+        <v>228</v>
+      </c>
+      <c r="F79" s="6">
+        <v>1.4456018518518519E-2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A80">
+        <f t="shared" si="1"/>
+        <v>79</v>
+      </c>
+      <c r="B80">
+        <v>9</v>
+      </c>
+      <c r="C80" s="3">
+        <v>46128.464583333334</v>
+      </c>
+      <c r="D80">
+        <v>228</v>
+      </c>
+      <c r="E80">
+        <v>246</v>
+      </c>
+      <c r="F80" s="6">
+        <v>1.4270833333333333E-2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A81">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+      <c r="B81">
+        <v>9</v>
+      </c>
+      <c r="C81" s="3">
+        <v>46128.798611111109</v>
+      </c>
+      <c r="D81">
+        <v>246</v>
+      </c>
+      <c r="E81">
+        <v>261</v>
+      </c>
+      <c r="F81" s="6">
+        <v>1.3009259259259259E-2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A82">
+        <f t="shared" si="1"/>
+        <v>81</v>
+      </c>
+      <c r="B82">
+        <v>9</v>
+      </c>
+      <c r="C82" s="3">
+        <v>46128.929861111108</v>
+      </c>
+      <c r="D82">
+        <v>261</v>
+      </c>
+      <c r="E82">
+        <v>278</v>
+      </c>
+      <c r="F82" s="6">
+        <v>1.5601851851851851E-2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A83">
+        <f t="shared" si="1"/>
+        <v>82</v>
+      </c>
+      <c r="B83">
+        <v>9</v>
+      </c>
+      <c r="C83" s="3">
+        <v>46129.954861111109</v>
+      </c>
+      <c r="D83">
+        <v>278</v>
+      </c>
+      <c r="E83">
+        <v>287</v>
+      </c>
+      <c r="F83" s="6">
+        <v>8.4837962962962966E-3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A84">
+        <f t="shared" si="1"/>
+        <v>83</v>
+      </c>
+      <c r="B84">
+        <v>9</v>
+      </c>
+      <c r="C84" s="3">
+        <v>46131.652083333334</v>
+      </c>
+      <c r="D84">
+        <v>287</v>
+      </c>
+      <c r="E84">
+        <v>310</v>
+      </c>
+      <c r="F84" s="6">
+        <v>1.7627314814814814E-2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A85">
+        <f t="shared" si="1"/>
+        <v>84</v>
+      </c>
+      <c r="B85">
+        <v>10</v>
+      </c>
+      <c r="C85" s="3">
+        <v>46135.461111111108</v>
+      </c>
+      <c r="D85">
+        <v>7</v>
+      </c>
+      <c r="E85" s="9">
+        <v>25</v>
+      </c>
+      <c r="F85" s="6">
+        <v>1.5775462962962963E-2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A86">
+        <f t="shared" si="1"/>
+        <v>85</v>
+      </c>
+      <c r="B86">
+        <v>10</v>
+      </c>
+      <c r="C86" s="3">
+        <v>46135.809027777781</v>
+      </c>
+      <c r="D86" s="9">
+        <v>25</v>
+      </c>
+      <c r="E86">
+        <v>35</v>
+      </c>
+      <c r="F86" s="6">
+        <v>7.858796296296296E-3</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A87">
+        <f t="shared" si="1"/>
+        <v>86</v>
+      </c>
+      <c r="B87">
+        <v>10</v>
+      </c>
+      <c r="C87" s="3">
+        <v>46136.99722222222</v>
+      </c>
+      <c r="D87">
+        <v>35</v>
+      </c>
+      <c r="E87">
+        <v>52</v>
+      </c>
+      <c r="F87" s="6">
+        <v>1.4490740740740742E-2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A88">
+        <f t="shared" si="1"/>
+        <v>87</v>
+      </c>
+      <c r="B88">
+        <v>10</v>
+      </c>
+      <c r="C88" s="3">
+        <v>46137.879166666666</v>
+      </c>
+      <c r="D88">
+        <v>52</v>
+      </c>
+      <c r="E88">
+        <v>84</v>
+      </c>
+      <c r="F88" s="6">
+        <v>2.5011574074074075E-2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A89">
+        <f t="shared" si="1"/>
+        <v>88</v>
+      </c>
+      <c r="B89">
+        <v>10</v>
+      </c>
+      <c r="C89" s="3">
+        <v>46138.981249999997</v>
+      </c>
+      <c r="D89">
+        <v>84</v>
+      </c>
+      <c r="E89">
+        <v>100</v>
+      </c>
+      <c r="F89" s="6">
+        <v>1.4513888888888889E-2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A90">
+        <f t="shared" si="1"/>
+        <v>89</v>
+      </c>
+      <c r="B90">
+        <v>10</v>
+      </c>
+      <c r="C90" s="3">
+        <v>46139.945833333331</v>
+      </c>
+      <c r="D90">
+        <v>100</v>
+      </c>
+      <c r="E90">
+        <v>110</v>
+      </c>
+      <c r="F90" s="6">
+        <v>7.9398148148148145E-3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A91">
+        <f t="shared" si="1"/>
+        <v>90</v>
+      </c>
+      <c r="B91">
+        <v>10</v>
+      </c>
+      <c r="C91" s="3">
+        <v>46141.45416666667</v>
+      </c>
+      <c r="D91">
+        <v>110</v>
+      </c>
+      <c r="E91">
+        <v>132</v>
+      </c>
+      <c r="F91" s="6">
+        <v>1.9016203703703705E-2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A92">
+        <f t="shared" si="1"/>
+        <v>91</v>
+      </c>
+      <c r="B92">
+        <v>10</v>
+      </c>
+      <c r="C92" s="3">
+        <v>46141.970833333333</v>
+      </c>
+      <c r="D92">
+        <v>132</v>
+      </c>
+      <c r="E92">
+        <v>149</v>
+      </c>
+      <c r="F92" s="6">
+        <v>1.494212962962963E-2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A93">
+        <f t="shared" si="1"/>
+        <v>92</v>
+      </c>
+      <c r="B93">
+        <v>10</v>
+      </c>
+      <c r="C93" s="3">
+        <v>46143.990277777775</v>
+      </c>
+      <c r="D93">
+        <v>149</v>
+      </c>
+      <c r="E93">
+        <v>165</v>
+      </c>
+      <c r="F93" s="6">
+        <v>1.224537037037037E-2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A94">
+        <f t="shared" si="1"/>
+        <v>93</v>
+      </c>
+      <c r="B94">
+        <v>10</v>
+      </c>
+      <c r="C94" s="3">
+        <v>46144.955555555556</v>
+      </c>
+      <c r="D94">
+        <v>165</v>
+      </c>
+      <c r="E94">
+        <v>193</v>
+      </c>
+      <c r="F94" s="6">
+        <v>2.3958333333333335E-2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A95">
+        <f t="shared" si="1"/>
+        <v>94</v>
+      </c>
+      <c r="B95">
+        <v>10</v>
+      </c>
+      <c r="C95" s="3">
+        <v>46145.529861111114</v>
+      </c>
+      <c r="D95">
+        <v>193</v>
+      </c>
+      <c r="E95">
+        <v>204</v>
+      </c>
+      <c r="F95" s="6">
+        <v>8.472222222222223E-3</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A96">
+        <f t="shared" si="1"/>
+        <v>95</v>
+      </c>
+      <c r="B96">
+        <v>10</v>
+      </c>
+      <c r="C96" s="3">
+        <v>46145.815972222219</v>
+      </c>
+      <c r="D96">
+        <v>204</v>
+      </c>
+      <c r="E96">
+        <v>225</v>
+      </c>
+      <c r="F96" s="6">
+        <v>1.5243055555555555E-2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A97">
+        <f t="shared" si="1"/>
+        <v>96</v>
+      </c>
+      <c r="B97">
+        <v>10</v>
+      </c>
+      <c r="C97" s="3">
+        <v>46146.943055555559</v>
+      </c>
+      <c r="D97">
+        <v>225</v>
+      </c>
+      <c r="E97">
+        <v>239</v>
+      </c>
+      <c r="F97" s="6">
+        <v>1.0532407407407407E-2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A98">
+        <f t="shared" si="1"/>
+        <v>97</v>
+      </c>
+      <c r="B98">
+        <v>10</v>
+      </c>
+      <c r="C98" s="3">
+        <v>46147.919444444444</v>
+      </c>
+      <c r="D98">
+        <v>239</v>
+      </c>
+      <c r="E98">
+        <v>251</v>
+      </c>
+      <c r="F98" s="6">
+        <v>9.8958333333333329E-3</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D102" s="10"/>
+      <c r="G102" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2415,12 +3287,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CC89663-E888-2445-AD16-77803353ADBB}">
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E112"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
   </cols>
@@ -3638,7 +4510,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67">
-        <f t="shared" ref="A67:A78" si="2" xml:space="preserve"> ROW() -1</f>
+        <f t="shared" ref="A67:A112" si="2" xml:space="preserve"> ROW() -1</f>
         <v>66</v>
       </c>
       <c r="B67">
@@ -3863,6 +4735,667 @@
         <v>261</v>
       </c>
     </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A79">
+        <f t="shared" si="2"/>
+        <v>78</v>
+      </c>
+      <c r="B79">
+        <v>9</v>
+      </c>
+      <c r="C79">
+        <v>1</v>
+      </c>
+      <c r="D79" t="s">
+        <v>88</v>
+      </c>
+      <c r="E79">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A80">
+        <f t="shared" si="2"/>
+        <v>79</v>
+      </c>
+      <c r="B80">
+        <v>9</v>
+      </c>
+      <c r="C80">
+        <v>2</v>
+      </c>
+      <c r="D80" t="s">
+        <v>89</v>
+      </c>
+      <c r="E80">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A81">
+        <f t="shared" si="2"/>
+        <v>80</v>
+      </c>
+      <c r="B81">
+        <v>9</v>
+      </c>
+      <c r="C81">
+        <f>C80+1</f>
+        <v>3</v>
+      </c>
+      <c r="D81" t="s">
+        <v>90</v>
+      </c>
+      <c r="E81">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A82">
+        <f t="shared" si="2"/>
+        <v>81</v>
+      </c>
+      <c r="B82">
+        <v>9</v>
+      </c>
+      <c r="C82">
+        <f t="shared" ref="C82:C93" si="3">C81+1</f>
+        <v>4</v>
+      </c>
+      <c r="D82" t="s">
+        <v>91</v>
+      </c>
+      <c r="E82">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A83">
+        <f t="shared" si="2"/>
+        <v>82</v>
+      </c>
+      <c r="B83">
+        <v>9</v>
+      </c>
+      <c r="C83">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="D83" t="s">
+        <v>92</v>
+      </c>
+      <c r="E83">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A84">
+        <f t="shared" si="2"/>
+        <v>83</v>
+      </c>
+      <c r="B84">
+        <v>9</v>
+      </c>
+      <c r="C84">
+        <f t="shared" si="3"/>
+        <v>6</v>
+      </c>
+      <c r="D84" t="s">
+        <v>93</v>
+      </c>
+      <c r="E84">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A85">
+        <f t="shared" si="2"/>
+        <v>84</v>
+      </c>
+      <c r="B85">
+        <v>9</v>
+      </c>
+      <c r="C85">
+        <f t="shared" si="3"/>
+        <v>7</v>
+      </c>
+      <c r="D85" t="s">
+        <v>94</v>
+      </c>
+      <c r="E85">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A86">
+        <f t="shared" si="2"/>
+        <v>85</v>
+      </c>
+      <c r="B86">
+        <v>9</v>
+      </c>
+      <c r="C86">
+        <f t="shared" si="3"/>
+        <v>8</v>
+      </c>
+      <c r="D86" t="s">
+        <v>95</v>
+      </c>
+      <c r="E86">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A87">
+        <f t="shared" si="2"/>
+        <v>86</v>
+      </c>
+      <c r="B87">
+        <v>9</v>
+      </c>
+      <c r="C87">
+        <f t="shared" si="3"/>
+        <v>9</v>
+      </c>
+      <c r="D87" t="s">
+        <v>96</v>
+      </c>
+      <c r="E87">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A88">
+        <f t="shared" si="2"/>
+        <v>87</v>
+      </c>
+      <c r="B88">
+        <v>9</v>
+      </c>
+      <c r="C88">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="D88" t="s">
+        <v>97</v>
+      </c>
+      <c r="E88">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A89">
+        <f t="shared" si="2"/>
+        <v>88</v>
+      </c>
+      <c r="B89">
+        <v>9</v>
+      </c>
+      <c r="C89">
+        <f t="shared" si="3"/>
+        <v>11</v>
+      </c>
+      <c r="D89" t="s">
+        <v>98</v>
+      </c>
+      <c r="E89">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A90">
+        <f t="shared" si="2"/>
+        <v>89</v>
+      </c>
+      <c r="B90">
+        <v>9</v>
+      </c>
+      <c r="C90">
+        <f t="shared" si="3"/>
+        <v>12</v>
+      </c>
+      <c r="D90" t="s">
+        <v>99</v>
+      </c>
+      <c r="E90">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A91">
+        <f t="shared" si="2"/>
+        <v>90</v>
+      </c>
+      <c r="B91">
+        <v>9</v>
+      </c>
+      <c r="C91">
+        <f t="shared" si="3"/>
+        <v>13</v>
+      </c>
+      <c r="D91" t="s">
+        <v>100</v>
+      </c>
+      <c r="E91">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A92">
+        <f t="shared" si="2"/>
+        <v>91</v>
+      </c>
+      <c r="B92">
+        <v>9</v>
+      </c>
+      <c r="C92">
+        <f t="shared" si="3"/>
+        <v>14</v>
+      </c>
+      <c r="D92" t="s">
+        <v>101</v>
+      </c>
+      <c r="E92">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A93">
+        <f t="shared" si="2"/>
+        <v>92</v>
+      </c>
+      <c r="B93">
+        <v>9</v>
+      </c>
+      <c r="C93">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+      <c r="D93" t="s">
+        <v>102</v>
+      </c>
+      <c r="E93">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A94">
+        <f t="shared" si="2"/>
+        <v>93</v>
+      </c>
+      <c r="B94">
+        <v>10</v>
+      </c>
+      <c r="C94">
+        <v>1</v>
+      </c>
+      <c r="D94">
+        <f>C94</f>
+        <v>1</v>
+      </c>
+      <c r="E94">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A95">
+        <f t="shared" si="2"/>
+        <v>94</v>
+      </c>
+      <c r="B95">
+        <v>10</v>
+      </c>
+      <c r="C95">
+        <v>2</v>
+      </c>
+      <c r="D95">
+        <f t="shared" ref="D95:D112" si="4">C95</f>
+        <v>2</v>
+      </c>
+      <c r="E95">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A96">
+        <f t="shared" si="2"/>
+        <v>95</v>
+      </c>
+      <c r="B96">
+        <v>10</v>
+      </c>
+      <c r="C96">
+        <f>C95+1</f>
+        <v>3</v>
+      </c>
+      <c r="D96">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="E96">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A97">
+        <f t="shared" si="2"/>
+        <v>96</v>
+      </c>
+      <c r="B97">
+        <v>10</v>
+      </c>
+      <c r="C97">
+        <f t="shared" ref="C97:C112" si="5">C96+1</f>
+        <v>4</v>
+      </c>
+      <c r="D97">
+        <f t="shared" si="4"/>
+        <v>4</v>
+      </c>
+      <c r="E97">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A98">
+        <f t="shared" si="2"/>
+        <v>97</v>
+      </c>
+      <c r="B98">
+        <v>10</v>
+      </c>
+      <c r="C98">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="D98">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="E98">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A99">
+        <f t="shared" si="2"/>
+        <v>98</v>
+      </c>
+      <c r="B99">
+        <v>10</v>
+      </c>
+      <c r="C99">
+        <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
+      <c r="D99">
+        <f t="shared" si="4"/>
+        <v>6</v>
+      </c>
+      <c r="E99">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A100">
+        <f t="shared" si="2"/>
+        <v>99</v>
+      </c>
+      <c r="B100">
+        <v>10</v>
+      </c>
+      <c r="C100">
+        <f t="shared" si="5"/>
+        <v>7</v>
+      </c>
+      <c r="D100">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
+      <c r="E100">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A101">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="B101">
+        <v>10</v>
+      </c>
+      <c r="C101">
+        <f t="shared" si="5"/>
+        <v>8</v>
+      </c>
+      <c r="D101">
+        <f t="shared" si="4"/>
+        <v>8</v>
+      </c>
+      <c r="E101">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A102">
+        <f t="shared" si="2"/>
+        <v>101</v>
+      </c>
+      <c r="B102">
+        <v>10</v>
+      </c>
+      <c r="C102">
+        <f t="shared" si="5"/>
+        <v>9</v>
+      </c>
+      <c r="D102">
+        <f t="shared" si="4"/>
+        <v>9</v>
+      </c>
+      <c r="E102">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A103">
+        <f t="shared" si="2"/>
+        <v>102</v>
+      </c>
+      <c r="B103">
+        <v>10</v>
+      </c>
+      <c r="C103">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="D103">
+        <f t="shared" si="4"/>
+        <v>10</v>
+      </c>
+      <c r="E103">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A104">
+        <f t="shared" si="2"/>
+        <v>103</v>
+      </c>
+      <c r="B104">
+        <v>10</v>
+      </c>
+      <c r="C104">
+        <f>C103+1</f>
+        <v>11</v>
+      </c>
+      <c r="D104">
+        <f t="shared" si="4"/>
+        <v>11</v>
+      </c>
+      <c r="E104">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A105">
+        <f t="shared" si="2"/>
+        <v>104</v>
+      </c>
+      <c r="B105">
+        <v>10</v>
+      </c>
+      <c r="C105">
+        <f t="shared" si="5"/>
+        <v>12</v>
+      </c>
+      <c r="D105">
+        <f t="shared" si="4"/>
+        <v>12</v>
+      </c>
+      <c r="E105">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A106">
+        <f t="shared" si="2"/>
+        <v>105</v>
+      </c>
+      <c r="B106">
+        <v>10</v>
+      </c>
+      <c r="C106">
+        <f t="shared" si="5"/>
+        <v>13</v>
+      </c>
+      <c r="D106">
+        <f t="shared" si="4"/>
+        <v>13</v>
+      </c>
+      <c r="E106">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A107">
+        <f t="shared" si="2"/>
+        <v>106</v>
+      </c>
+      <c r="B107">
+        <v>10</v>
+      </c>
+      <c r="C107">
+        <f t="shared" si="5"/>
+        <v>14</v>
+      </c>
+      <c r="D107">
+        <f t="shared" si="4"/>
+        <v>14</v>
+      </c>
+      <c r="E107">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A108">
+        <f t="shared" si="2"/>
+        <v>107</v>
+      </c>
+      <c r="B108">
+        <v>10</v>
+      </c>
+      <c r="C108">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+      <c r="D108">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="E108">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A109">
+        <f t="shared" si="2"/>
+        <v>108</v>
+      </c>
+      <c r="B109">
+        <v>10</v>
+      </c>
+      <c r="C109">
+        <f t="shared" si="5"/>
+        <v>16</v>
+      </c>
+      <c r="D109">
+        <f t="shared" si="4"/>
+        <v>16</v>
+      </c>
+      <c r="E109">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A110">
+        <f t="shared" si="2"/>
+        <v>109</v>
+      </c>
+      <c r="B110">
+        <v>10</v>
+      </c>
+      <c r="C110">
+        <f>C109+1</f>
+        <v>17</v>
+      </c>
+      <c r="D110">
+        <f t="shared" si="4"/>
+        <v>17</v>
+      </c>
+      <c r="E110">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A111">
+        <f t="shared" si="2"/>
+        <v>110</v>
+      </c>
+      <c r="B111">
+        <v>10</v>
+      </c>
+      <c r="C111">
+        <f t="shared" si="5"/>
+        <v>18</v>
+      </c>
+      <c r="D111">
+        <f t="shared" si="4"/>
+        <v>18</v>
+      </c>
+      <c r="E111">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A112">
+        <f t="shared" si="2"/>
+        <v>111</v>
+      </c>
+      <c r="B112">
+        <v>10</v>
+      </c>
+      <c r="C112">
+        <f t="shared" si="5"/>
+        <v>19</v>
+      </c>
+      <c r="D112">
+        <f t="shared" si="4"/>
+        <v>19</v>
+      </c>
+      <c r="E112">
+        <v>251</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data (prelude to foundation)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/Stuff/reading-analysis/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/stuff/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B986209A-4126-B448-80E0-6553C44A0A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{065AEB2F-1AE7-CE4E-8E7D-AB73C3240F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="680" windowWidth="15040" windowHeight="18980" activeTab="2" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="15040" windowHeight="18980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="128">
   <si>
     <t>book_id</t>
   </si>
@@ -359,6 +359,66 @@
   </si>
   <si>
     <t>Jan Kerouac</t>
+  </si>
+  <si>
+    <t>Prelude to Foundation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mathematician </t>
+  </si>
+  <si>
+    <t>Flight</t>
+  </si>
+  <si>
+    <t>Library</t>
+  </si>
+  <si>
+    <t>Upperside</t>
+  </si>
+  <si>
+    <t>Rescue</t>
+  </si>
+  <si>
+    <t>Mycogen</t>
+  </si>
+  <si>
+    <t>Sunmaster</t>
+  </si>
+  <si>
+    <t>Microfarm</t>
+  </si>
+  <si>
+    <t>Book</t>
+  </si>
+  <si>
+    <t>Sacratorium</t>
+  </si>
+  <si>
+    <t>Aerie</t>
+  </si>
+  <si>
+    <t>Heatsink</t>
+  </si>
+  <si>
+    <t>Billibottom</t>
+  </si>
+  <si>
+    <t>Undercover</t>
+  </si>
+  <si>
+    <t>Officers</t>
+  </si>
+  <si>
+    <t>Wye</t>
+  </si>
+  <si>
+    <t>Overthrow</t>
+  </si>
+  <si>
+    <t>Dors</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -423,9 +483,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -760,7 +820,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -769,7 +829,7 @@
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.6640625" style="7" bestFit="1" customWidth="1"/>
@@ -798,7 +858,7 @@
       <c r="G1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="11" t="s">
         <v>65</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -837,7 +897,7 @@
       <c r="G2">
         <v>136</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="10">
         <v>38544</v>
       </c>
       <c r="I2" t="s">
@@ -876,7 +936,7 @@
       <c r="G3">
         <v>160</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="10">
         <v>36949</v>
       </c>
       <c r="I3" t="s">
@@ -915,7 +975,7 @@
       <c r="G4">
         <v>487</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="10">
         <v>205432</v>
       </c>
       <c r="I4" t="s">
@@ -954,7 +1014,7 @@
       <c r="G5">
         <v>449</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="10">
         <v>136496</v>
       </c>
       <c r="I5" t="s">
@@ -993,7 +1053,7 @@
       <c r="G6">
         <v>499</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="10">
         <v>142714</v>
       </c>
       <c r="I6" t="s">
@@ -1032,7 +1092,7 @@
       <c r="G7">
         <v>210</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="10">
         <v>53760</v>
       </c>
       <c r="I7" t="s">
@@ -1070,7 +1130,7 @@
       <c r="G8">
         <v>266</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="10" t="s">
         <v>63</v>
       </c>
       <c r="I8" t="s">
@@ -1108,7 +1168,7 @@
       <c r="G9">
         <v>261</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="10">
         <v>105626</v>
       </c>
       <c r="I9" t="s">
@@ -1146,7 +1206,7 @@
       <c r="G10">
         <v>310</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="10">
         <v>105413</v>
       </c>
       <c r="I10" t="s">
@@ -1184,7 +1244,7 @@
       <c r="G11">
         <v>244</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="10">
         <v>90974</v>
       </c>
       <c r="I11" t="s">
@@ -1198,6 +1258,49 @@
       </c>
       <c r="L11" s="7">
         <v>46147</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12">
+        <v>1988</v>
+      </c>
+      <c r="F12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12">
+        <v>490</v>
+      </c>
+      <c r="H12" s="10">
+        <v>130823</v>
+      </c>
+      <c r="I12" t="s">
+        <v>104</v>
+      </c>
+      <c r="J12" t="s">
+        <v>67</v>
+      </c>
+      <c r="K12" s="7">
+        <v>46151</v>
+      </c>
+      <c r="L12" s="7">
+        <v>46155</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K13" s="7" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -1207,7 +1310,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I102"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -2606,7 +2709,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67">
-        <f t="shared" ref="A67:A98" si="1">ROW() - 1</f>
+        <f t="shared" ref="A67:A109" si="1">ROW() - 1</f>
         <v>66</v>
       </c>
       <c r="B67">
@@ -2996,7 +3099,7 @@
       <c r="D85">
         <v>7</v>
       </c>
-      <c r="E85" s="9">
+      <c r="E85">
         <v>25</v>
       </c>
       <c r="F85" s="6">
@@ -3014,7 +3117,7 @@
       <c r="C86" s="3">
         <v>46135.809027777781</v>
       </c>
-      <c r="D86" s="9">
+      <c r="D86">
         <v>25</v>
       </c>
       <c r="E86">
@@ -3276,9 +3379,237 @@
         <v>9.8958333333333329E-3</v>
       </c>
     </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A99">
+        <f t="shared" si="1"/>
+        <v>98</v>
+      </c>
+      <c r="B99">
+        <v>11</v>
+      </c>
+      <c r="C99" s="3">
+        <v>46151.415972222225</v>
+      </c>
+      <c r="D99">
+        <v>3</v>
+      </c>
+      <c r="E99">
+        <v>31</v>
+      </c>
+      <c r="F99" s="6">
+        <v>1.7060185185185185E-2</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A100">
+        <f t="shared" si="1"/>
+        <v>99</v>
+      </c>
+      <c r="B100">
+        <v>11</v>
+      </c>
+      <c r="C100" s="3">
+        <v>46151.720833333333</v>
+      </c>
+      <c r="D100">
+        <v>31</v>
+      </c>
+      <c r="E100">
+        <v>77</v>
+      </c>
+      <c r="F100" s="6">
+        <v>2.2766203703703705E-2</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A101">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="B101">
+        <v>11</v>
+      </c>
+      <c r="C101" s="3">
+        <v>46152.706944444442</v>
+      </c>
+      <c r="D101">
+        <v>77</v>
+      </c>
+      <c r="E101">
+        <v>105</v>
+      </c>
+      <c r="F101" s="6">
+        <v>1.5057870370370371E-2</v>
+      </c>
+    </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="D102" s="10"/>
-      <c r="G102" s="11"/>
+      <c r="A102">
+        <f t="shared" si="1"/>
+        <v>101</v>
+      </c>
+      <c r="B102">
+        <v>11</v>
+      </c>
+      <c r="C102" s="3">
+        <v>46152.932638888888</v>
+      </c>
+      <c r="D102" s="10">
+        <v>105</v>
+      </c>
+      <c r="E102">
+        <v>157</v>
+      </c>
+      <c r="F102" s="6">
+        <v>2.6215277777777778E-2</v>
+      </c>
+      <c r="G102" s="9"/>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A103">
+        <f t="shared" si="1"/>
+        <v>102</v>
+      </c>
+      <c r="B103">
+        <v>11</v>
+      </c>
+      <c r="C103" s="3">
+        <v>46153.714583333334</v>
+      </c>
+      <c r="D103">
+        <v>157</v>
+      </c>
+      <c r="E103">
+        <v>209</v>
+      </c>
+      <c r="F103" s="6">
+        <v>2.5358796296296296E-2</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A104">
+        <f t="shared" si="1"/>
+        <v>103</v>
+      </c>
+      <c r="B104">
+        <v>11</v>
+      </c>
+      <c r="C104" s="3">
+        <v>46153.786805555559</v>
+      </c>
+      <c r="D104">
+        <v>209</v>
+      </c>
+      <c r="E104">
+        <v>235</v>
+      </c>
+      <c r="F104" s="6">
+        <v>1.2951388888888889E-2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A105">
+        <f t="shared" si="1"/>
+        <v>104</v>
+      </c>
+      <c r="B105">
+        <v>11</v>
+      </c>
+      <c r="C105" s="3">
+        <v>46153.900694444441</v>
+      </c>
+      <c r="D105">
+        <v>235</v>
+      </c>
+      <c r="E105">
+        <v>289</v>
+      </c>
+      <c r="F105" s="6">
+        <v>2.7407407407407408E-2</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A106">
+        <f t="shared" si="1"/>
+        <v>105</v>
+      </c>
+      <c r="B106">
+        <v>11</v>
+      </c>
+      <c r="C106" s="3">
+        <v>46154.393750000003</v>
+      </c>
+      <c r="D106">
+        <v>289</v>
+      </c>
+      <c r="E106">
+        <v>317</v>
+      </c>
+      <c r="F106" s="6">
+        <v>1.4166666666666666E-2</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A107">
+        <f t="shared" si="1"/>
+        <v>106</v>
+      </c>
+      <c r="B107">
+        <v>11</v>
+      </c>
+      <c r="C107" s="3">
+        <v>46154.787499999999</v>
+      </c>
+      <c r="D107">
+        <v>317</v>
+      </c>
+      <c r="E107">
+        <v>349</v>
+      </c>
+      <c r="F107" s="6">
+        <v>1.6643518518518519E-2</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A108">
+        <f t="shared" si="1"/>
+        <v>107</v>
+      </c>
+      <c r="B108">
+        <v>11</v>
+      </c>
+      <c r="C108" s="3">
+        <v>46154.845138888886</v>
+      </c>
+      <c r="D108">
+        <v>349</v>
+      </c>
+      <c r="E108">
+        <v>451</v>
+      </c>
+      <c r="F108" s="6">
+        <v>4.5613425925925925E-2</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A109">
+        <f t="shared" si="1"/>
+        <v>108</v>
+      </c>
+      <c r="B109">
+        <v>11</v>
+      </c>
+      <c r="C109" s="3">
+        <v>46155.425000000003</v>
+      </c>
+      <c r="D109">
+        <v>451</v>
+      </c>
+      <c r="E109">
+        <v>493</v>
+      </c>
+      <c r="F109" s="6">
+        <v>2.1099537037037038E-2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3287,7 +3618,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CC89663-E888-2445-AD16-77803353ADBB}">
-  <dimension ref="A1:E112"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -4510,7 +4841,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67">
-        <f t="shared" ref="A67:A112" si="2" xml:space="preserve"> ROW() -1</f>
+        <f t="shared" ref="A67:A130" si="2" xml:space="preserve"> ROW() -1</f>
         <v>66</v>
       </c>
       <c r="B67">
@@ -5049,7 +5380,7 @@
         <v>2</v>
       </c>
       <c r="D95">
-        <f t="shared" ref="D95:D112" si="4">C95</f>
+        <f t="shared" ref="D95:D114" si="4">C95</f>
         <v>2</v>
       </c>
       <c r="E95">
@@ -5394,6 +5725,366 @@
       </c>
       <c r="E112">
         <v>251</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A113">
+        <f t="shared" si="2"/>
+        <v>112</v>
+      </c>
+      <c r="B113">
+        <v>11</v>
+      </c>
+      <c r="C113">
+        <v>1</v>
+      </c>
+      <c r="D113" t="s">
+        <v>109</v>
+      </c>
+      <c r="E113">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A114">
+        <f t="shared" si="2"/>
+        <v>113</v>
+      </c>
+      <c r="B114">
+        <v>11</v>
+      </c>
+      <c r="C114">
+        <f>C113+1</f>
+        <v>2</v>
+      </c>
+      <c r="D114" t="s">
+        <v>110</v>
+      </c>
+      <c r="E114">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A115">
+        <f t="shared" si="2"/>
+        <v>114</v>
+      </c>
+      <c r="B115">
+        <v>11</v>
+      </c>
+      <c r="C115">
+        <f t="shared" ref="C115:C131" si="6">C114+1</f>
+        <v>3</v>
+      </c>
+      <c r="D115" t="s">
+        <v>29</v>
+      </c>
+      <c r="E115">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A116">
+        <f t="shared" si="2"/>
+        <v>115</v>
+      </c>
+      <c r="B116">
+        <v>11</v>
+      </c>
+      <c r="C116">
+        <f t="shared" si="6"/>
+        <v>4</v>
+      </c>
+      <c r="D116" t="s">
+        <v>111</v>
+      </c>
+      <c r="E116">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A117">
+        <f t="shared" si="2"/>
+        <v>116</v>
+      </c>
+      <c r="B117">
+        <v>11</v>
+      </c>
+      <c r="C117">
+        <f t="shared" si="6"/>
+        <v>5</v>
+      </c>
+      <c r="D117" t="s">
+        <v>112</v>
+      </c>
+      <c r="E117">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A118">
+        <f t="shared" si="2"/>
+        <v>117</v>
+      </c>
+      <c r="B118">
+        <v>11</v>
+      </c>
+      <c r="C118">
+        <f t="shared" si="6"/>
+        <v>6</v>
+      </c>
+      <c r="D118" t="s">
+        <v>113</v>
+      </c>
+      <c r="E118">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A119">
+        <f t="shared" si="2"/>
+        <v>118</v>
+      </c>
+      <c r="B119">
+        <v>11</v>
+      </c>
+      <c r="C119">
+        <f t="shared" si="6"/>
+        <v>7</v>
+      </c>
+      <c r="D119" t="s">
+        <v>114</v>
+      </c>
+      <c r="E119">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A120">
+        <f t="shared" si="2"/>
+        <v>119</v>
+      </c>
+      <c r="B120">
+        <v>11</v>
+      </c>
+      <c r="C120">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="D120" t="s">
+        <v>115</v>
+      </c>
+      <c r="E120">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A121">
+        <f t="shared" si="2"/>
+        <v>120</v>
+      </c>
+      <c r="B121">
+        <v>11</v>
+      </c>
+      <c r="C121">
+        <f t="shared" si="6"/>
+        <v>9</v>
+      </c>
+      <c r="D121" t="s">
+        <v>116</v>
+      </c>
+      <c r="E121">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A122">
+        <f t="shared" si="2"/>
+        <v>121</v>
+      </c>
+      <c r="B122">
+        <v>11</v>
+      </c>
+      <c r="C122">
+        <f t="shared" si="6"/>
+        <v>10</v>
+      </c>
+      <c r="D122" t="s">
+        <v>117</v>
+      </c>
+      <c r="E122">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A123">
+        <f t="shared" si="2"/>
+        <v>122</v>
+      </c>
+      <c r="B123">
+        <v>11</v>
+      </c>
+      <c r="C123">
+        <f t="shared" si="6"/>
+        <v>11</v>
+      </c>
+      <c r="D123" t="s">
+        <v>118</v>
+      </c>
+      <c r="E123">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A124">
+        <f t="shared" si="2"/>
+        <v>123</v>
+      </c>
+      <c r="B124">
+        <v>11</v>
+      </c>
+      <c r="C124">
+        <f t="shared" si="6"/>
+        <v>12</v>
+      </c>
+      <c r="D124" t="s">
+        <v>119</v>
+      </c>
+      <c r="E124">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A125">
+        <f t="shared" si="2"/>
+        <v>124</v>
+      </c>
+      <c r="B125">
+        <v>11</v>
+      </c>
+      <c r="C125">
+        <f t="shared" si="6"/>
+        <v>13</v>
+      </c>
+      <c r="D125" t="s">
+        <v>120</v>
+      </c>
+      <c r="E125">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A126">
+        <f t="shared" si="2"/>
+        <v>125</v>
+      </c>
+      <c r="B126">
+        <v>11</v>
+      </c>
+      <c r="C126">
+        <f t="shared" si="6"/>
+        <v>14</v>
+      </c>
+      <c r="D126" t="s">
+        <v>121</v>
+      </c>
+      <c r="E126">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A127">
+        <f t="shared" si="2"/>
+        <v>126</v>
+      </c>
+      <c r="B127">
+        <v>11</v>
+      </c>
+      <c r="C127">
+        <f t="shared" si="6"/>
+        <v>15</v>
+      </c>
+      <c r="D127" t="s">
+        <v>122</v>
+      </c>
+      <c r="E127">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A128">
+        <f t="shared" si="2"/>
+        <v>127</v>
+      </c>
+      <c r="B128">
+        <v>11</v>
+      </c>
+      <c r="C128">
+        <f t="shared" si="6"/>
+        <v>16</v>
+      </c>
+      <c r="D128" t="s">
+        <v>123</v>
+      </c>
+      <c r="E128">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A129">
+        <f t="shared" si="2"/>
+        <v>128</v>
+      </c>
+      <c r="B129">
+        <v>11</v>
+      </c>
+      <c r="C129">
+        <f t="shared" si="6"/>
+        <v>17</v>
+      </c>
+      <c r="D129" t="s">
+        <v>124</v>
+      </c>
+      <c r="E129">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A130">
+        <f t="shared" si="2"/>
+        <v>129</v>
+      </c>
+      <c r="B130">
+        <v>11</v>
+      </c>
+      <c r="C130">
+        <f t="shared" si="6"/>
+        <v>18</v>
+      </c>
+      <c r="D130" t="s">
+        <v>125</v>
+      </c>
+      <c r="E130">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A131">
+        <f t="shared" ref="A131" si="7" xml:space="preserve"> ROW() -1</f>
+        <v>130</v>
+      </c>
+      <c r="B131">
+        <v>11</v>
+      </c>
+      <c r="C131">
+        <f t="shared" si="6"/>
+        <v>19</v>
+      </c>
+      <c r="D131" t="s">
+        <v>126</v>
+      </c>
+      <c r="E131">
+        <v>493</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add README.md with notes, fix spelling of billibotton chapter
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/stuff/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{065AEB2F-1AE7-CE4E-8E7D-AB73C3240F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D138C95-8D94-FC4E-9230-EDF31CF3CE3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="15040" windowHeight="18980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="128">
   <si>
     <t>book_id</t>
   </si>
@@ -400,9 +400,6 @@
     <t>Heatsink</t>
   </si>
   <si>
-    <t>Billibottom</t>
-  </si>
-  <si>
     <t>Undercover</t>
   </si>
   <si>
@@ -418,7 +415,10 @@
     <t>Dors</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t>Billibotton</t>
+  </si>
+  <si>
+    <t>Forward the Foundation</t>
   </si>
 </sst>
 </file>
@@ -473,7 +473,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -484,8 +484,6 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -829,7 +827,7 @@
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.6640625" style="7" bestFit="1" customWidth="1"/>
@@ -858,7 +856,7 @@
       <c r="G1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -897,7 +895,7 @@
       <c r="G2">
         <v>136</v>
       </c>
-      <c r="H2" s="10">
+      <c r="H2">
         <v>38544</v>
       </c>
       <c r="I2" t="s">
@@ -936,7 +934,7 @@
       <c r="G3">
         <v>160</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3">
         <v>36949</v>
       </c>
       <c r="I3" t="s">
@@ -975,7 +973,7 @@
       <c r="G4">
         <v>487</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4">
         <v>205432</v>
       </c>
       <c r="I4" t="s">
@@ -1014,7 +1012,7 @@
       <c r="G5">
         <v>449</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5">
         <v>136496</v>
       </c>
       <c r="I5" t="s">
@@ -1053,7 +1051,7 @@
       <c r="G6">
         <v>499</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6">
         <v>142714</v>
       </c>
       <c r="I6" t="s">
@@ -1092,7 +1090,7 @@
       <c r="G7">
         <v>210</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7">
         <v>53760</v>
       </c>
       <c r="I7" t="s">
@@ -1130,7 +1128,7 @@
       <c r="G8">
         <v>266</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" t="s">
         <v>63</v>
       </c>
       <c r="I8" t="s">
@@ -1168,7 +1166,7 @@
       <c r="G9">
         <v>261</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H9">
         <v>105626</v>
       </c>
       <c r="I9" t="s">
@@ -1206,7 +1204,7 @@
       <c r="G10">
         <v>310</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10">
         <v>105413</v>
       </c>
       <c r="I10" t="s">
@@ -1244,7 +1242,7 @@
       <c r="G11">
         <v>244</v>
       </c>
-      <c r="H11" s="10">
+      <c r="H11">
         <v>90974</v>
       </c>
       <c r="I11" t="s">
@@ -1282,7 +1280,7 @@
       <c r="G12">
         <v>490</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H12">
         <v>130823</v>
       </c>
       <c r="I12" t="s">
@@ -1299,8 +1297,29 @@
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="K13" s="7" t="s">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
         <v>127</v>
+      </c>
+      <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13">
+        <v>1993</v>
+      </c>
+      <c r="F13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J13" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" s="7">
+        <v>46155</v>
       </c>
     </row>
   </sheetData>
@@ -3453,7 +3472,7 @@
       <c r="C102" s="3">
         <v>46152.932638888888</v>
       </c>
-      <c r="D102" s="10">
+      <c r="D102">
         <v>105</v>
       </c>
       <c r="E102">
@@ -5380,7 +5399,7 @@
         <v>2</v>
       </c>
       <c r="D95">
-        <f t="shared" ref="D95:D114" si="4">C95</f>
+        <f t="shared" ref="D95:D112" si="4">C95</f>
         <v>2</v>
       </c>
       <c r="E95">
@@ -5986,7 +6005,7 @@
         <v>14</v>
       </c>
       <c r="D126" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="E126">
         <v>375</v>
@@ -6005,7 +6024,7 @@
         <v>15</v>
       </c>
       <c r="D127" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E127">
         <v>399</v>
@@ -6024,7 +6043,7 @@
         <v>16</v>
       </c>
       <c r="D128" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E128">
         <v>423</v>
@@ -6043,7 +6062,7 @@
         <v>17</v>
       </c>
       <c r="D129" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E129">
         <v>449</v>
@@ -6062,7 +6081,7 @@
         <v>18</v>
       </c>
       <c r="D130" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E130">
         <v>473</v>
@@ -6081,7 +6100,7 @@
         <v>19</v>
       </c>
       <c r="D131" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E131">
         <v>493</v>

</xml_diff>

<commit_message>
data (forward the foundation) and update README.md
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/stuff/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D138C95-8D94-FC4E-9230-EDF31CF3CE3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D7D333-F84F-7E41-AF19-26336BAB8711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="15040" windowHeight="18980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="-20" yWindow="680" windowWidth="15040" windowHeight="18980" activeTab="2" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="136">
   <si>
     <t>book_id</t>
   </si>
@@ -419,6 +419,30 @@
   </si>
   <si>
     <t>Forward the Foundation</t>
+  </si>
+  <si>
+    <t>Keats: A Brief Life in Nine Poems and One Epitaph</t>
+  </si>
+  <si>
+    <t>Lucasta Miller</t>
+  </si>
+  <si>
+    <t>ebook</t>
+  </si>
+  <si>
+    <t>Eto Demerzel</t>
+  </si>
+  <si>
+    <t>Cleon I</t>
+  </si>
+  <si>
+    <t>Dors Venabili</t>
+  </si>
+  <si>
+    <t>Wanda Seldon</t>
+  </si>
+  <si>
+    <t>Epilogue</t>
   </si>
 </sst>
 </file>
@@ -473,7 +497,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -484,6 +508,8 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -818,16 +844,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" customWidth="1"/>
     <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.6640625" style="7" bestFit="1" customWidth="1"/>
@@ -856,7 +882,7 @@
       <c r="G1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="10" t="s">
         <v>65</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -895,7 +921,7 @@
       <c r="G2">
         <v>136</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="11">
         <v>38544</v>
       </c>
       <c r="I2" t="s">
@@ -934,7 +960,7 @@
       <c r="G3">
         <v>160</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="11">
         <v>36949</v>
       </c>
       <c r="I3" t="s">
@@ -973,7 +999,7 @@
       <c r="G4">
         <v>487</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="11">
         <v>205432</v>
       </c>
       <c r="I4" t="s">
@@ -1012,7 +1038,7 @@
       <c r="G5">
         <v>449</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="11">
         <v>136496</v>
       </c>
       <c r="I5" t="s">
@@ -1051,7 +1077,7 @@
       <c r="G6">
         <v>499</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="11">
         <v>142714</v>
       </c>
       <c r="I6" t="s">
@@ -1090,7 +1116,7 @@
       <c r="G7">
         <v>210</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="11">
         <v>53760</v>
       </c>
       <c r="I7" t="s">
@@ -1128,7 +1154,7 @@
       <c r="G8">
         <v>266</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="11" t="s">
         <v>63</v>
       </c>
       <c r="I8" t="s">
@@ -1166,7 +1192,7 @@
       <c r="G9">
         <v>261</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="11">
         <v>105626</v>
       </c>
       <c r="I9" t="s">
@@ -1204,7 +1230,7 @@
       <c r="G10">
         <v>310</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="11">
         <v>105413</v>
       </c>
       <c r="I10" t="s">
@@ -1242,7 +1268,7 @@
       <c r="G11">
         <v>244</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="11">
         <v>90974</v>
       </c>
       <c r="I11" t="s">
@@ -1280,7 +1306,7 @@
       <c r="G12">
         <v>490</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="11">
         <v>130823</v>
       </c>
       <c r="I12" t="s">
@@ -1315,11 +1341,52 @@
       <c r="F13" t="s">
         <v>16</v>
       </c>
+      <c r="G13">
+        <v>432</v>
+      </c>
+      <c r="H13" s="11">
+        <v>121312</v>
+      </c>
+      <c r="I13" t="s">
+        <v>104</v>
+      </c>
       <c r="J13" t="s">
         <v>67</v>
       </c>
       <c r="K13" s="7">
         <v>46155</v>
+      </c>
+      <c r="L13" s="7">
+        <v>46158</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>128</v>
+      </c>
+      <c r="C14" t="s">
+        <v>129</v>
+      </c>
+      <c r="D14" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14">
+        <v>2021</v>
+      </c>
+      <c r="F14" t="s">
+        <v>130</v>
+      </c>
+      <c r="G14" t="s">
+        <v>63</v>
+      </c>
+      <c r="J14" t="s">
+        <v>76</v>
+      </c>
+      <c r="K14" s="7">
+        <v>45792</v>
       </c>
     </row>
   </sheetData>
@@ -1329,7 +1396,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:I119"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -2728,7 +2795,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67">
-        <f t="shared" ref="A67:A109" si="1">ROW() - 1</f>
+        <f t="shared" ref="A67:A119" si="1">ROW() - 1</f>
         <v>66</v>
       </c>
       <c r="B67">
@@ -3628,6 +3695,216 @@
       </c>
       <c r="F109" s="6">
         <v>2.1099537037037038E-2</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A110">
+        <f t="shared" si="1"/>
+        <v>109</v>
+      </c>
+      <c r="B110">
+        <v>12</v>
+      </c>
+      <c r="C110" s="3">
+        <v>46155.876388888886</v>
+      </c>
+      <c r="D110">
+        <v>3</v>
+      </c>
+      <c r="E110">
+        <v>39</v>
+      </c>
+      <c r="F110" s="6">
+        <v>2.0844907407407406E-2</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A111">
+        <f t="shared" si="1"/>
+        <v>110</v>
+      </c>
+      <c r="B111">
+        <v>12</v>
+      </c>
+      <c r="C111" s="3">
+        <v>46156.767361111109</v>
+      </c>
+      <c r="D111">
+        <v>39</v>
+      </c>
+      <c r="E111">
+        <v>88</v>
+      </c>
+      <c r="F111" s="6">
+        <v>2.5138888888888888E-2</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A112">
+        <f t="shared" si="1"/>
+        <v>111</v>
+      </c>
+      <c r="B112">
+        <v>12</v>
+      </c>
+      <c r="C112" s="3">
+        <v>46157.352083333331</v>
+      </c>
+      <c r="D112">
+        <v>88</v>
+      </c>
+      <c r="E112">
+        <v>107</v>
+      </c>
+      <c r="F112" s="6">
+        <v>7.2800925925925923E-3</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A113">
+        <f t="shared" si="1"/>
+        <v>112</v>
+      </c>
+      <c r="B113">
+        <v>12</v>
+      </c>
+      <c r="C113" s="3">
+        <v>46157.385416666664</v>
+      </c>
+      <c r="D113">
+        <v>107</v>
+      </c>
+      <c r="E113">
+        <v>133</v>
+      </c>
+      <c r="F113" s="6">
+        <v>1.3344907407407408E-2</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A114">
+        <f t="shared" si="1"/>
+        <v>113</v>
+      </c>
+      <c r="B114">
+        <v>12</v>
+      </c>
+      <c r="C114" s="3">
+        <v>46157.62777777778</v>
+      </c>
+      <c r="D114">
+        <v>133</v>
+      </c>
+      <c r="E114">
+        <v>205</v>
+      </c>
+      <c r="F114" s="6">
+        <v>3.471064814814815E-2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A115">
+        <f t="shared" si="1"/>
+        <v>114</v>
+      </c>
+      <c r="B115">
+        <v>12</v>
+      </c>
+      <c r="C115" s="3">
+        <v>46157.85</v>
+      </c>
+      <c r="D115">
+        <v>205</v>
+      </c>
+      <c r="E115">
+        <v>258</v>
+      </c>
+      <c r="F115" s="6">
+        <v>2.6145833333333333E-2</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A116">
+        <f t="shared" si="1"/>
+        <v>115</v>
+      </c>
+      <c r="B116">
+        <v>12</v>
+      </c>
+      <c r="C116" s="3">
+        <v>46158.631249999999</v>
+      </c>
+      <c r="D116">
+        <v>258</v>
+      </c>
+      <c r="E116">
+        <v>307</v>
+      </c>
+      <c r="F116" s="6">
+        <v>2.0902777777777777E-2</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A117">
+        <f t="shared" si="1"/>
+        <v>116</v>
+      </c>
+      <c r="B117">
+        <v>12</v>
+      </c>
+      <c r="C117" s="3">
+        <v>46158.688888888886</v>
+      </c>
+      <c r="D117">
+        <v>307</v>
+      </c>
+      <c r="E117">
+        <v>412</v>
+      </c>
+      <c r="F117" s="6">
+        <v>4.8240740740740744E-2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A118">
+        <f t="shared" si="1"/>
+        <v>117</v>
+      </c>
+      <c r="B118">
+        <v>12</v>
+      </c>
+      <c r="C118" s="3">
+        <v>46158.809027777781</v>
+      </c>
+      <c r="D118">
+        <v>412</v>
+      </c>
+      <c r="E118">
+        <v>431</v>
+      </c>
+      <c r="F118" s="6">
+        <v>6.9444444444444441E-3</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A119">
+        <f t="shared" si="1"/>
+        <v>118</v>
+      </c>
+      <c r="B119">
+        <v>12</v>
+      </c>
+      <c r="C119" s="3">
+        <v>46158.831944444442</v>
+      </c>
+      <c r="D119">
+        <v>431</v>
+      </c>
+      <c r="E119">
+        <v>435</v>
+      </c>
+      <c r="F119" s="6">
+        <v>2.2222222222222222E-3</v>
       </c>
     </row>
   </sheetData>
@@ -3637,7 +3914,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CC89663-E888-2445-AD16-77803353ADBB}">
-  <dimension ref="A1:E131"/>
+  <dimension ref="A1:E136"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -6089,7 +6366,7 @@
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131">
-        <f t="shared" ref="A131" si="7" xml:space="preserve"> ROW() -1</f>
+        <f t="shared" ref="A131:A136" si="7" xml:space="preserve"> ROW() -1</f>
         <v>130</v>
       </c>
       <c r="B131">
@@ -6104,6 +6381,96 @@
       </c>
       <c r="E131">
         <v>493</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A132">
+        <f t="shared" si="7"/>
+        <v>131</v>
+      </c>
+      <c r="B132">
+        <v>12</v>
+      </c>
+      <c r="C132">
+        <v>1</v>
+      </c>
+      <c r="D132" t="s">
+        <v>131</v>
+      </c>
+      <c r="E132">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A133">
+        <f t="shared" si="7"/>
+        <v>132</v>
+      </c>
+      <c r="B133">
+        <v>12</v>
+      </c>
+      <c r="C133">
+        <v>2</v>
+      </c>
+      <c r="D133" t="s">
+        <v>132</v>
+      </c>
+      <c r="E133">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A134">
+        <f t="shared" si="7"/>
+        <v>133</v>
+      </c>
+      <c r="B134">
+        <v>12</v>
+      </c>
+      <c r="C134">
+        <v>3</v>
+      </c>
+      <c r="D134" t="s">
+        <v>133</v>
+      </c>
+      <c r="E134">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A135">
+        <f t="shared" si="7"/>
+        <v>134</v>
+      </c>
+      <c r="B135">
+        <v>12</v>
+      </c>
+      <c r="C135">
+        <v>4</v>
+      </c>
+      <c r="D135" t="s">
+        <v>134</v>
+      </c>
+      <c r="E135">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A136">
+        <f t="shared" si="7"/>
+        <v>135</v>
+      </c>
+      <c r="B136">
+        <v>12</v>
+      </c>
+      <c r="C136">
+        <v>5</v>
+      </c>
+      <c r="D136" t="s">
+        <v>135</v>
+      </c>
+      <c r="E136">
+        <v>435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data (keats: a brief life...)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/stuff/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D7D333-F84F-7E41-AF19-26336BAB8711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FDC7439-45B8-CD4F-824C-61CEBA9BA773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="680" windowWidth="15040" windowHeight="18980" activeTab="2" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="15420" windowHeight="18980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -497,7 +497,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -508,7 +508,6 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -853,7 +852,7 @@
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" style="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.6640625" style="7" bestFit="1" customWidth="1"/>
@@ -882,7 +881,7 @@
       <c r="G1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -921,7 +920,7 @@
       <c r="G2">
         <v>136</v>
       </c>
-      <c r="H2" s="11">
+      <c r="H2">
         <v>38544</v>
       </c>
       <c r="I2" t="s">
@@ -960,7 +959,7 @@
       <c r="G3">
         <v>160</v>
       </c>
-      <c r="H3" s="11">
+      <c r="H3">
         <v>36949</v>
       </c>
       <c r="I3" t="s">
@@ -999,7 +998,7 @@
       <c r="G4">
         <v>487</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4">
         <v>205432</v>
       </c>
       <c r="I4" t="s">
@@ -1038,7 +1037,7 @@
       <c r="G5">
         <v>449</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5">
         <v>136496</v>
       </c>
       <c r="I5" t="s">
@@ -1077,7 +1076,7 @@
       <c r="G6">
         <v>499</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6">
         <v>142714</v>
       </c>
       <c r="I6" t="s">
@@ -1116,7 +1115,7 @@
       <c r="G7">
         <v>210</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7">
         <v>53760</v>
       </c>
       <c r="I7" t="s">
@@ -1154,7 +1153,7 @@
       <c r="G8">
         <v>266</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" t="s">
         <v>63</v>
       </c>
       <c r="I8" t="s">
@@ -1192,7 +1191,7 @@
       <c r="G9">
         <v>261</v>
       </c>
-      <c r="H9" s="11">
+      <c r="H9">
         <v>105626</v>
       </c>
       <c r="I9" t="s">
@@ -1230,7 +1229,7 @@
       <c r="G10">
         <v>310</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10">
         <v>105413</v>
       </c>
       <c r="I10" t="s">
@@ -1268,7 +1267,7 @@
       <c r="G11">
         <v>244</v>
       </c>
-      <c r="H11" s="11">
+      <c r="H11">
         <v>90974</v>
       </c>
       <c r="I11" t="s">
@@ -1306,7 +1305,7 @@
       <c r="G12">
         <v>490</v>
       </c>
-      <c r="H12" s="11">
+      <c r="H12">
         <v>130823</v>
       </c>
       <c r="I12" t="s">
@@ -1344,7 +1343,7 @@
       <c r="G13">
         <v>432</v>
       </c>
-      <c r="H13" s="11">
+      <c r="H13">
         <v>121312</v>
       </c>
       <c r="I13" t="s">
@@ -1379,14 +1378,23 @@
       <c r="F14" t="s">
         <v>130</v>
       </c>
-      <c r="G14" t="s">
-        <v>63</v>
+      <c r="G14">
+        <v>309</v>
+      </c>
+      <c r="H14" s="10">
+        <v>85019</v>
+      </c>
+      <c r="I14" t="s">
+        <v>104</v>
       </c>
       <c r="J14" t="s">
         <v>76</v>
       </c>
       <c r="K14" s="7">
-        <v>45792</v>
+        <v>46157</v>
+      </c>
+      <c r="L14" s="7">
+        <v>46163</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data (The Death of Ivan Ilyich)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/dev/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8219024-5450-FB49-A4E3-00F5CEFAE8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E27D1597-3B0C-8244-B788-624F757C5E9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="15080" windowHeight="18980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="-20" yWindow="640" windowWidth="19140" windowHeight="20980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="155">
   <si>
     <t>book_id</t>
   </si>
@@ -473,6 +473,33 @@
   </si>
   <si>
     <t>Seamus Heaney</t>
+  </si>
+  <si>
+    <t>The Death of Ivan Ilyich and Other Stories</t>
+  </si>
+  <si>
+    <t>Leo Tolstoy</t>
+  </si>
+  <si>
+    <t>The Raid</t>
+  </si>
+  <si>
+    <t>The Woodfelling</t>
+  </si>
+  <si>
+    <t>Three Deaths</t>
+  </si>
+  <si>
+    <t>Polikushka</t>
+  </si>
+  <si>
+    <t>The Death of Ivan Ilyich</t>
+  </si>
+  <si>
+    <t>After the Ball</t>
+  </si>
+  <si>
+    <t>The Forged Coupon</t>
   </si>
 </sst>
 </file>
@@ -873,7 +900,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -1525,7 +1552,7 @@
       <c r="G17">
         <v>106</v>
       </c>
-      <c r="H17" s="10">
+      <c r="H17">
         <v>25711</v>
       </c>
       <c r="I17" t="s">
@@ -1539,6 +1566,44 @@
       </c>
       <c r="L17" s="7">
         <v>46180</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>146</v>
+      </c>
+      <c r="C18" t="s">
+        <v>147</v>
+      </c>
+      <c r="D18" t="s">
+        <v>62</v>
+      </c>
+      <c r="E18">
+        <v>1886</v>
+      </c>
+      <c r="F18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18">
+        <v>309</v>
+      </c>
+      <c r="H18" s="10">
+        <v>108141</v>
+      </c>
+      <c r="I18" t="s">
+        <v>104</v>
+      </c>
+      <c r="J18" t="s">
+        <v>67</v>
+      </c>
+      <c r="K18" s="7">
+        <v>46181</v>
+      </c>
+      <c r="L18" s="7">
+        <v>46186</v>
       </c>
     </row>
   </sheetData>
@@ -1548,7 +1613,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I161"/>
+  <dimension ref="A1:I176"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -4292,7 +4357,7 @@
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131">
-        <f t="shared" ref="A131:A161" si="2">ROW() - 1</f>
+        <f t="shared" ref="A131:A176" si="2">ROW() - 1</f>
         <v>130</v>
       </c>
       <c r="B131">
@@ -4939,6 +5004,321 @@
       </c>
       <c r="F161" s="6">
         <v>7.4305555555555557E-3</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A162">
+        <f t="shared" si="2"/>
+        <v>161</v>
+      </c>
+      <c r="B162">
+        <v>17</v>
+      </c>
+      <c r="C162" s="3">
+        <v>46181.560416666667</v>
+      </c>
+      <c r="D162">
+        <v>3</v>
+      </c>
+      <c r="E162">
+        <v>17</v>
+      </c>
+      <c r="F162" s="6">
+        <v>1.119212962962963E-2</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A163">
+        <f t="shared" si="2"/>
+        <v>162</v>
+      </c>
+      <c r="B163">
+        <v>17</v>
+      </c>
+      <c r="C163" s="3">
+        <v>46181.849305555559</v>
+      </c>
+      <c r="D163">
+        <v>17</v>
+      </c>
+      <c r="E163">
+        <v>31</v>
+      </c>
+      <c r="F163" s="6">
+        <v>1.0532407407407407E-2</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A164">
+        <f t="shared" si="2"/>
+        <v>163</v>
+      </c>
+      <c r="B164">
+        <v>17</v>
+      </c>
+      <c r="C164" s="3">
+        <v>46182.519444444442</v>
+      </c>
+      <c r="D164">
+        <v>31</v>
+      </c>
+      <c r="E164">
+        <v>53</v>
+      </c>
+      <c r="F164" s="6">
+        <v>1.5613425925925926E-2</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A165">
+        <f t="shared" si="2"/>
+        <v>164</v>
+      </c>
+      <c r="B165">
+        <v>17</v>
+      </c>
+      <c r="C165" s="3">
+        <v>46182.84375</v>
+      </c>
+      <c r="D165">
+        <v>53</v>
+      </c>
+      <c r="E165">
+        <v>73</v>
+      </c>
+      <c r="F165" s="6">
+        <v>1.5416666666666667E-2</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A166">
+        <f t="shared" si="2"/>
+        <v>165</v>
+      </c>
+      <c r="B166">
+        <v>17</v>
+      </c>
+      <c r="C166" s="3">
+        <v>46183.890972222223</v>
+      </c>
+      <c r="D166">
+        <v>73</v>
+      </c>
+      <c r="E166">
+        <v>91</v>
+      </c>
+      <c r="F166" s="6">
+        <v>1.2430555555555556E-2</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A167">
+        <f t="shared" si="2"/>
+        <v>166</v>
+      </c>
+      <c r="B167">
+        <v>17</v>
+      </c>
+      <c r="C167" s="3">
+        <v>46184.511111111111</v>
+      </c>
+      <c r="D167">
+        <v>91</v>
+      </c>
+      <c r="E167">
+        <v>111</v>
+      </c>
+      <c r="F167" s="6">
+        <v>1.7500000000000002E-2</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A168">
+        <f t="shared" si="2"/>
+        <v>167</v>
+      </c>
+      <c r="B168">
+        <v>17</v>
+      </c>
+      <c r="C168" s="3">
+        <v>46184.626388888886</v>
+      </c>
+      <c r="D168">
+        <v>111</v>
+      </c>
+      <c r="E168">
+        <v>144</v>
+      </c>
+      <c r="F168" s="6">
+        <v>2.3125E-2</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A169">
+        <f t="shared" si="2"/>
+        <v>168</v>
+      </c>
+      <c r="B169">
+        <v>17</v>
+      </c>
+      <c r="C169" s="3">
+        <v>46184.695138888892</v>
+      </c>
+      <c r="D169">
+        <v>144</v>
+      </c>
+      <c r="E169">
+        <v>157</v>
+      </c>
+      <c r="F169" s="6">
+        <v>7.7314814814814815E-3</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A170">
+        <f t="shared" si="2"/>
+        <v>169</v>
+      </c>
+      <c r="B170">
+        <v>17</v>
+      </c>
+      <c r="C170" s="3">
+        <v>46185.379861111112</v>
+      </c>
+      <c r="D170">
+        <v>157</v>
+      </c>
+      <c r="E170">
+        <v>174</v>
+      </c>
+      <c r="F170" s="6">
+        <v>1.3969907407407407E-2</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A171">
+        <f t="shared" si="2"/>
+        <v>170</v>
+      </c>
+      <c r="B171">
+        <v>17</v>
+      </c>
+      <c r="C171" s="3">
+        <v>46185.621527777781</v>
+      </c>
+      <c r="D171">
+        <v>174</v>
+      </c>
+      <c r="E171">
+        <v>196</v>
+      </c>
+      <c r="F171" s="6">
+        <v>1.6168981481481482E-2</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A172">
+        <f t="shared" si="2"/>
+        <v>171</v>
+      </c>
+      <c r="B172">
+        <v>17</v>
+      </c>
+      <c r="C172" s="3">
+        <v>46185.750694444447</v>
+      </c>
+      <c r="D172">
+        <v>196</v>
+      </c>
+      <c r="E172">
+        <v>207</v>
+      </c>
+      <c r="F172" s="6">
+        <v>8.6458333333333335E-3</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A173">
+        <f t="shared" si="2"/>
+        <v>172</v>
+      </c>
+      <c r="B173">
+        <v>17</v>
+      </c>
+      <c r="C173" s="3">
+        <v>46185.861111111109</v>
+      </c>
+      <c r="D173">
+        <v>207</v>
+      </c>
+      <c r="E173">
+        <v>221</v>
+      </c>
+      <c r="F173" s="6">
+        <v>7.9976851851851858E-3</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A174">
+        <f t="shared" si="2"/>
+        <v>173</v>
+      </c>
+      <c r="B174">
+        <v>17</v>
+      </c>
+      <c r="C174" s="3">
+        <v>46186.5</v>
+      </c>
+      <c r="D174">
+        <v>221</v>
+      </c>
+      <c r="E174">
+        <v>235</v>
+      </c>
+      <c r="F174" s="6">
+        <v>7.951388888888888E-3</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A175">
+        <f t="shared" si="2"/>
+        <v>174</v>
+      </c>
+      <c r="B175">
+        <v>17</v>
+      </c>
+      <c r="C175" s="3">
+        <v>46186.518055555556</v>
+      </c>
+      <c r="D175">
+        <v>235</v>
+      </c>
+      <c r="E175">
+        <v>268</v>
+      </c>
+      <c r="F175" s="6">
+        <v>2.2002314814814815E-2</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A176">
+        <f t="shared" si="2"/>
+        <v>175</v>
+      </c>
+      <c r="B176">
+        <v>17</v>
+      </c>
+      <c r="C176" s="3">
+        <v>46186.558333333334</v>
+      </c>
+      <c r="D176">
+        <v>268</v>
+      </c>
+      <c r="E176">
+        <v>312</v>
+      </c>
+      <c r="F176" s="6">
+        <v>2.613425925925926E-2</v>
       </c>
     </row>
   </sheetData>
@@ -4948,7 +5328,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CC89663-E888-2445-AD16-77803353ADBB}">
-  <dimension ref="A1:E160"/>
+  <dimension ref="A1:E167"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -7400,7 +7780,7 @@
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131">
-        <f t="shared" ref="A131:A160" si="7" xml:space="preserve"> ROW() -1</f>
+        <f t="shared" ref="A131:A167" si="7" xml:space="preserve"> ROW() -1</f>
         <v>130</v>
       </c>
       <c r="B131">
@@ -7984,6 +8364,132 @@
         <v>351</v>
       </c>
     </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A161">
+        <f t="shared" si="7"/>
+        <v>160</v>
+      </c>
+      <c r="B161">
+        <v>17</v>
+      </c>
+      <c r="C161">
+        <v>1</v>
+      </c>
+      <c r="D161" t="s">
+        <v>148</v>
+      </c>
+      <c r="E161">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A162">
+        <f t="shared" si="7"/>
+        <v>161</v>
+      </c>
+      <c r="B162">
+        <v>17</v>
+      </c>
+      <c r="C162">
+        <v>2</v>
+      </c>
+      <c r="D162" t="s">
+        <v>149</v>
+      </c>
+      <c r="E162">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A163">
+        <f t="shared" si="7"/>
+        <v>162</v>
+      </c>
+      <c r="B163">
+        <v>17</v>
+      </c>
+      <c r="C163">
+        <v>3</v>
+      </c>
+      <c r="D163" t="s">
+        <v>150</v>
+      </c>
+      <c r="E163">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A164">
+        <f t="shared" si="7"/>
+        <v>163</v>
+      </c>
+      <c r="B164">
+        <v>17</v>
+      </c>
+      <c r="C164">
+        <v>4</v>
+      </c>
+      <c r="D164" t="s">
+        <v>151</v>
+      </c>
+      <c r="E164">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A165">
+        <f t="shared" si="7"/>
+        <v>164</v>
+      </c>
+      <c r="B165">
+        <v>17</v>
+      </c>
+      <c r="C165">
+        <v>5</v>
+      </c>
+      <c r="D165" t="s">
+        <v>152</v>
+      </c>
+      <c r="E165">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A166">
+        <f t="shared" si="7"/>
+        <v>165</v>
+      </c>
+      <c r="B166">
+        <v>17</v>
+      </c>
+      <c r="C166">
+        <v>6</v>
+      </c>
+      <c r="D166" t="s">
+        <v>153</v>
+      </c>
+      <c r="E166">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A167">
+        <f t="shared" si="7"/>
+        <v>166</v>
+      </c>
+      <c r="B167">
+        <v>17</v>
+      </c>
+      <c r="C167">
+        <v>7</v>
+      </c>
+      <c r="D167" t="s">
+        <v>154</v>
+      </c>
+      <c r="E167">
+        <v>312</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data (A Tale of Two Cities)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/dev/reading-analysis/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/code/projects/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E27D1597-3B0C-8244-B788-624F757C5E9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9763620-1A60-C545-B0D0-0DB3D86D787E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="640" windowWidth="19140" windowHeight="20980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="-20" yWindow="640" windowWidth="19200" windowHeight="20980" activeTab="2" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="202">
   <si>
     <t>book_id</t>
   </si>
@@ -500,6 +500,147 @@
   </si>
   <si>
     <t>The Forged Coupon</t>
+  </si>
+  <si>
+    <t>A Tale of Two Cites</t>
+  </si>
+  <si>
+    <t>Charles Dickens</t>
+  </si>
+  <si>
+    <t>1-1. The Period</t>
+  </si>
+  <si>
+    <t>1-2. The Mail</t>
+  </si>
+  <si>
+    <t>1-3. The Night Shadows</t>
+  </si>
+  <si>
+    <t>1-4. The Preparation</t>
+  </si>
+  <si>
+    <t>1-5. The Wine Shop</t>
+  </si>
+  <si>
+    <t>1-6. The Shoemaker</t>
+  </si>
+  <si>
+    <t>2-1. Five Years Later</t>
+  </si>
+  <si>
+    <t>2-2. A Sight</t>
+  </si>
+  <si>
+    <t>2-3. A Disappointment</t>
+  </si>
+  <si>
+    <t>2-4. Congratulatory</t>
+  </si>
+  <si>
+    <t>2-5. The Jackal</t>
+  </si>
+  <si>
+    <t>2-6. Hundreds of People</t>
+  </si>
+  <si>
+    <t>2-7. Monseigneur in Town</t>
+  </si>
+  <si>
+    <t>2-8. Monseigneur in the Country</t>
+  </si>
+  <si>
+    <t>2-9. The Gorgon's Head</t>
+  </si>
+  <si>
+    <t>2-10. Two Promises</t>
+  </si>
+  <si>
+    <t>2-11. A Companion Picture</t>
+  </si>
+  <si>
+    <t>2-12. The Fellow of Delicacy</t>
+  </si>
+  <si>
+    <t>2-13. The Fellow of No Delicacy</t>
+  </si>
+  <si>
+    <t>2-14. The Honest Tradesman</t>
+  </si>
+  <si>
+    <t>2-16. Still Knitting</t>
+  </si>
+  <si>
+    <t>2-15. Knitting</t>
+  </si>
+  <si>
+    <t>2-17. One Night</t>
+  </si>
+  <si>
+    <t>2-18. Nine Days</t>
+  </si>
+  <si>
+    <t>2-19. An Opinion</t>
+  </si>
+  <si>
+    <t>2-20. A Plea</t>
+  </si>
+  <si>
+    <t>2-21. Echoing footsteps</t>
+  </si>
+  <si>
+    <t>2-22. The Sea Still Rises</t>
+  </si>
+  <si>
+    <t>2-23. Fire Rises</t>
+  </si>
+  <si>
+    <t>2-24. Drawn to the Loadstone Rock</t>
+  </si>
+  <si>
+    <t>3-1. In Secret</t>
+  </si>
+  <si>
+    <t>3-2. The Grindstone</t>
+  </si>
+  <si>
+    <t>3-3. The Shadow</t>
+  </si>
+  <si>
+    <t>3-4. Calm in Storm</t>
+  </si>
+  <si>
+    <t>3-5. The Wood-Sawyer</t>
+  </si>
+  <si>
+    <t>3-6. Triumph</t>
+  </si>
+  <si>
+    <t>3-7. A Knock at the Door</t>
+  </si>
+  <si>
+    <t>3-8. A Hand at Cards</t>
+  </si>
+  <si>
+    <t>3-9. The Game Made</t>
+  </si>
+  <si>
+    <t>3-10. The Substance of the Shadow</t>
+  </si>
+  <si>
+    <t>3-11. Dusk</t>
+  </si>
+  <si>
+    <t>3-12. Darkness</t>
+  </si>
+  <si>
+    <t>3-13. Fifty-two</t>
+  </si>
+  <si>
+    <t>3-15. The Footsteps Die Out For Ever</t>
+  </si>
+  <si>
+    <t>3-14. The Knitting Done</t>
   </si>
 </sst>
 </file>
@@ -554,7 +695,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -565,7 +706,8 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -900,7 +1042,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -909,7 +1051,7 @@
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.6640625" style="7" bestFit="1" customWidth="1"/>
@@ -935,10 +1077,10 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="10" t="s">
         <v>65</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -977,7 +1119,7 @@
       <c r="G2">
         <v>136</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="11">
         <v>38544</v>
       </c>
       <c r="I2" t="s">
@@ -1016,7 +1158,7 @@
       <c r="G3">
         <v>160</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="11">
         <v>36949</v>
       </c>
       <c r="I3" t="s">
@@ -1055,7 +1197,7 @@
       <c r="G4">
         <v>487</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="11">
         <v>205432</v>
       </c>
       <c r="I4" t="s">
@@ -1094,7 +1236,7 @@
       <c r="G5">
         <v>449</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="11">
         <v>136496</v>
       </c>
       <c r="I5" t="s">
@@ -1133,7 +1275,7 @@
       <c r="G6">
         <v>499</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="11">
         <v>142714</v>
       </c>
       <c r="I6" t="s">
@@ -1172,7 +1314,7 @@
       <c r="G7">
         <v>210</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="11">
         <v>53760</v>
       </c>
       <c r="I7" t="s">
@@ -1210,7 +1352,7 @@
       <c r="G8">
         <v>266</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="11" t="s">
         <v>63</v>
       </c>
       <c r="I8" t="s">
@@ -1248,7 +1390,7 @@
       <c r="G9">
         <v>261</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="11">
         <v>105626</v>
       </c>
       <c r="I9" t="s">
@@ -1286,7 +1428,7 @@
       <c r="G10">
         <v>310</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="11">
         <v>105413</v>
       </c>
       <c r="I10" t="s">
@@ -1324,7 +1466,7 @@
       <c r="G11">
         <v>244</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="11">
         <v>90974</v>
       </c>
       <c r="I11" t="s">
@@ -1362,7 +1504,7 @@
       <c r="G12">
         <v>490</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="11">
         <v>130823</v>
       </c>
       <c r="I12" t="s">
@@ -1400,7 +1542,7 @@
       <c r="G13">
         <v>432</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="11">
         <v>121312</v>
       </c>
       <c r="I13" t="s">
@@ -1438,7 +1580,7 @@
       <c r="G14">
         <v>309</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="11">
         <v>85019</v>
       </c>
       <c r="I14" t="s">
@@ -1476,7 +1618,7 @@
       <c r="G15">
         <v>348</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="11">
         <v>116376</v>
       </c>
       <c r="I15" t="s">
@@ -1514,7 +1656,7 @@
       <c r="G16">
         <v>527</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="11">
         <v>200177</v>
       </c>
       <c r="I16" t="s">
@@ -1552,7 +1694,7 @@
       <c r="G17">
         <v>106</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="11">
         <v>25711</v>
       </c>
       <c r="I17" t="s">
@@ -1590,7 +1732,7 @@
       <c r="G18">
         <v>309</v>
       </c>
-      <c r="H18" s="10">
+      <c r="H18" s="11">
         <v>108141</v>
       </c>
       <c r="I18" t="s">
@@ -1604,6 +1746,44 @@
       </c>
       <c r="L18" s="7">
         <v>46186</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>155</v>
+      </c>
+      <c r="C19" t="s">
+        <v>156</v>
+      </c>
+      <c r="D19" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19">
+        <v>1859</v>
+      </c>
+      <c r="F19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19">
+        <v>379</v>
+      </c>
+      <c r="H19" s="11">
+        <v>136367</v>
+      </c>
+      <c r="I19" t="s">
+        <v>104</v>
+      </c>
+      <c r="J19" t="s">
+        <v>67</v>
+      </c>
+      <c r="K19" s="7">
+        <v>46187</v>
+      </c>
+      <c r="L19" s="7">
+        <v>46194</v>
       </c>
     </row>
   </sheetData>
@@ -1613,7 +1793,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I176"/>
+  <dimension ref="A1:I200"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -4357,7 +4537,7 @@
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131">
-        <f t="shared" ref="A131:A176" si="2">ROW() - 1</f>
+        <f t="shared" ref="A131:A194" si="2">ROW() - 1</f>
         <v>130</v>
       </c>
       <c r="B131">
@@ -5319,6 +5499,510 @@
       </c>
       <c r="F176" s="6">
         <v>2.613425925925926E-2</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A177">
+        <f t="shared" si="2"/>
+        <v>176</v>
+      </c>
+      <c r="B177">
+        <v>18</v>
+      </c>
+      <c r="C177" s="3">
+        <v>46187.836805555555</v>
+      </c>
+      <c r="D177">
+        <v>7</v>
+      </c>
+      <c r="E177">
+        <v>20</v>
+      </c>
+      <c r="F177" s="6">
+        <v>1.5844907407407408E-2</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A178">
+        <f t="shared" si="2"/>
+        <v>177</v>
+      </c>
+      <c r="B178">
+        <v>18</v>
+      </c>
+      <c r="C178" s="3">
+        <v>46187.947916666664</v>
+      </c>
+      <c r="D178">
+        <v>20</v>
+      </c>
+      <c r="E178">
+        <v>32</v>
+      </c>
+      <c r="F178" s="6">
+        <v>1.3715277777777778E-2</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A179">
+        <f t="shared" si="2"/>
+        <v>178</v>
+      </c>
+      <c r="B179">
+        <v>18</v>
+      </c>
+      <c r="C179" s="3">
+        <v>46188.484722222223</v>
+      </c>
+      <c r="D179">
+        <v>32</v>
+      </c>
+      <c r="E179">
+        <v>57</v>
+      </c>
+      <c r="F179" s="6">
+        <v>1.9108796296296297E-2</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A180">
+        <f t="shared" si="2"/>
+        <v>179</v>
+      </c>
+      <c r="B180">
+        <v>18</v>
+      </c>
+      <c r="C180" s="3">
+        <v>46188.568749999999</v>
+      </c>
+      <c r="D180">
+        <v>57</v>
+      </c>
+      <c r="E180">
+        <v>70</v>
+      </c>
+      <c r="F180" s="6">
+        <v>1.2337962962962964E-2</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A181">
+        <f t="shared" si="2"/>
+        <v>180</v>
+      </c>
+      <c r="B181">
+        <v>18</v>
+      </c>
+      <c r="C181" s="3">
+        <v>46188.706944444442</v>
+      </c>
+      <c r="D181">
+        <v>70</v>
+      </c>
+      <c r="E181">
+        <v>90</v>
+      </c>
+      <c r="F181" s="6">
+        <v>1.6886574074074075E-2</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A182">
+        <f t="shared" si="2"/>
+        <v>181</v>
+      </c>
+      <c r="B182">
+        <v>18</v>
+      </c>
+      <c r="C182" s="3">
+        <v>46189.550694444442</v>
+      </c>
+      <c r="D182">
+        <v>90</v>
+      </c>
+      <c r="E182">
+        <v>109</v>
+      </c>
+      <c r="F182" s="6">
+        <v>1.8287037037037036E-2</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A183">
+        <f t="shared" si="2"/>
+        <v>182</v>
+      </c>
+      <c r="B183">
+        <v>18</v>
+      </c>
+      <c r="C183" s="3">
+        <v>46189.681250000001</v>
+      </c>
+      <c r="D183">
+        <v>109</v>
+      </c>
+      <c r="E183">
+        <v>118</v>
+      </c>
+      <c r="F183" s="6">
+        <v>9.7337962962962959E-3</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A184">
+        <f t="shared" si="2"/>
+        <v>183</v>
+      </c>
+      <c r="B184">
+        <v>18</v>
+      </c>
+      <c r="C184" s="3">
+        <v>46189.709722222222</v>
+      </c>
+      <c r="D184">
+        <v>118</v>
+      </c>
+      <c r="E184">
+        <v>123</v>
+      </c>
+      <c r="F184" s="6">
+        <v>5.9490740740740745E-3</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A185">
+        <f t="shared" si="2"/>
+        <v>184</v>
+      </c>
+      <c r="B185">
+        <v>18</v>
+      </c>
+      <c r="C185" s="3">
+        <v>46189.819444444445</v>
+      </c>
+      <c r="D185">
+        <v>123</v>
+      </c>
+      <c r="E185">
+        <v>135</v>
+      </c>
+      <c r="F185" s="6">
+        <v>1.1064814814814816E-2</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A186">
+        <f t="shared" si="2"/>
+        <v>185</v>
+      </c>
+      <c r="B186">
+        <v>18</v>
+      </c>
+      <c r="C186" s="3">
+        <v>46190.748611111114</v>
+      </c>
+      <c r="D186">
+        <v>135</v>
+      </c>
+      <c r="E186">
+        <v>147</v>
+      </c>
+      <c r="F186" s="6">
+        <v>9.0162037037037034E-3</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A187">
+        <f t="shared" si="2"/>
+        <v>186</v>
+      </c>
+      <c r="B187">
+        <v>18</v>
+      </c>
+      <c r="C187" s="3">
+        <v>46190.890972222223</v>
+      </c>
+      <c r="D187">
+        <v>147</v>
+      </c>
+      <c r="E187">
+        <v>159</v>
+      </c>
+      <c r="F187" s="6">
+        <v>9.4675925925925934E-3</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A188">
+        <f t="shared" si="2"/>
+        <v>187</v>
+      </c>
+      <c r="B188">
+        <v>18</v>
+      </c>
+      <c r="C188" s="3">
+        <v>46191.899305555555</v>
+      </c>
+      <c r="D188">
+        <v>159</v>
+      </c>
+      <c r="E188">
+        <v>181</v>
+      </c>
+      <c r="F188" s="6">
+        <v>1.8865740740740742E-2</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A189">
+        <f t="shared" si="2"/>
+        <v>188</v>
+      </c>
+      <c r="B189">
+        <v>18</v>
+      </c>
+      <c r="C189" s="3">
+        <v>46192.59097222222</v>
+      </c>
+      <c r="D189">
+        <v>181</v>
+      </c>
+      <c r="E189">
+        <v>192</v>
+      </c>
+      <c r="F189" s="6">
+        <v>1.0347222222222223E-2</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A190">
+        <f t="shared" si="2"/>
+        <v>189</v>
+      </c>
+      <c r="B190">
+        <v>18</v>
+      </c>
+      <c r="C190" s="3">
+        <v>46192.634027777778</v>
+      </c>
+      <c r="D190">
+        <v>192</v>
+      </c>
+      <c r="E190">
+        <v>204</v>
+      </c>
+      <c r="F190" s="6">
+        <v>9.5023148148148141E-3</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A191">
+        <f t="shared" si="2"/>
+        <v>190</v>
+      </c>
+      <c r="B191">
+        <v>18</v>
+      </c>
+      <c r="C191" s="3">
+        <v>46192.668055555558</v>
+      </c>
+      <c r="D191">
+        <v>204</v>
+      </c>
+      <c r="E191">
+        <v>227</v>
+      </c>
+      <c r="F191" s="6">
+        <v>1.8078703703703704E-2</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A192">
+        <f t="shared" si="2"/>
+        <v>191</v>
+      </c>
+      <c r="B192">
+        <v>18</v>
+      </c>
+      <c r="C192" s="3">
+        <v>46193.4375</v>
+      </c>
+      <c r="D192">
+        <v>227</v>
+      </c>
+      <c r="E192">
+        <v>255</v>
+      </c>
+      <c r="F192" s="6">
+        <v>2.1956018518518517E-2</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A193">
+        <f t="shared" si="2"/>
+        <v>192</v>
+      </c>
+      <c r="B193">
+        <v>18</v>
+      </c>
+      <c r="C193" s="3">
+        <v>46193.538194444445</v>
+      </c>
+      <c r="D193">
+        <v>255</v>
+      </c>
+      <c r="E193">
+        <v>267</v>
+      </c>
+      <c r="F193" s="6">
+        <v>9.9305555555555553E-3</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A194">
+        <f t="shared" si="2"/>
+        <v>193</v>
+      </c>
+      <c r="B194">
+        <v>18</v>
+      </c>
+      <c r="C194" s="3">
+        <v>46193.570138888892</v>
+      </c>
+      <c r="D194">
+        <v>267</v>
+      </c>
+      <c r="E194">
+        <v>278</v>
+      </c>
+      <c r="F194" s="6">
+        <v>9.6296296296296303E-3</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A195">
+        <f t="shared" ref="A195:A200" si="3">ROW() - 1</f>
+        <v>194</v>
+      </c>
+      <c r="B195">
+        <v>18</v>
+      </c>
+      <c r="C195" s="3">
+        <v>46193.8125</v>
+      </c>
+      <c r="D195">
+        <v>278</v>
+      </c>
+      <c r="E195">
+        <v>284</v>
+      </c>
+      <c r="F195" s="6">
+        <v>5.1736111111111115E-3</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A196">
+        <f t="shared" si="3"/>
+        <v>195</v>
+      </c>
+      <c r="B196">
+        <v>18</v>
+      </c>
+      <c r="C196" s="3">
+        <v>46193.834027777775</v>
+      </c>
+      <c r="D196">
+        <v>284</v>
+      </c>
+      <c r="E196">
+        <v>302</v>
+      </c>
+      <c r="F196" s="6">
+        <v>1.4525462962962962E-2</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A197">
+        <f t="shared" si="3"/>
+        <v>196</v>
+      </c>
+      <c r="B197">
+        <v>18</v>
+      </c>
+      <c r="C197" s="3">
+        <v>46194.553472222222</v>
+      </c>
+      <c r="D197">
+        <v>302</v>
+      </c>
+      <c r="E197">
+        <v>328</v>
+      </c>
+      <c r="F197" s="6">
+        <v>1.9780092592592592E-2</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A198">
+        <f t="shared" si="3"/>
+        <v>197</v>
+      </c>
+      <c r="B198">
+        <v>18</v>
+      </c>
+      <c r="C198" s="3">
+        <v>46194.663194444445</v>
+      </c>
+      <c r="D198">
+        <v>328</v>
+      </c>
+      <c r="E198">
+        <v>343</v>
+      </c>
+      <c r="F198" s="6">
+        <v>1.1412037037037037E-2</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A199">
+        <f t="shared" si="3"/>
+        <v>198</v>
+      </c>
+      <c r="B199">
+        <v>18</v>
+      </c>
+      <c r="C199" s="3">
+        <v>46194.694444444445</v>
+      </c>
+      <c r="D199">
+        <v>343</v>
+      </c>
+      <c r="E199">
+        <v>356</v>
+      </c>
+      <c r="F199" s="6">
+        <v>8.9351851851851849E-3</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A200">
+        <f t="shared" si="3"/>
+        <v>199</v>
+      </c>
+      <c r="B200">
+        <v>18</v>
+      </c>
+      <c r="C200" s="3">
+        <v>46194.756249999999</v>
+      </c>
+      <c r="D200">
+        <v>356</v>
+      </c>
+      <c r="E200">
+        <v>386</v>
+      </c>
+      <c r="F200" s="6">
+        <v>2.2037037037037036E-2</v>
       </c>
     </row>
   </sheetData>
@@ -5328,7 +6012,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CC89663-E888-2445-AD16-77803353ADBB}">
-  <dimension ref="A1:E167"/>
+  <dimension ref="A1:E212"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -7780,7 +8464,7 @@
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131">
-        <f t="shared" ref="A131:A167" si="7" xml:space="preserve"> ROW() -1</f>
+        <f t="shared" ref="A131:A194" si="7" xml:space="preserve"> ROW() -1</f>
         <v>130</v>
       </c>
       <c r="B131">
@@ -8490,6 +9174,860 @@
         <v>312</v>
       </c>
     </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A168">
+        <f t="shared" si="7"/>
+        <v>167</v>
+      </c>
+      <c r="B168">
+        <v>18</v>
+      </c>
+      <c r="C168">
+        <v>1</v>
+      </c>
+      <c r="D168" t="s">
+        <v>157</v>
+      </c>
+      <c r="E168">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A169">
+        <f t="shared" si="7"/>
+        <v>168</v>
+      </c>
+      <c r="B169">
+        <v>18</v>
+      </c>
+      <c r="C169">
+        <f>C168+1</f>
+        <v>2</v>
+      </c>
+      <c r="D169" t="s">
+        <v>158</v>
+      </c>
+      <c r="E169">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A170">
+        <f t="shared" si="7"/>
+        <v>169</v>
+      </c>
+      <c r="B170">
+        <v>18</v>
+      </c>
+      <c r="C170">
+        <f t="shared" ref="C170:C212" si="10">C169+1</f>
+        <v>3</v>
+      </c>
+      <c r="D170" t="s">
+        <v>159</v>
+      </c>
+      <c r="E170">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A171">
+        <f t="shared" si="7"/>
+        <v>170</v>
+      </c>
+      <c r="B171">
+        <v>18</v>
+      </c>
+      <c r="C171">
+        <f t="shared" si="10"/>
+        <v>4</v>
+      </c>
+      <c r="D171" t="s">
+        <v>160</v>
+      </c>
+      <c r="E171">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A172">
+        <f t="shared" si="7"/>
+        <v>171</v>
+      </c>
+      <c r="B172">
+        <v>18</v>
+      </c>
+      <c r="C172">
+        <f t="shared" si="10"/>
+        <v>5</v>
+      </c>
+      <c r="D172" t="s">
+        <v>161</v>
+      </c>
+      <c r="E172">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A173">
+        <f t="shared" si="7"/>
+        <v>172</v>
+      </c>
+      <c r="B173">
+        <v>18</v>
+      </c>
+      <c r="C173">
+        <f t="shared" si="10"/>
+        <v>6</v>
+      </c>
+      <c r="D173" t="s">
+        <v>162</v>
+      </c>
+      <c r="E173">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A174">
+        <f t="shared" si="7"/>
+        <v>173</v>
+      </c>
+      <c r="B174">
+        <v>18</v>
+      </c>
+      <c r="C174">
+        <f t="shared" si="10"/>
+        <v>7</v>
+      </c>
+      <c r="D174" t="s">
+        <v>163</v>
+      </c>
+      <c r="E174">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A175">
+        <f t="shared" si="7"/>
+        <v>174</v>
+      </c>
+      <c r="B175">
+        <v>18</v>
+      </c>
+      <c r="C175">
+        <f t="shared" si="10"/>
+        <v>8</v>
+      </c>
+      <c r="D175" t="s">
+        <v>164</v>
+      </c>
+      <c r="E175">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A176">
+        <f t="shared" si="7"/>
+        <v>175</v>
+      </c>
+      <c r="B176">
+        <v>18</v>
+      </c>
+      <c r="C176">
+        <f t="shared" si="10"/>
+        <v>9</v>
+      </c>
+      <c r="D176" t="s">
+        <v>165</v>
+      </c>
+      <c r="E176">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A177">
+        <f t="shared" si="7"/>
+        <v>176</v>
+      </c>
+      <c r="B177">
+        <v>18</v>
+      </c>
+      <c r="C177">
+        <f t="shared" si="10"/>
+        <v>10</v>
+      </c>
+      <c r="D177" t="s">
+        <v>166</v>
+      </c>
+      <c r="E177">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A178">
+        <f t="shared" si="7"/>
+        <v>177</v>
+      </c>
+      <c r="B178">
+        <v>18</v>
+      </c>
+      <c r="C178">
+        <f t="shared" si="10"/>
+        <v>11</v>
+      </c>
+      <c r="D178" t="s">
+        <v>167</v>
+      </c>
+      <c r="E178">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A179">
+        <f t="shared" si="7"/>
+        <v>178</v>
+      </c>
+      <c r="B179">
+        <v>18</v>
+      </c>
+      <c r="C179">
+        <f t="shared" si="10"/>
+        <v>12</v>
+      </c>
+      <c r="D179" t="s">
+        <v>168</v>
+      </c>
+      <c r="E179">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A180">
+        <f t="shared" si="7"/>
+        <v>179</v>
+      </c>
+      <c r="B180">
+        <v>18</v>
+      </c>
+      <c r="C180">
+        <f t="shared" si="10"/>
+        <v>13</v>
+      </c>
+      <c r="D180" t="s">
+        <v>169</v>
+      </c>
+      <c r="E180">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A181">
+        <f t="shared" si="7"/>
+        <v>180</v>
+      </c>
+      <c r="B181">
+        <v>18</v>
+      </c>
+      <c r="C181">
+        <f t="shared" si="10"/>
+        <v>14</v>
+      </c>
+      <c r="D181" t="s">
+        <v>170</v>
+      </c>
+      <c r="E181">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A182">
+        <f t="shared" si="7"/>
+        <v>181</v>
+      </c>
+      <c r="B182">
+        <v>18</v>
+      </c>
+      <c r="C182">
+        <f t="shared" si="10"/>
+        <v>15</v>
+      </c>
+      <c r="D182" t="s">
+        <v>171</v>
+      </c>
+      <c r="E182">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A183">
+        <f t="shared" si="7"/>
+        <v>182</v>
+      </c>
+      <c r="B183">
+        <v>18</v>
+      </c>
+      <c r="C183">
+        <f t="shared" si="10"/>
+        <v>16</v>
+      </c>
+      <c r="D183" t="s">
+        <v>172</v>
+      </c>
+      <c r="E183">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A184">
+        <f t="shared" si="7"/>
+        <v>183</v>
+      </c>
+      <c r="B184">
+        <v>18</v>
+      </c>
+      <c r="C184">
+        <f t="shared" si="10"/>
+        <v>17</v>
+      </c>
+      <c r="D184" t="s">
+        <v>173</v>
+      </c>
+      <c r="E184">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A185">
+        <f t="shared" si="7"/>
+        <v>184</v>
+      </c>
+      <c r="B185">
+        <v>18</v>
+      </c>
+      <c r="C185">
+        <f t="shared" si="10"/>
+        <v>18</v>
+      </c>
+      <c r="D185" t="s">
+        <v>174</v>
+      </c>
+      <c r="E185">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A186">
+        <f t="shared" si="7"/>
+        <v>185</v>
+      </c>
+      <c r="B186">
+        <v>18</v>
+      </c>
+      <c r="C186">
+        <f t="shared" si="10"/>
+        <v>19</v>
+      </c>
+      <c r="D186" t="s">
+        <v>175</v>
+      </c>
+      <c r="E186">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A187">
+        <f t="shared" si="7"/>
+        <v>186</v>
+      </c>
+      <c r="B187">
+        <v>18</v>
+      </c>
+      <c r="C187">
+        <f t="shared" si="10"/>
+        <v>20</v>
+      </c>
+      <c r="D187" t="s">
+        <v>176</v>
+      </c>
+      <c r="E187">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A188">
+        <f t="shared" si="7"/>
+        <v>187</v>
+      </c>
+      <c r="B188">
+        <v>18</v>
+      </c>
+      <c r="C188">
+        <f t="shared" si="10"/>
+        <v>21</v>
+      </c>
+      <c r="D188" t="s">
+        <v>178</v>
+      </c>
+      <c r="E188">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A189">
+        <f t="shared" si="7"/>
+        <v>188</v>
+      </c>
+      <c r="B189">
+        <v>18</v>
+      </c>
+      <c r="C189">
+        <f t="shared" si="10"/>
+        <v>22</v>
+      </c>
+      <c r="D189" t="s">
+        <v>177</v>
+      </c>
+      <c r="E189">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A190">
+        <f t="shared" si="7"/>
+        <v>189</v>
+      </c>
+      <c r="B190">
+        <v>18</v>
+      </c>
+      <c r="C190">
+        <f t="shared" si="10"/>
+        <v>23</v>
+      </c>
+      <c r="D190" t="s">
+        <v>179</v>
+      </c>
+      <c r="E190">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A191">
+        <f t="shared" si="7"/>
+        <v>190</v>
+      </c>
+      <c r="B191">
+        <v>18</v>
+      </c>
+      <c r="C191">
+        <f t="shared" si="10"/>
+        <v>24</v>
+      </c>
+      <c r="D191" t="s">
+        <v>180</v>
+      </c>
+      <c r="E191">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A192">
+        <f t="shared" si="7"/>
+        <v>191</v>
+      </c>
+      <c r="B192">
+        <v>18</v>
+      </c>
+      <c r="C192">
+        <f t="shared" si="10"/>
+        <v>25</v>
+      </c>
+      <c r="D192" t="s">
+        <v>181</v>
+      </c>
+      <c r="E192">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A193">
+        <f t="shared" si="7"/>
+        <v>192</v>
+      </c>
+      <c r="B193">
+        <v>18</v>
+      </c>
+      <c r="C193">
+        <f t="shared" si="10"/>
+        <v>26</v>
+      </c>
+      <c r="D193" t="s">
+        <v>182</v>
+      </c>
+      <c r="E193">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A194">
+        <f t="shared" si="7"/>
+        <v>193</v>
+      </c>
+      <c r="B194">
+        <v>18</v>
+      </c>
+      <c r="C194">
+        <f t="shared" si="10"/>
+        <v>27</v>
+      </c>
+      <c r="D194" t="s">
+        <v>183</v>
+      </c>
+      <c r="E194">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A195">
+        <f t="shared" ref="A195:A212" si="11" xml:space="preserve"> ROW() -1</f>
+        <v>194</v>
+      </c>
+      <c r="B195">
+        <v>18</v>
+      </c>
+      <c r="C195">
+        <f t="shared" si="10"/>
+        <v>28</v>
+      </c>
+      <c r="D195" t="s">
+        <v>184</v>
+      </c>
+      <c r="E195">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A196">
+        <f t="shared" si="11"/>
+        <v>195</v>
+      </c>
+      <c r="B196">
+        <v>18</v>
+      </c>
+      <c r="C196">
+        <f t="shared" si="10"/>
+        <v>29</v>
+      </c>
+      <c r="D196" t="s">
+        <v>185</v>
+      </c>
+      <c r="E196">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A197">
+        <f t="shared" si="11"/>
+        <v>196</v>
+      </c>
+      <c r="B197">
+        <v>18</v>
+      </c>
+      <c r="C197">
+        <f t="shared" si="10"/>
+        <v>30</v>
+      </c>
+      <c r="D197" t="s">
+        <v>186</v>
+      </c>
+      <c r="E197">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A198">
+        <f t="shared" si="11"/>
+        <v>197</v>
+      </c>
+      <c r="B198">
+        <v>18</v>
+      </c>
+      <c r="C198">
+        <f t="shared" si="10"/>
+        <v>31</v>
+      </c>
+      <c r="D198" t="s">
+        <v>187</v>
+      </c>
+      <c r="E198">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A199">
+        <f t="shared" si="11"/>
+        <v>198</v>
+      </c>
+      <c r="B199">
+        <v>18</v>
+      </c>
+      <c r="C199">
+        <f t="shared" si="10"/>
+        <v>32</v>
+      </c>
+      <c r="D199" t="s">
+        <v>188</v>
+      </c>
+      <c r="E199">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A200">
+        <f t="shared" si="11"/>
+        <v>199</v>
+      </c>
+      <c r="B200">
+        <v>18</v>
+      </c>
+      <c r="C200">
+        <f t="shared" si="10"/>
+        <v>33</v>
+      </c>
+      <c r="D200" t="s">
+        <v>189</v>
+      </c>
+      <c r="E200">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A201">
+        <f t="shared" si="11"/>
+        <v>200</v>
+      </c>
+      <c r="B201">
+        <v>18</v>
+      </c>
+      <c r="C201">
+        <f t="shared" si="10"/>
+        <v>34</v>
+      </c>
+      <c r="D201" t="s">
+        <v>190</v>
+      </c>
+      <c r="E201">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A202">
+        <f t="shared" si="11"/>
+        <v>201</v>
+      </c>
+      <c r="B202">
+        <v>18</v>
+      </c>
+      <c r="C202">
+        <f t="shared" si="10"/>
+        <v>35</v>
+      </c>
+      <c r="D202" t="s">
+        <v>191</v>
+      </c>
+      <c r="E202">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A203">
+        <f t="shared" si="11"/>
+        <v>202</v>
+      </c>
+      <c r="B203">
+        <v>18</v>
+      </c>
+      <c r="C203">
+        <f t="shared" si="10"/>
+        <v>36</v>
+      </c>
+      <c r="D203" t="s">
+        <v>192</v>
+      </c>
+      <c r="E203">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A204">
+        <f t="shared" si="11"/>
+        <v>203</v>
+      </c>
+      <c r="B204">
+        <v>18</v>
+      </c>
+      <c r="C204">
+        <f t="shared" si="10"/>
+        <v>37</v>
+      </c>
+      <c r="D204" t="s">
+        <v>193</v>
+      </c>
+      <c r="E204">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A205">
+        <f t="shared" si="11"/>
+        <v>204</v>
+      </c>
+      <c r="B205">
+        <v>18</v>
+      </c>
+      <c r="C205">
+        <f t="shared" si="10"/>
+        <v>38</v>
+      </c>
+      <c r="D205" t="s">
+        <v>194</v>
+      </c>
+      <c r="E205">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A206">
+        <f t="shared" si="11"/>
+        <v>205</v>
+      </c>
+      <c r="B206">
+        <v>18</v>
+      </c>
+      <c r="C206">
+        <f t="shared" si="10"/>
+        <v>39</v>
+      </c>
+      <c r="D206" t="s">
+        <v>195</v>
+      </c>
+      <c r="E206">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A207">
+        <f t="shared" si="11"/>
+        <v>206</v>
+      </c>
+      <c r="B207">
+        <v>18</v>
+      </c>
+      <c r="C207">
+        <f t="shared" si="10"/>
+        <v>40</v>
+      </c>
+      <c r="D207" t="s">
+        <v>196</v>
+      </c>
+      <c r="E207">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A208">
+        <f t="shared" si="11"/>
+        <v>207</v>
+      </c>
+      <c r="B208">
+        <v>18</v>
+      </c>
+      <c r="C208">
+        <f t="shared" si="10"/>
+        <v>41</v>
+      </c>
+      <c r="D208" t="s">
+        <v>197</v>
+      </c>
+      <c r="E208">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A209">
+        <f t="shared" si="11"/>
+        <v>208</v>
+      </c>
+      <c r="B209">
+        <v>18</v>
+      </c>
+      <c r="C209">
+        <f t="shared" si="10"/>
+        <v>42</v>
+      </c>
+      <c r="D209" t="s">
+        <v>198</v>
+      </c>
+      <c r="E209">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A210">
+        <f t="shared" si="11"/>
+        <v>209</v>
+      </c>
+      <c r="B210">
+        <v>18</v>
+      </c>
+      <c r="C210">
+        <f t="shared" si="10"/>
+        <v>43</v>
+      </c>
+      <c r="D210" t="s">
+        <v>199</v>
+      </c>
+      <c r="E210">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A211">
+        <f t="shared" si="11"/>
+        <v>210</v>
+      </c>
+      <c r="B211">
+        <v>18</v>
+      </c>
+      <c r="C211">
+        <f t="shared" si="10"/>
+        <v>44</v>
+      </c>
+      <c r="D211" t="s">
+        <v>201</v>
+      </c>
+      <c r="E211">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A212">
+        <f t="shared" si="11"/>
+        <v>211</v>
+      </c>
+      <c r="B212">
+        <v>18</v>
+      </c>
+      <c r="C212">
+        <f t="shared" si="10"/>
+        <v>45</v>
+      </c>
+      <c r="D212" t="s">
+        <v>200</v>
+      </c>
+      <c r="E212">
+        <v>387</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data (2 S.K Books + Friday)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/code/projects/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9763620-1A60-C545-B0D0-0DB3D86D787E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F7900B-2BF9-6147-AC01-E1A6CE576E48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="640" windowWidth="19200" windowHeight="20980" activeTab="2" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="15040" windowHeight="18980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="209">
   <si>
     <t>book_id</t>
   </si>
@@ -641,6 +641,27 @@
   </si>
   <si>
     <t>3-14. The Knitting Done</t>
+  </si>
+  <si>
+    <t>Christine</t>
+  </si>
+  <si>
+    <t>mixed</t>
+  </si>
+  <si>
+    <t>Cycle of the Werewolf</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>Michel Tournier</t>
+  </si>
+  <si>
+    <t>Prologue</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -695,7 +716,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -708,6 +729,10 @@
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1042,7 +1067,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -1051,6 +1076,7 @@
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" style="13"/>
     <col min="8" max="8" width="10.6640625" style="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.1640625" bestFit="1" customWidth="1"/>
@@ -1077,7 +1103,7 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="12" t="s">
         <v>64</v>
       </c>
       <c r="H1" s="10" t="s">
@@ -1116,7 +1142,7 @@
       <c r="F2" t="s">
         <v>16</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="13">
         <v>136</v>
       </c>
       <c r="H2" s="11">
@@ -1155,7 +1181,7 @@
       <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="13">
         <v>160</v>
       </c>
       <c r="H3" s="11">
@@ -1194,7 +1220,7 @@
       <c r="F4" t="s">
         <v>16</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="13">
         <v>487</v>
       </c>
       <c r="H4" s="11">
@@ -1233,7 +1259,7 @@
       <c r="F5" t="s">
         <v>16</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="13">
         <v>449</v>
       </c>
       <c r="H5" s="11">
@@ -1272,7 +1298,7 @@
       <c r="F6" t="s">
         <v>16</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="13">
         <v>499</v>
       </c>
       <c r="H6" s="11">
@@ -1311,7 +1337,7 @@
       <c r="F7" t="s">
         <v>16</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="13">
         <v>210</v>
       </c>
       <c r="H7" s="11">
@@ -1349,7 +1375,7 @@
       <c r="F8" t="s">
         <v>16</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="13">
         <v>266</v>
       </c>
       <c r="H8" s="11" t="s">
@@ -1387,7 +1413,7 @@
       <c r="F9" t="s">
         <v>16</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="13">
         <v>261</v>
       </c>
       <c r="H9" s="11">
@@ -1425,7 +1451,7 @@
       <c r="F10" t="s">
         <v>16</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="13">
         <v>310</v>
       </c>
       <c r="H10" s="11">
@@ -1463,7 +1489,7 @@
       <c r="F11" t="s">
         <v>16</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="13">
         <v>244</v>
       </c>
       <c r="H11" s="11">
@@ -1501,7 +1527,7 @@
       <c r="F12" t="s">
         <v>16</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="13">
         <v>490</v>
       </c>
       <c r="H12" s="11">
@@ -1539,7 +1565,7 @@
       <c r="F13" t="s">
         <v>16</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="13">
         <v>432</v>
       </c>
       <c r="H13" s="11">
@@ -1577,7 +1603,7 @@
       <c r="F14" t="s">
         <v>130</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="13">
         <v>309</v>
       </c>
       <c r="H14" s="11">
@@ -1615,7 +1641,7 @@
       <c r="F15" t="s">
         <v>16</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="13">
         <v>348</v>
       </c>
       <c r="H15" s="11">
@@ -1653,7 +1679,7 @@
       <c r="F16" t="s">
         <v>130</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="13">
         <v>527</v>
       </c>
       <c r="H16" s="11">
@@ -1691,7 +1717,7 @@
       <c r="F17" t="s">
         <v>16</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="13">
         <v>106</v>
       </c>
       <c r="H17" s="11">
@@ -1729,7 +1755,7 @@
       <c r="F18" t="s">
         <v>16</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="13">
         <v>309</v>
       </c>
       <c r="H18" s="11">
@@ -1767,7 +1793,7 @@
       <c r="F19" t="s">
         <v>16</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="13">
         <v>379</v>
       </c>
       <c r="H19" s="11">
@@ -1784,6 +1810,125 @@
       </c>
       <c r="L19" s="7">
         <v>46194</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>202</v>
+      </c>
+      <c r="C20" t="s">
+        <v>140</v>
+      </c>
+      <c r="D20" t="s">
+        <v>141</v>
+      </c>
+      <c r="E20">
+        <v>1983</v>
+      </c>
+      <c r="F20" t="s">
+        <v>203</v>
+      </c>
+      <c r="G20" s="13">
+        <v>644</v>
+      </c>
+      <c r="H20" s="11">
+        <v>193735</v>
+      </c>
+      <c r="I20" t="s">
+        <v>104</v>
+      </c>
+      <c r="J20" t="s">
+        <v>67</v>
+      </c>
+      <c r="K20" s="7">
+        <v>46195</v>
+      </c>
+      <c r="L20" s="7">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>204</v>
+      </c>
+      <c r="C21" t="s">
+        <v>140</v>
+      </c>
+      <c r="D21" t="s">
+        <v>141</v>
+      </c>
+      <c r="E21">
+        <v>1983</v>
+      </c>
+      <c r="F21" t="s">
+        <v>16</v>
+      </c>
+      <c r="G21" s="13">
+        <v>114</v>
+      </c>
+      <c r="H21" s="11">
+        <v>16022</v>
+      </c>
+      <c r="I21" t="s">
+        <v>104</v>
+      </c>
+      <c r="J21" t="s">
+        <v>81</v>
+      </c>
+      <c r="K21" s="7">
+        <v>46197</v>
+      </c>
+      <c r="L21" s="7">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>205</v>
+      </c>
+      <c r="C22" t="s">
+        <v>206</v>
+      </c>
+      <c r="D22" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22">
+        <v>1967</v>
+      </c>
+      <c r="F22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G22" s="13">
+        <v>226</v>
+      </c>
+      <c r="H22" s="11">
+        <v>64666</v>
+      </c>
+      <c r="I22" t="s">
+        <v>105</v>
+      </c>
+      <c r="J22" t="s">
+        <v>67</v>
+      </c>
+      <c r="K22" s="7">
+        <v>46198</v>
+      </c>
+      <c r="L22" s="7">
+        <v>46201</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="I23" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -1793,7 +1938,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I200"/>
+  <dimension ref="A1:I230"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -5881,7 +6026,7 @@
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A195">
-        <f t="shared" ref="A195:A200" si="3">ROW() - 1</f>
+        <f t="shared" ref="A195:A230" si="3">ROW() - 1</f>
         <v>194</v>
       </c>
       <c r="B195">
@@ -6003,6 +6148,636 @@
       </c>
       <c r="F200" s="6">
         <v>2.2037037037037036E-2</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A201">
+        <f t="shared" si="3"/>
+        <v>200</v>
+      </c>
+      <c r="B201">
+        <v>19</v>
+      </c>
+      <c r="C201" s="3">
+        <v>46195.57708333333</v>
+      </c>
+      <c r="D201">
+        <v>1</v>
+      </c>
+      <c r="E201">
+        <v>29</v>
+      </c>
+      <c r="F201" s="6">
+        <v>1.6064814814814816E-2</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A202">
+        <f t="shared" si="3"/>
+        <v>201</v>
+      </c>
+      <c r="B202">
+        <v>19</v>
+      </c>
+      <c r="C202" s="3">
+        <v>46195.604861111111</v>
+      </c>
+      <c r="D202">
+        <v>29</v>
+      </c>
+      <c r="E202">
+        <v>67</v>
+      </c>
+      <c r="F202" s="6">
+        <v>2.0150462962962964E-2</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A203">
+        <f t="shared" si="3"/>
+        <v>202</v>
+      </c>
+      <c r="B203">
+        <v>19</v>
+      </c>
+      <c r="C203" s="3">
+        <v>46195.700694444444</v>
+      </c>
+      <c r="D203">
+        <v>67</v>
+      </c>
+      <c r="E203">
+        <v>100</v>
+      </c>
+      <c r="F203" s="6">
+        <v>1.7118055555555556E-2</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A204">
+        <f t="shared" si="3"/>
+        <v>203</v>
+      </c>
+      <c r="B204">
+        <v>19</v>
+      </c>
+      <c r="C204" s="3">
+        <v>46195.724999999999</v>
+      </c>
+      <c r="D204">
+        <v>100</v>
+      </c>
+      <c r="E204">
+        <v>136</v>
+      </c>
+      <c r="F204" s="6">
+        <v>1.7881944444444443E-2</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A205">
+        <f t="shared" si="3"/>
+        <v>204</v>
+      </c>
+      <c r="B205">
+        <v>19</v>
+      </c>
+      <c r="C205" s="3">
+        <v>46195.796527777777</v>
+      </c>
+      <c r="D205">
+        <v>136</v>
+      </c>
+      <c r="E205">
+        <v>165</v>
+      </c>
+      <c r="F205" s="6">
+        <v>1.457175925925926E-2</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A206">
+        <f t="shared" si="3"/>
+        <v>205</v>
+      </c>
+      <c r="B206">
+        <v>19</v>
+      </c>
+      <c r="C206" s="3">
+        <v>46195.95208333333</v>
+      </c>
+      <c r="D206">
+        <v>165</v>
+      </c>
+      <c r="E206">
+        <v>215</v>
+      </c>
+      <c r="F206" s="6">
+        <v>2.6793981481481481E-2</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A207">
+        <f t="shared" si="3"/>
+        <v>206</v>
+      </c>
+      <c r="B207">
+        <v>19</v>
+      </c>
+      <c r="C207" s="3">
+        <v>46196.511805555558</v>
+      </c>
+      <c r="D207">
+        <v>215</v>
+      </c>
+      <c r="E207">
+        <v>260</v>
+      </c>
+      <c r="F207" s="6">
+        <v>1.9780092592592592E-2</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A208">
+        <f t="shared" si="3"/>
+        <v>207</v>
+      </c>
+      <c r="B208">
+        <v>19</v>
+      </c>
+      <c r="C208" s="3">
+        <v>46196.588888888888</v>
+      </c>
+      <c r="D208">
+        <v>260</v>
+      </c>
+      <c r="E208">
+        <v>291</v>
+      </c>
+      <c r="F208" s="6">
+        <v>1.4386574074074074E-2</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A209">
+        <f t="shared" si="3"/>
+        <v>208</v>
+      </c>
+      <c r="B209">
+        <v>19</v>
+      </c>
+      <c r="C209" s="3">
+        <v>46196.61041666667</v>
+      </c>
+      <c r="D209">
+        <v>291</v>
+      </c>
+      <c r="E209">
+        <v>312</v>
+      </c>
+      <c r="F209" s="6">
+        <v>1.0428240740740741E-2</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A210">
+        <f t="shared" si="3"/>
+        <v>209</v>
+      </c>
+      <c r="B210">
+        <v>19</v>
+      </c>
+      <c r="C210" s="3">
+        <v>46196.625694444447</v>
+      </c>
+      <c r="D210">
+        <v>312</v>
+      </c>
+      <c r="E210">
+        <v>359</v>
+      </c>
+      <c r="F210" s="6">
+        <v>2.2349537037037036E-2</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A211">
+        <f t="shared" si="3"/>
+        <v>210</v>
+      </c>
+      <c r="B211">
+        <v>19</v>
+      </c>
+      <c r="C211" s="3">
+        <v>46196.693749999999</v>
+      </c>
+      <c r="D211">
+        <v>359</v>
+      </c>
+      <c r="E211">
+        <v>397</v>
+      </c>
+      <c r="F211" s="6">
+        <v>2.1979166666666668E-2</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A212">
+        <f t="shared" si="3"/>
+        <v>211</v>
+      </c>
+      <c r="B212">
+        <v>19</v>
+      </c>
+      <c r="C212" s="3">
+        <v>46196.747916666667</v>
+      </c>
+      <c r="D212">
+        <v>397</v>
+      </c>
+      <c r="E212">
+        <v>426</v>
+      </c>
+      <c r="F212" s="6">
+        <v>1.3506944444444445E-2</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A213">
+        <f t="shared" si="3"/>
+        <v>212</v>
+      </c>
+      <c r="B213">
+        <v>19</v>
+      </c>
+      <c r="C213" s="3">
+        <v>46196.82916666667</v>
+      </c>
+      <c r="D213">
+        <v>426</v>
+      </c>
+      <c r="E213">
+        <v>461</v>
+      </c>
+      <c r="F213" s="6">
+        <v>1.9456018518518518E-2</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A214">
+        <f t="shared" si="3"/>
+        <v>213</v>
+      </c>
+      <c r="B214">
+        <v>19</v>
+      </c>
+      <c r="C214" s="3">
+        <v>46196.93472222222</v>
+      </c>
+      <c r="D214">
+        <v>461</v>
+      </c>
+      <c r="E214">
+        <v>483</v>
+      </c>
+      <c r="F214" s="6">
+        <v>1.1875E-2</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A215">
+        <f t="shared" si="3"/>
+        <v>214</v>
+      </c>
+      <c r="B215">
+        <v>19</v>
+      </c>
+      <c r="C215" s="3">
+        <v>46197.365277777775</v>
+      </c>
+      <c r="D215">
+        <v>483</v>
+      </c>
+      <c r="E215">
+        <v>515</v>
+      </c>
+      <c r="F215" s="6">
+        <v>1.4189814814814815E-2</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A216">
+        <f t="shared" si="3"/>
+        <v>215</v>
+      </c>
+      <c r="B216">
+        <v>19</v>
+      </c>
+      <c r="C216" s="3">
+        <v>46197.399305555555</v>
+      </c>
+      <c r="D216">
+        <v>515</v>
+      </c>
+      <c r="E216">
+        <v>540</v>
+      </c>
+      <c r="F216" s="6">
+        <v>1.2731481481481481E-2</v>
+      </c>
+    </row>
+    <row r="217" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A217">
+        <f t="shared" si="3"/>
+        <v>216</v>
+      </c>
+      <c r="B217">
+        <v>19</v>
+      </c>
+      <c r="C217" s="3">
+        <v>46197.433333333334</v>
+      </c>
+      <c r="D217">
+        <v>540</v>
+      </c>
+      <c r="E217">
+        <v>568</v>
+      </c>
+      <c r="F217" s="6">
+        <v>1.2685185185185185E-2</v>
+      </c>
+    </row>
+    <row r="218" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A218">
+        <f t="shared" si="3"/>
+        <v>217</v>
+      </c>
+      <c r="B218">
+        <v>19</v>
+      </c>
+      <c r="C218" s="3">
+        <v>46197.454861111109</v>
+      </c>
+      <c r="D218">
+        <v>568</v>
+      </c>
+      <c r="E218">
+        <v>644</v>
+      </c>
+      <c r="F218" s="6">
+        <v>3.5138888888888886E-2</v>
+      </c>
+    </row>
+    <row r="219" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A219">
+        <f t="shared" si="3"/>
+        <v>218</v>
+      </c>
+      <c r="B219">
+        <v>20</v>
+      </c>
+      <c r="C219" s="3">
+        <v>46197.527083333334</v>
+      </c>
+      <c r="D219" t="s">
+        <v>63</v>
+      </c>
+      <c r="E219" t="s">
+        <v>63</v>
+      </c>
+      <c r="F219" s="6">
+        <v>3.1365740740740743E-2</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A220">
+        <f t="shared" si="3"/>
+        <v>219</v>
+      </c>
+      <c r="B220">
+        <v>21</v>
+      </c>
+      <c r="C220" s="3">
+        <v>46198.461111111108</v>
+      </c>
+      <c r="D220">
+        <v>9</v>
+      </c>
+      <c r="E220">
+        <v>29</v>
+      </c>
+      <c r="F220" s="6">
+        <v>1.2858796296296297E-2</v>
+      </c>
+    </row>
+    <row r="221" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A221">
+        <f t="shared" si="3"/>
+        <v>220</v>
+      </c>
+      <c r="B221">
+        <v>21</v>
+      </c>
+      <c r="C221" s="3">
+        <v>46198.490277777775</v>
+      </c>
+      <c r="D221">
+        <v>29</v>
+      </c>
+      <c r="E221">
+        <v>45</v>
+      </c>
+      <c r="F221" s="6">
+        <v>1.2060185185185186E-2</v>
+      </c>
+    </row>
+    <row r="222" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A222">
+        <f t="shared" si="3"/>
+        <v>221</v>
+      </c>
+      <c r="B222">
+        <v>21</v>
+      </c>
+      <c r="C222" s="3">
+        <v>46198.554166666669</v>
+      </c>
+      <c r="D222">
+        <v>45</v>
+      </c>
+      <c r="E222">
+        <v>69</v>
+      </c>
+      <c r="F222" s="6">
+        <v>1.5601851851851851E-2</v>
+      </c>
+    </row>
+    <row r="223" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A223">
+        <f t="shared" si="3"/>
+        <v>222</v>
+      </c>
+      <c r="B223">
+        <v>21</v>
+      </c>
+      <c r="C223" s="3">
+        <v>46198.60833333333</v>
+      </c>
+      <c r="D223">
+        <v>69</v>
+      </c>
+      <c r="E223">
+        <v>97</v>
+      </c>
+      <c r="F223" s="6">
+        <v>1.5972222222222221E-2</v>
+      </c>
+    </row>
+    <row r="224" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A224">
+        <f t="shared" si="3"/>
+        <v>223</v>
+      </c>
+      <c r="B224">
+        <v>21</v>
+      </c>
+      <c r="C224" s="3">
+        <v>46198.910416666666</v>
+      </c>
+      <c r="D224">
+        <v>97</v>
+      </c>
+      <c r="E224">
+        <v>117</v>
+      </c>
+      <c r="F224" s="6">
+        <v>1.4826388888888889E-2</v>
+      </c>
+    </row>
+    <row r="225" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A225">
+        <f t="shared" si="3"/>
+        <v>224</v>
+      </c>
+      <c r="B225">
+        <v>21</v>
+      </c>
+      <c r="C225" s="3">
+        <v>46199.894444444442</v>
+      </c>
+      <c r="D225">
+        <v>117</v>
+      </c>
+      <c r="E225">
+        <v>131</v>
+      </c>
+      <c r="F225" s="6">
+        <v>1.0416666666666666E-2</v>
+      </c>
+    </row>
+    <row r="226" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A226">
+        <f t="shared" si="3"/>
+        <v>225</v>
+      </c>
+      <c r="B226">
+        <v>21</v>
+      </c>
+      <c r="C226" s="3">
+        <v>46199.929861111108</v>
+      </c>
+      <c r="D226">
+        <v>131</v>
+      </c>
+      <c r="E226">
+        <v>149</v>
+      </c>
+      <c r="F226" s="6">
+        <v>1.0787037037037038E-2</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A227">
+        <f t="shared" si="3"/>
+        <v>226</v>
+      </c>
+      <c r="B227">
+        <v>21</v>
+      </c>
+      <c r="C227" s="3">
+        <v>46200.443055555559</v>
+      </c>
+      <c r="D227">
+        <v>149</v>
+      </c>
+      <c r="E227">
+        <v>158</v>
+      </c>
+      <c r="F227" s="6">
+        <v>6.053240740740741E-3</v>
+      </c>
+    </row>
+    <row r="228" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A228">
+        <f t="shared" si="3"/>
+        <v>227</v>
+      </c>
+      <c r="B228">
+        <v>21</v>
+      </c>
+      <c r="C228" s="3">
+        <v>46200.911805555559</v>
+      </c>
+      <c r="D228">
+        <v>158</v>
+      </c>
+      <c r="E228">
+        <v>177</v>
+      </c>
+      <c r="F228" s="6">
+        <v>1.2210648148148148E-2</v>
+      </c>
+    </row>
+    <row r="229" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A229">
+        <f t="shared" si="3"/>
+        <v>228</v>
+      </c>
+      <c r="B229">
+        <v>21</v>
+      </c>
+      <c r="C229" s="3">
+        <v>46200.938888888886</v>
+      </c>
+      <c r="D229">
+        <v>177</v>
+      </c>
+      <c r="E229">
+        <v>201</v>
+      </c>
+      <c r="F229" s="6">
+        <v>1.699074074074074E-2</v>
+      </c>
+    </row>
+    <row r="230" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A230">
+        <f t="shared" si="3"/>
+        <v>229</v>
+      </c>
+      <c r="B230">
+        <v>21</v>
+      </c>
+      <c r="C230" s="3">
+        <v>46201.40625</v>
+      </c>
+      <c r="D230">
+        <v>201</v>
+      </c>
+      <c r="E230">
+        <v>235</v>
+      </c>
+      <c r="F230" s="6">
+        <v>1.8958333333333334E-2</v>
       </c>
     </row>
   </sheetData>
@@ -6012,12 +6787,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CC89663-E888-2445-AD16-77803353ADBB}">
-  <dimension ref="A1:E212"/>
+  <dimension ref="A1:E225"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.5" style="15" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
   </cols>
@@ -6032,7 +6807,7 @@
       <c r="C1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="14" t="s">
         <v>13</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -6050,7 +6825,7 @@
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="15" t="s">
         <v>37</v>
       </c>
       <c r="E2">
@@ -6068,7 +6843,7 @@
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="15" t="s">
         <v>18</v>
       </c>
       <c r="E3">
@@ -6086,7 +6861,7 @@
       <c r="C4">
         <v>3</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="15" t="s">
         <v>19</v>
       </c>
       <c r="E4">
@@ -6104,7 +6879,7 @@
       <c r="C5">
         <v>4</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="15" t="s">
         <v>20</v>
       </c>
       <c r="E5">
@@ -6122,7 +6897,7 @@
       <c r="C6">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="15" t="s">
         <v>21</v>
       </c>
       <c r="E6">
@@ -6140,7 +6915,7 @@
       <c r="C7">
         <v>6</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E7">
@@ -6158,7 +6933,7 @@
       <c r="C8">
         <v>7</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="15" t="s">
         <v>23</v>
       </c>
       <c r="E8">
@@ -6176,7 +6951,7 @@
       <c r="C9">
         <v>8</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="15" t="s">
         <v>24</v>
       </c>
       <c r="E9">
@@ -6194,7 +6969,7 @@
       <c r="C10">
         <v>9</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="15" t="s">
         <v>25</v>
       </c>
       <c r="E10">
@@ -6212,7 +6987,7 @@
       <c r="C11">
         <v>10</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E11">
@@ -6230,7 +7005,7 @@
       <c r="C12">
         <v>11</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="15" t="s">
         <v>27</v>
       </c>
       <c r="E12">
@@ -6248,7 +7023,7 @@
       <c r="C13">
         <v>12</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="15" t="s">
         <v>28</v>
       </c>
       <c r="E13">
@@ -6266,7 +7041,7 @@
       <c r="C14">
         <v>13</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="15" t="s">
         <v>29</v>
       </c>
       <c r="E14">
@@ -6284,7 +7059,7 @@
       <c r="C15">
         <v>14</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E15">
@@ -6302,7 +7077,7 @@
       <c r="C16">
         <v>15</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="15" t="s">
         <v>31</v>
       </c>
       <c r="E16">
@@ -6320,7 +7095,7 @@
       <c r="C17">
         <v>16</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="15" t="s">
         <v>32</v>
       </c>
       <c r="E17">
@@ -6338,7 +7113,7 @@
       <c r="C18">
         <v>17</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="15" t="s">
         <v>33</v>
       </c>
       <c r="E18">
@@ -6356,7 +7131,7 @@
       <c r="C19">
         <v>18</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="15" t="s">
         <v>34</v>
       </c>
       <c r="E19">
@@ -6374,7 +7149,7 @@
       <c r="C20">
         <v>19</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="15" t="s">
         <v>35</v>
       </c>
       <c r="E20">
@@ -6392,7 +7167,7 @@
       <c r="C21">
         <v>20</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="15" t="s">
         <v>36</v>
       </c>
       <c r="E21">
@@ -6410,7 +7185,7 @@
       <c r="C22">
         <v>1</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="15" t="s">
         <v>39</v>
       </c>
       <c r="E22">
@@ -6428,7 +7203,7 @@
       <c r="C23">
         <v>2</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="15" t="s">
         <v>40</v>
       </c>
       <c r="E23">
@@ -6446,7 +7221,7 @@
       <c r="C24">
         <v>3</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="15" t="s">
         <v>41</v>
       </c>
       <c r="E24">
@@ -6464,7 +7239,7 @@
       <c r="C25">
         <v>4</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="15" t="s">
         <v>42</v>
       </c>
       <c r="E25">
@@ -6482,7 +7257,7 @@
       <c r="C26">
         <v>5</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="15" t="s">
         <v>43</v>
       </c>
       <c r="E26">
@@ -6500,7 +7275,7 @@
       <c r="C27">
         <v>6</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="15" t="s">
         <v>44</v>
       </c>
       <c r="E27">
@@ -6518,7 +7293,7 @@
       <c r="C28">
         <v>7</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="15" t="s">
         <v>45</v>
       </c>
       <c r="E28">
@@ -6536,7 +7311,7 @@
       <c r="C29">
         <v>8</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="15" t="s">
         <v>46</v>
       </c>
       <c r="E29">
@@ -6554,7 +7329,7 @@
       <c r="C30">
         <v>9</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="15" t="s">
         <v>47</v>
       </c>
       <c r="E30">
@@ -6572,7 +7347,7 @@
       <c r="C31">
         <v>10</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="15" t="s">
         <v>48</v>
       </c>
       <c r="E31">
@@ -6590,7 +7365,7 @@
       <c r="C32">
         <v>11</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="15" t="s">
         <v>49</v>
       </c>
       <c r="E32">
@@ -6608,7 +7383,7 @@
       <c r="C33">
         <v>12</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="15" t="s">
         <v>50</v>
       </c>
       <c r="E33">
@@ -6626,7 +7401,7 @@
       <c r="C34">
         <v>13</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="15" t="s">
         <v>51</v>
       </c>
       <c r="E34">
@@ -6644,7 +7419,7 @@
       <c r="C35">
         <v>14</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="15" t="s">
         <v>52</v>
       </c>
       <c r="E35">
@@ -6662,7 +7437,7 @@
       <c r="C36">
         <v>15</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="15" t="s">
         <v>53</v>
       </c>
       <c r="E36">
@@ -6680,7 +7455,7 @@
       <c r="C37">
         <v>16</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="15" t="s">
         <v>54</v>
       </c>
       <c r="E37">
@@ -6698,7 +7473,7 @@
       <c r="C38">
         <v>17</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="15" t="s">
         <v>55</v>
       </c>
       <c r="E38">
@@ -6716,7 +7491,7 @@
       <c r="C39">
         <v>18</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="15" t="s">
         <v>56</v>
       </c>
       <c r="E39">
@@ -6734,7 +7509,7 @@
       <c r="C40">
         <v>19</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="15" t="s">
         <v>57</v>
       </c>
       <c r="E40">
@@ -6752,7 +7527,7 @@
       <c r="C41">
         <v>20</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" s="15" t="s">
         <v>58</v>
       </c>
       <c r="E41">
@@ -6770,7 +7545,7 @@
       <c r="C42">
         <v>21</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D42" s="15" t="s">
         <v>59</v>
       </c>
       <c r="E42">
@@ -6788,7 +7563,7 @@
       <c r="C43">
         <v>1</v>
       </c>
-      <c r="D43">
+      <c r="D43" s="15">
         <f>C43</f>
         <v>1</v>
       </c>
@@ -6807,7 +7582,7 @@
       <c r="C44">
         <v>2</v>
       </c>
-      <c r="D44">
+      <c r="D44" s="15">
         <f t="shared" ref="D44:D77" si="1">C44</f>
         <v>2</v>
       </c>
@@ -6826,7 +7601,7 @@
       <c r="C45">
         <v>3</v>
       </c>
-      <c r="D45">
+      <c r="D45" s="15">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -6845,7 +7620,7 @@
       <c r="C46">
         <v>4</v>
       </c>
-      <c r="D46">
+      <c r="D46" s="15">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
@@ -6864,7 +7639,7 @@
       <c r="C47">
         <v>5</v>
       </c>
-      <c r="D47">
+      <c r="D47" s="15">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
@@ -6883,7 +7658,7 @@
       <c r="C48">
         <v>6</v>
       </c>
-      <c r="D48">
+      <c r="D48" s="15">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
@@ -6902,7 +7677,7 @@
       <c r="C49">
         <v>7</v>
       </c>
-      <c r="D49">
+      <c r="D49" s="15">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -6921,7 +7696,7 @@
       <c r="C50">
         <v>8</v>
       </c>
-      <c r="D50">
+      <c r="D50" s="15">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -6940,7 +7715,7 @@
       <c r="C51">
         <v>9</v>
       </c>
-      <c r="D51">
+      <c r="D51" s="15">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
@@ -6959,7 +7734,7 @@
       <c r="C52">
         <v>10</v>
       </c>
-      <c r="D52">
+      <c r="D52" s="15">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
@@ -6978,7 +7753,7 @@
       <c r="C53">
         <v>11</v>
       </c>
-      <c r="D53">
+      <c r="D53" s="15">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
@@ -6997,7 +7772,7 @@
       <c r="C54">
         <v>12</v>
       </c>
-      <c r="D54">
+      <c r="D54" s="15">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
@@ -7016,7 +7791,7 @@
       <c r="C55">
         <v>13</v>
       </c>
-      <c r="D55">
+      <c r="D55" s="15">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
@@ -7035,7 +7810,7 @@
       <c r="C56">
         <v>14</v>
       </c>
-      <c r="D56">
+      <c r="D56" s="15">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
@@ -7054,7 +7829,7 @@
       <c r="C57">
         <v>15</v>
       </c>
-      <c r="D57">
+      <c r="D57" s="15">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
@@ -7073,7 +7848,7 @@
       <c r="C58">
         <v>16</v>
       </c>
-      <c r="D58">
+      <c r="D58" s="15">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
@@ -7092,7 +7867,7 @@
       <c r="C59">
         <v>17</v>
       </c>
-      <c r="D59">
+      <c r="D59" s="15">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
@@ -7111,7 +7886,7 @@
       <c r="C60">
         <v>18</v>
       </c>
-      <c r="D60">
+      <c r="D60" s="15">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
@@ -7130,7 +7905,7 @@
       <c r="C61">
         <v>19</v>
       </c>
-      <c r="D61">
+      <c r="D61" s="15">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
@@ -7149,7 +7924,7 @@
       <c r="C62">
         <v>20</v>
       </c>
-      <c r="D62">
+      <c r="D62" s="15">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
@@ -7168,7 +7943,7 @@
       <c r="C63">
         <v>21</v>
       </c>
-      <c r="D63">
+      <c r="D63" s="15">
         <f t="shared" si="1"/>
         <v>21</v>
       </c>
@@ -7187,7 +7962,7 @@
       <c r="C64">
         <v>22</v>
       </c>
-      <c r="D64">
+      <c r="D64" s="15">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
@@ -7206,7 +7981,7 @@
       <c r="C65">
         <v>23</v>
       </c>
-      <c r="D65">
+      <c r="D65" s="15">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
@@ -7225,7 +8000,7 @@
       <c r="C66">
         <v>24</v>
       </c>
-      <c r="D66">
+      <c r="D66" s="15">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
@@ -7244,7 +8019,7 @@
       <c r="C67">
         <v>25</v>
       </c>
-      <c r="D67">
+      <c r="D67" s="15">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
@@ -7263,7 +8038,7 @@
       <c r="C68">
         <v>1</v>
       </c>
-      <c r="D68">
+      <c r="D68" s="15">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
@@ -7282,7 +8057,7 @@
       <c r="C69">
         <v>2</v>
       </c>
-      <c r="D69">
+      <c r="D69" s="15">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
@@ -7301,7 +8076,7 @@
       <c r="C70">
         <v>3</v>
       </c>
-      <c r="D70">
+      <c r="D70" s="15">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -7320,7 +8095,7 @@
       <c r="C71">
         <v>4</v>
       </c>
-      <c r="D71">
+      <c r="D71" s="15">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
@@ -7339,7 +8114,7 @@
       <c r="C72">
         <v>5</v>
       </c>
-      <c r="D72">
+      <c r="D72" s="15">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
@@ -7358,7 +8133,7 @@
       <c r="C73">
         <v>6</v>
       </c>
-      <c r="D73">
+      <c r="D73" s="15">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
@@ -7377,7 +8152,7 @@
       <c r="C74">
         <v>7</v>
       </c>
-      <c r="D74">
+      <c r="D74" s="15">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -7396,7 +8171,7 @@
       <c r="C75">
         <v>8</v>
       </c>
-      <c r="D75">
+      <c r="D75" s="15">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -7415,7 +8190,7 @@
       <c r="C76">
         <v>9</v>
       </c>
-      <c r="D76">
+      <c r="D76" s="15">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
@@ -7434,7 +8209,7 @@
       <c r="C77">
         <v>10</v>
       </c>
-      <c r="D77">
+      <c r="D77" s="15">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
@@ -7453,7 +8228,7 @@
       <c r="C78">
         <v>11</v>
       </c>
-      <c r="D78" t="s">
+      <c r="D78" s="15" t="s">
         <v>84</v>
       </c>
       <c r="E78">
@@ -7471,7 +8246,7 @@
       <c r="C79">
         <v>1</v>
       </c>
-      <c r="D79" t="s">
+      <c r="D79" s="15" t="s">
         <v>88</v>
       </c>
       <c r="E79">
@@ -7489,7 +8264,7 @@
       <c r="C80">
         <v>2</v>
       </c>
-      <c r="D80" t="s">
+      <c r="D80" s="15" t="s">
         <v>89</v>
       </c>
       <c r="E80">
@@ -7508,7 +8283,7 @@
         <f>C80+1</f>
         <v>3</v>
       </c>
-      <c r="D81" t="s">
+      <c r="D81" s="15" t="s">
         <v>90</v>
       </c>
       <c r="E81">
@@ -7527,7 +8302,7 @@
         <f t="shared" ref="C82:C93" si="3">C81+1</f>
         <v>4</v>
       </c>
-      <c r="D82" t="s">
+      <c r="D82" s="15" t="s">
         <v>91</v>
       </c>
       <c r="E82">
@@ -7546,7 +8321,7 @@
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="D83" t="s">
+      <c r="D83" s="15" t="s">
         <v>92</v>
       </c>
       <c r="E83">
@@ -7565,7 +8340,7 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="D84" t="s">
+      <c r="D84" s="15" t="s">
         <v>93</v>
       </c>
       <c r="E84">
@@ -7584,7 +8359,7 @@
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
-      <c r="D85" t="s">
+      <c r="D85" s="15" t="s">
         <v>94</v>
       </c>
       <c r="E85">
@@ -7603,7 +8378,7 @@
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="D86" t="s">
+      <c r="D86" s="15" t="s">
         <v>95</v>
       </c>
       <c r="E86">
@@ -7622,7 +8397,7 @@
         <f t="shared" si="3"/>
         <v>9</v>
       </c>
-      <c r="D87" t="s">
+      <c r="D87" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E87">
@@ -7641,7 +8416,7 @@
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="D88" t="s">
+      <c r="D88" s="15" t="s">
         <v>97</v>
       </c>
       <c r="E88">
@@ -7660,7 +8435,7 @@
         <f t="shared" si="3"/>
         <v>11</v>
       </c>
-      <c r="D89" t="s">
+      <c r="D89" s="15" t="s">
         <v>98</v>
       </c>
       <c r="E89">
@@ -7679,7 +8454,7 @@
         <f t="shared" si="3"/>
         <v>12</v>
       </c>
-      <c r="D90" t="s">
+      <c r="D90" s="15" t="s">
         <v>99</v>
       </c>
       <c r="E90">
@@ -7698,7 +8473,7 @@
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="D91" t="s">
+      <c r="D91" s="15" t="s">
         <v>100</v>
       </c>
       <c r="E91">
@@ -7717,7 +8492,7 @@
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="D92" t="s">
+      <c r="D92" s="15" t="s">
         <v>101</v>
       </c>
       <c r="E92">
@@ -7736,7 +8511,7 @@
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="D93" t="s">
+      <c r="D93" s="15" t="s">
         <v>102</v>
       </c>
       <c r="E93">
@@ -7754,7 +8529,7 @@
       <c r="C94">
         <v>1</v>
       </c>
-      <c r="D94">
+      <c r="D94" s="15">
         <f>C94</f>
         <v>1</v>
       </c>
@@ -7773,7 +8548,7 @@
       <c r="C95">
         <v>2</v>
       </c>
-      <c r="D95">
+      <c r="D95" s="15">
         <f t="shared" ref="D95:D112" si="4">C95</f>
         <v>2</v>
       </c>
@@ -7793,7 +8568,7 @@
         <f>C95+1</f>
         <v>3</v>
       </c>
-      <c r="D96">
+      <c r="D96" s="15">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
@@ -7813,7 +8588,7 @@
         <f t="shared" ref="C97:C112" si="5">C96+1</f>
         <v>4</v>
       </c>
-      <c r="D97">
+      <c r="D97" s="15">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
@@ -7833,7 +8608,7 @@
         <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="D98">
+      <c r="D98" s="15">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
@@ -7853,7 +8628,7 @@
         <f t="shared" si="5"/>
         <v>6</v>
       </c>
-      <c r="D99">
+      <c r="D99" s="15">
         <f t="shared" si="4"/>
         <v>6</v>
       </c>
@@ -7873,7 +8648,7 @@
         <f t="shared" si="5"/>
         <v>7</v>
       </c>
-      <c r="D100">
+      <c r="D100" s="15">
         <f t="shared" si="4"/>
         <v>7</v>
       </c>
@@ -7893,7 +8668,7 @@
         <f t="shared" si="5"/>
         <v>8</v>
       </c>
-      <c r="D101">
+      <c r="D101" s="15">
         <f t="shared" si="4"/>
         <v>8</v>
       </c>
@@ -7913,7 +8688,7 @@
         <f t="shared" si="5"/>
         <v>9</v>
       </c>
-      <c r="D102">
+      <c r="D102" s="15">
         <f t="shared" si="4"/>
         <v>9</v>
       </c>
@@ -7933,7 +8708,7 @@
         <f t="shared" si="5"/>
         <v>10</v>
       </c>
-      <c r="D103">
+      <c r="D103" s="15">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
@@ -7953,7 +8728,7 @@
         <f>C103+1</f>
         <v>11</v>
       </c>
-      <c r="D104">
+      <c r="D104" s="15">
         <f t="shared" si="4"/>
         <v>11</v>
       </c>
@@ -7973,7 +8748,7 @@
         <f t="shared" si="5"/>
         <v>12</v>
       </c>
-      <c r="D105">
+      <c r="D105" s="15">
         <f t="shared" si="4"/>
         <v>12</v>
       </c>
@@ -7993,7 +8768,7 @@
         <f t="shared" si="5"/>
         <v>13</v>
       </c>
-      <c r="D106">
+      <c r="D106" s="15">
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
@@ -8013,7 +8788,7 @@
         <f t="shared" si="5"/>
         <v>14</v>
       </c>
-      <c r="D107">
+      <c r="D107" s="15">
         <f t="shared" si="4"/>
         <v>14</v>
       </c>
@@ -8033,7 +8808,7 @@
         <f t="shared" si="5"/>
         <v>15</v>
       </c>
-      <c r="D108">
+      <c r="D108" s="15">
         <f t="shared" si="4"/>
         <v>15</v>
       </c>
@@ -8053,7 +8828,7 @@
         <f t="shared" si="5"/>
         <v>16</v>
       </c>
-      <c r="D109">
+      <c r="D109" s="15">
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
@@ -8073,7 +8848,7 @@
         <f>C109+1</f>
         <v>17</v>
       </c>
-      <c r="D110">
+      <c r="D110" s="15">
         <f t="shared" si="4"/>
         <v>17</v>
       </c>
@@ -8093,7 +8868,7 @@
         <f t="shared" si="5"/>
         <v>18</v>
       </c>
-      <c r="D111">
+      <c r="D111" s="15">
         <f t="shared" si="4"/>
         <v>18</v>
       </c>
@@ -8113,7 +8888,7 @@
         <f t="shared" si="5"/>
         <v>19</v>
       </c>
-      <c r="D112">
+      <c r="D112" s="15">
         <f t="shared" si="4"/>
         <v>19</v>
       </c>
@@ -8132,7 +8907,7 @@
       <c r="C113">
         <v>1</v>
       </c>
-      <c r="D113" t="s">
+      <c r="D113" s="15" t="s">
         <v>109</v>
       </c>
       <c r="E113">
@@ -8151,7 +8926,7 @@
         <f>C113+1</f>
         <v>2</v>
       </c>
-      <c r="D114" t="s">
+      <c r="D114" s="15" t="s">
         <v>110</v>
       </c>
       <c r="E114">
@@ -8170,7 +8945,7 @@
         <f t="shared" ref="C115:C131" si="6">C114+1</f>
         <v>3</v>
       </c>
-      <c r="D115" t="s">
+      <c r="D115" s="15" t="s">
         <v>29</v>
       </c>
       <c r="E115">
@@ -8189,7 +8964,7 @@
         <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="D116" t="s">
+      <c r="D116" s="15" t="s">
         <v>111</v>
       </c>
       <c r="E116">
@@ -8208,7 +8983,7 @@
         <f t="shared" si="6"/>
         <v>5</v>
       </c>
-      <c r="D117" t="s">
+      <c r="D117" s="15" t="s">
         <v>112</v>
       </c>
       <c r="E117">
@@ -8227,7 +9002,7 @@
         <f t="shared" si="6"/>
         <v>6</v>
       </c>
-      <c r="D118" t="s">
+      <c r="D118" s="15" t="s">
         <v>113</v>
       </c>
       <c r="E118">
@@ -8246,7 +9021,7 @@
         <f t="shared" si="6"/>
         <v>7</v>
       </c>
-      <c r="D119" t="s">
+      <c r="D119" s="15" t="s">
         <v>114</v>
       </c>
       <c r="E119">
@@ -8265,7 +9040,7 @@
         <f t="shared" si="6"/>
         <v>8</v>
       </c>
-      <c r="D120" t="s">
+      <c r="D120" s="15" t="s">
         <v>115</v>
       </c>
       <c r="E120">
@@ -8284,7 +9059,7 @@
         <f t="shared" si="6"/>
         <v>9</v>
       </c>
-      <c r="D121" t="s">
+      <c r="D121" s="15" t="s">
         <v>116</v>
       </c>
       <c r="E121">
@@ -8303,7 +9078,7 @@
         <f t="shared" si="6"/>
         <v>10</v>
       </c>
-      <c r="D122" t="s">
+      <c r="D122" s="15" t="s">
         <v>117</v>
       </c>
       <c r="E122">
@@ -8322,7 +9097,7 @@
         <f t="shared" si="6"/>
         <v>11</v>
       </c>
-      <c r="D123" t="s">
+      <c r="D123" s="15" t="s">
         <v>118</v>
       </c>
       <c r="E123">
@@ -8341,7 +9116,7 @@
         <f t="shared" si="6"/>
         <v>12</v>
       </c>
-      <c r="D124" t="s">
+      <c r="D124" s="15" t="s">
         <v>119</v>
       </c>
       <c r="E124">
@@ -8360,7 +9135,7 @@
         <f t="shared" si="6"/>
         <v>13</v>
       </c>
-      <c r="D125" t="s">
+      <c r="D125" s="15" t="s">
         <v>120</v>
       </c>
       <c r="E125">
@@ -8379,7 +9154,7 @@
         <f t="shared" si="6"/>
         <v>14</v>
       </c>
-      <c r="D126" t="s">
+      <c r="D126" s="15" t="s">
         <v>126</v>
       </c>
       <c r="E126">
@@ -8398,7 +9173,7 @@
         <f t="shared" si="6"/>
         <v>15</v>
       </c>
-      <c r="D127" t="s">
+      <c r="D127" s="15" t="s">
         <v>121</v>
       </c>
       <c r="E127">
@@ -8417,7 +9192,7 @@
         <f t="shared" si="6"/>
         <v>16</v>
       </c>
-      <c r="D128" t="s">
+      <c r="D128" s="15" t="s">
         <v>122</v>
       </c>
       <c r="E128">
@@ -8436,7 +9211,7 @@
         <f t="shared" si="6"/>
         <v>17</v>
       </c>
-      <c r="D129" t="s">
+      <c r="D129" s="15" t="s">
         <v>123</v>
       </c>
       <c r="E129">
@@ -8455,7 +9230,7 @@
         <f t="shared" si="6"/>
         <v>18</v>
       </c>
-      <c r="D130" t="s">
+      <c r="D130" s="15" t="s">
         <v>124</v>
       </c>
       <c r="E130">
@@ -8474,7 +9249,7 @@
         <f t="shared" si="6"/>
         <v>19</v>
       </c>
-      <c r="D131" t="s">
+      <c r="D131" s="15" t="s">
         <v>125</v>
       </c>
       <c r="E131">
@@ -8492,7 +9267,7 @@
       <c r="C132">
         <v>1</v>
       </c>
-      <c r="D132" t="s">
+      <c r="D132" s="15" t="s">
         <v>131</v>
       </c>
       <c r="E132">
@@ -8510,7 +9285,7 @@
       <c r="C133">
         <v>2</v>
       </c>
-      <c r="D133" t="s">
+      <c r="D133" s="15" t="s">
         <v>132</v>
       </c>
       <c r="E133">
@@ -8528,7 +9303,7 @@
       <c r="C134">
         <v>3</v>
       </c>
-      <c r="D134" t="s">
+      <c r="D134" s="15" t="s">
         <v>133</v>
       </c>
       <c r="E134">
@@ -8546,7 +9321,7 @@
       <c r="C135">
         <v>4</v>
       </c>
-      <c r="D135" t="s">
+      <c r="D135" s="15" t="s">
         <v>134</v>
       </c>
       <c r="E135">
@@ -8564,7 +9339,7 @@
       <c r="C136">
         <v>5</v>
       </c>
-      <c r="D136" t="s">
+      <c r="D136" s="15" t="s">
         <v>135</v>
       </c>
       <c r="E136">
@@ -8582,7 +9357,7 @@
       <c r="C137">
         <v>1</v>
       </c>
-      <c r="D137">
+      <c r="D137" s="15">
         <f>C137</f>
         <v>1</v>
       </c>
@@ -8602,7 +9377,7 @@
         <f>C137+1</f>
         <v>2</v>
       </c>
-      <c r="D138">
+      <c r="D138" s="15">
         <f t="shared" ref="D138:D159" si="8">C138</f>
         <v>2</v>
       </c>
@@ -8622,7 +9397,7 @@
         <f t="shared" ref="C139:C159" si="9">C138+1</f>
         <v>3</v>
       </c>
-      <c r="D139">
+      <c r="D139" s="15">
         <f t="shared" si="8"/>
         <v>3</v>
       </c>
@@ -8642,7 +9417,7 @@
         <f t="shared" si="9"/>
         <v>4</v>
       </c>
-      <c r="D140">
+      <c r="D140" s="15">
         <f t="shared" si="8"/>
         <v>4</v>
       </c>
@@ -8662,7 +9437,7 @@
         <f t="shared" si="9"/>
         <v>5</v>
       </c>
-      <c r="D141">
+      <c r="D141" s="15">
         <f t="shared" si="8"/>
         <v>5</v>
       </c>
@@ -8682,7 +9457,7 @@
         <f t="shared" si="9"/>
         <v>6</v>
       </c>
-      <c r="D142">
+      <c r="D142" s="15">
         <f t="shared" si="8"/>
         <v>6</v>
       </c>
@@ -8702,7 +9477,7 @@
         <f t="shared" si="9"/>
         <v>7</v>
       </c>
-      <c r="D143">
+      <c r="D143" s="15">
         <f t="shared" si="8"/>
         <v>7</v>
       </c>
@@ -8722,7 +9497,7 @@
         <f t="shared" si="9"/>
         <v>8</v>
       </c>
-      <c r="D144">
+      <c r="D144" s="15">
         <f t="shared" si="8"/>
         <v>8</v>
       </c>
@@ -8742,7 +9517,7 @@
         <f t="shared" si="9"/>
         <v>9</v>
       </c>
-      <c r="D145">
+      <c r="D145" s="15">
         <f t="shared" si="8"/>
         <v>9</v>
       </c>
@@ -8762,7 +9537,7 @@
         <f t="shared" si="9"/>
         <v>10</v>
       </c>
-      <c r="D146">
+      <c r="D146" s="15">
         <f t="shared" si="8"/>
         <v>10</v>
       </c>
@@ -8782,7 +9557,7 @@
         <f t="shared" si="9"/>
         <v>11</v>
       </c>
-      <c r="D147">
+      <c r="D147" s="15">
         <f t="shared" si="8"/>
         <v>11</v>
       </c>
@@ -8802,7 +9577,7 @@
         <f t="shared" si="9"/>
         <v>12</v>
       </c>
-      <c r="D148">
+      <c r="D148" s="15">
         <f t="shared" si="8"/>
         <v>12</v>
       </c>
@@ -8822,7 +9597,7 @@
         <f t="shared" si="9"/>
         <v>13</v>
       </c>
-      <c r="D149">
+      <c r="D149" s="15">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
@@ -8842,7 +9617,7 @@
         <f t="shared" si="9"/>
         <v>14</v>
       </c>
-      <c r="D150">
+      <c r="D150" s="15">
         <f t="shared" si="8"/>
         <v>14</v>
       </c>
@@ -8862,7 +9637,7 @@
         <f t="shared" si="9"/>
         <v>15</v>
       </c>
-      <c r="D151">
+      <c r="D151" s="15">
         <f t="shared" si="8"/>
         <v>15</v>
       </c>
@@ -8882,7 +9657,7 @@
         <f t="shared" si="9"/>
         <v>16</v>
       </c>
-      <c r="D152">
+      <c r="D152" s="15">
         <f t="shared" si="8"/>
         <v>16</v>
       </c>
@@ -8902,7 +9677,7 @@
         <f t="shared" si="9"/>
         <v>17</v>
       </c>
-      <c r="D153">
+      <c r="D153" s="15">
         <f t="shared" si="8"/>
         <v>17</v>
       </c>
@@ -8922,7 +9697,7 @@
         <f t="shared" si="9"/>
         <v>18</v>
       </c>
-      <c r="D154">
+      <c r="D154" s="15">
         <f t="shared" si="8"/>
         <v>18</v>
       </c>
@@ -8942,7 +9717,7 @@
         <f t="shared" si="9"/>
         <v>19</v>
       </c>
-      <c r="D155">
+      <c r="D155" s="15">
         <f t="shared" si="8"/>
         <v>19</v>
       </c>
@@ -8962,7 +9737,7 @@
         <f t="shared" si="9"/>
         <v>20</v>
       </c>
-      <c r="D156">
+      <c r="D156" s="15">
         <f t="shared" si="8"/>
         <v>20</v>
       </c>
@@ -8982,7 +9757,7 @@
         <f t="shared" si="9"/>
         <v>21</v>
       </c>
-      <c r="D157">
+      <c r="D157" s="15">
         <f t="shared" si="8"/>
         <v>21</v>
       </c>
@@ -9002,7 +9777,7 @@
         <f t="shared" si="9"/>
         <v>22</v>
       </c>
-      <c r="D158">
+      <c r="D158" s="15">
         <f t="shared" si="8"/>
         <v>22</v>
       </c>
@@ -9022,7 +9797,7 @@
         <f t="shared" si="9"/>
         <v>23</v>
       </c>
-      <c r="D159">
+      <c r="D159" s="15">
         <f t="shared" si="8"/>
         <v>23</v>
       </c>
@@ -9041,7 +9816,7 @@
       <c r="C160">
         <v>24</v>
       </c>
-      <c r="D160" t="s">
+      <c r="D160" s="15" t="s">
         <v>135</v>
       </c>
       <c r="E160">
@@ -9059,7 +9834,7 @@
       <c r="C161">
         <v>1</v>
       </c>
-      <c r="D161" t="s">
+      <c r="D161" s="15" t="s">
         <v>148</v>
       </c>
       <c r="E161">
@@ -9077,7 +9852,7 @@
       <c r="C162">
         <v>2</v>
       </c>
-      <c r="D162" t="s">
+      <c r="D162" s="15" t="s">
         <v>149</v>
       </c>
       <c r="E162">
@@ -9095,7 +9870,7 @@
       <c r="C163">
         <v>3</v>
       </c>
-      <c r="D163" t="s">
+      <c r="D163" s="15" t="s">
         <v>150</v>
       </c>
       <c r="E163">
@@ -9113,7 +9888,7 @@
       <c r="C164">
         <v>4</v>
       </c>
-      <c r="D164" t="s">
+      <c r="D164" s="15" t="s">
         <v>151</v>
       </c>
       <c r="E164">
@@ -9131,7 +9906,7 @@
       <c r="C165">
         <v>5</v>
       </c>
-      <c r="D165" t="s">
+      <c r="D165" s="15" t="s">
         <v>152</v>
       </c>
       <c r="E165">
@@ -9149,7 +9924,7 @@
       <c r="C166">
         <v>6</v>
       </c>
-      <c r="D166" t="s">
+      <c r="D166" s="15" t="s">
         <v>153</v>
       </c>
       <c r="E166">
@@ -9167,7 +9942,7 @@
       <c r="C167">
         <v>7</v>
       </c>
-      <c r="D167" t="s">
+      <c r="D167" s="15" t="s">
         <v>154</v>
       </c>
       <c r="E167">
@@ -9185,7 +9960,7 @@
       <c r="C168">
         <v>1</v>
       </c>
-      <c r="D168" t="s">
+      <c r="D168" s="15" t="s">
         <v>157</v>
       </c>
       <c r="E168">
@@ -9204,7 +9979,7 @@
         <f>C168+1</f>
         <v>2</v>
       </c>
-      <c r="D169" t="s">
+      <c r="D169" s="15" t="s">
         <v>158</v>
       </c>
       <c r="E169">
@@ -9223,7 +9998,7 @@
         <f t="shared" ref="C170:C212" si="10">C169+1</f>
         <v>3</v>
       </c>
-      <c r="D170" t="s">
+      <c r="D170" s="15" t="s">
         <v>159</v>
       </c>
       <c r="E170">
@@ -9242,7 +10017,7 @@
         <f t="shared" si="10"/>
         <v>4</v>
       </c>
-      <c r="D171" t="s">
+      <c r="D171" s="15" t="s">
         <v>160</v>
       </c>
       <c r="E171">
@@ -9261,7 +10036,7 @@
         <f t="shared" si="10"/>
         <v>5</v>
       </c>
-      <c r="D172" t="s">
+      <c r="D172" s="15" t="s">
         <v>161</v>
       </c>
       <c r="E172">
@@ -9280,7 +10055,7 @@
         <f t="shared" si="10"/>
         <v>6</v>
       </c>
-      <c r="D173" t="s">
+      <c r="D173" s="15" t="s">
         <v>162</v>
       </c>
       <c r="E173">
@@ -9299,7 +10074,7 @@
         <f t="shared" si="10"/>
         <v>7</v>
       </c>
-      <c r="D174" t="s">
+      <c r="D174" s="15" t="s">
         <v>163</v>
       </c>
       <c r="E174">
@@ -9318,7 +10093,7 @@
         <f t="shared" si="10"/>
         <v>8</v>
       </c>
-      <c r="D175" t="s">
+      <c r="D175" s="15" t="s">
         <v>164</v>
       </c>
       <c r="E175">
@@ -9337,7 +10112,7 @@
         <f t="shared" si="10"/>
         <v>9</v>
       </c>
-      <c r="D176" t="s">
+      <c r="D176" s="15" t="s">
         <v>165</v>
       </c>
       <c r="E176">
@@ -9356,7 +10131,7 @@
         <f t="shared" si="10"/>
         <v>10</v>
       </c>
-      <c r="D177" t="s">
+      <c r="D177" s="15" t="s">
         <v>166</v>
       </c>
       <c r="E177">
@@ -9375,7 +10150,7 @@
         <f t="shared" si="10"/>
         <v>11</v>
       </c>
-      <c r="D178" t="s">
+      <c r="D178" s="15" t="s">
         <v>167</v>
       </c>
       <c r="E178">
@@ -9394,7 +10169,7 @@
         <f t="shared" si="10"/>
         <v>12</v>
       </c>
-      <c r="D179" t="s">
+      <c r="D179" s="15" t="s">
         <v>168</v>
       </c>
       <c r="E179">
@@ -9413,7 +10188,7 @@
         <f t="shared" si="10"/>
         <v>13</v>
       </c>
-      <c r="D180" t="s">
+      <c r="D180" s="15" t="s">
         <v>169</v>
       </c>
       <c r="E180">
@@ -9432,7 +10207,7 @@
         <f t="shared" si="10"/>
         <v>14</v>
       </c>
-      <c r="D181" t="s">
+      <c r="D181" s="15" t="s">
         <v>170</v>
       </c>
       <c r="E181">
@@ -9451,7 +10226,7 @@
         <f t="shared" si="10"/>
         <v>15</v>
       </c>
-      <c r="D182" t="s">
+      <c r="D182" s="15" t="s">
         <v>171</v>
       </c>
       <c r="E182">
@@ -9470,7 +10245,7 @@
         <f t="shared" si="10"/>
         <v>16</v>
       </c>
-      <c r="D183" t="s">
+      <c r="D183" s="15" t="s">
         <v>172</v>
       </c>
       <c r="E183">
@@ -9489,7 +10264,7 @@
         <f t="shared" si="10"/>
         <v>17</v>
       </c>
-      <c r="D184" t="s">
+      <c r="D184" s="15" t="s">
         <v>173</v>
       </c>
       <c r="E184">
@@ -9508,7 +10283,7 @@
         <f t="shared" si="10"/>
         <v>18</v>
       </c>
-      <c r="D185" t="s">
+      <c r="D185" s="15" t="s">
         <v>174</v>
       </c>
       <c r="E185">
@@ -9527,7 +10302,7 @@
         <f t="shared" si="10"/>
         <v>19</v>
       </c>
-      <c r="D186" t="s">
+      <c r="D186" s="15" t="s">
         <v>175</v>
       </c>
       <c r="E186">
@@ -9546,7 +10321,7 @@
         <f t="shared" si="10"/>
         <v>20</v>
       </c>
-      <c r="D187" t="s">
+      <c r="D187" s="15" t="s">
         <v>176</v>
       </c>
       <c r="E187">
@@ -9565,7 +10340,7 @@
         <f t="shared" si="10"/>
         <v>21</v>
       </c>
-      <c r="D188" t="s">
+      <c r="D188" s="15" t="s">
         <v>178</v>
       </c>
       <c r="E188">
@@ -9584,7 +10359,7 @@
         <f t="shared" si="10"/>
         <v>22</v>
       </c>
-      <c r="D189" t="s">
+      <c r="D189" s="15" t="s">
         <v>177</v>
       </c>
       <c r="E189">
@@ -9603,7 +10378,7 @@
         <f t="shared" si="10"/>
         <v>23</v>
       </c>
-      <c r="D190" t="s">
+      <c r="D190" s="15" t="s">
         <v>179</v>
       </c>
       <c r="E190">
@@ -9622,7 +10397,7 @@
         <f t="shared" si="10"/>
         <v>24</v>
       </c>
-      <c r="D191" t="s">
+      <c r="D191" s="15" t="s">
         <v>180</v>
       </c>
       <c r="E191">
@@ -9641,7 +10416,7 @@
         <f t="shared" si="10"/>
         <v>25</v>
       </c>
-      <c r="D192" t="s">
+      <c r="D192" s="15" t="s">
         <v>181</v>
       </c>
       <c r="E192">
@@ -9660,7 +10435,7 @@
         <f t="shared" si="10"/>
         <v>26</v>
       </c>
-      <c r="D193" t="s">
+      <c r="D193" s="15" t="s">
         <v>182</v>
       </c>
       <c r="E193">
@@ -9679,7 +10454,7 @@
         <f t="shared" si="10"/>
         <v>27</v>
       </c>
-      <c r="D194" t="s">
+      <c r="D194" s="15" t="s">
         <v>183</v>
       </c>
       <c r="E194">
@@ -9688,7 +10463,7 @@
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A195">
-        <f t="shared" ref="A195:A212" si="11" xml:space="preserve"> ROW() -1</f>
+        <f t="shared" ref="A195:A225" si="11" xml:space="preserve"> ROW() -1</f>
         <v>194</v>
       </c>
       <c r="B195">
@@ -9698,7 +10473,7 @@
         <f t="shared" si="10"/>
         <v>28</v>
       </c>
-      <c r="D195" t="s">
+      <c r="D195" s="15" t="s">
         <v>184</v>
       </c>
       <c r="E195">
@@ -9717,7 +10492,7 @@
         <f t="shared" si="10"/>
         <v>29</v>
       </c>
-      <c r="D196" t="s">
+      <c r="D196" s="15" t="s">
         <v>185</v>
       </c>
       <c r="E196">
@@ -9736,7 +10511,7 @@
         <f t="shared" si="10"/>
         <v>30</v>
       </c>
-      <c r="D197" t="s">
+      <c r="D197" s="15" t="s">
         <v>186</v>
       </c>
       <c r="E197">
@@ -9755,7 +10530,7 @@
         <f t="shared" si="10"/>
         <v>31</v>
       </c>
-      <c r="D198" t="s">
+      <c r="D198" s="15" t="s">
         <v>187</v>
       </c>
       <c r="E198">
@@ -9774,7 +10549,7 @@
         <f t="shared" si="10"/>
         <v>32</v>
       </c>
-      <c r="D199" t="s">
+      <c r="D199" s="15" t="s">
         <v>188</v>
       </c>
       <c r="E199">
@@ -9793,7 +10568,7 @@
         <f t="shared" si="10"/>
         <v>33</v>
       </c>
-      <c r="D200" t="s">
+      <c r="D200" s="15" t="s">
         <v>189</v>
       </c>
       <c r="E200">
@@ -9812,7 +10587,7 @@
         <f t="shared" si="10"/>
         <v>34</v>
       </c>
-      <c r="D201" t="s">
+      <c r="D201" s="15" t="s">
         <v>190</v>
       </c>
       <c r="E201">
@@ -9831,7 +10606,7 @@
         <f t="shared" si="10"/>
         <v>35</v>
       </c>
-      <c r="D202" t="s">
+      <c r="D202" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E202">
@@ -9850,7 +10625,7 @@
         <f t="shared" si="10"/>
         <v>36</v>
       </c>
-      <c r="D203" t="s">
+      <c r="D203" s="15" t="s">
         <v>192</v>
       </c>
       <c r="E203">
@@ -9869,7 +10644,7 @@
         <f t="shared" si="10"/>
         <v>37</v>
       </c>
-      <c r="D204" t="s">
+      <c r="D204" s="15" t="s">
         <v>193</v>
       </c>
       <c r="E204">
@@ -9888,7 +10663,7 @@
         <f t="shared" si="10"/>
         <v>38</v>
       </c>
-      <c r="D205" t="s">
+      <c r="D205" s="15" t="s">
         <v>194</v>
       </c>
       <c r="E205">
@@ -9907,7 +10682,7 @@
         <f t="shared" si="10"/>
         <v>39</v>
       </c>
-      <c r="D206" t="s">
+      <c r="D206" s="15" t="s">
         <v>195</v>
       </c>
       <c r="E206">
@@ -9926,7 +10701,7 @@
         <f t="shared" si="10"/>
         <v>40</v>
       </c>
-      <c r="D207" t="s">
+      <c r="D207" s="15" t="s">
         <v>196</v>
       </c>
       <c r="E207">
@@ -9945,7 +10720,7 @@
         <f t="shared" si="10"/>
         <v>41</v>
       </c>
-      <c r="D208" t="s">
+      <c r="D208" s="15" t="s">
         <v>197</v>
       </c>
       <c r="E208">
@@ -9964,7 +10739,7 @@
         <f t="shared" si="10"/>
         <v>42</v>
       </c>
-      <c r="D209" t="s">
+      <c r="D209" s="15" t="s">
         <v>198</v>
       </c>
       <c r="E209">
@@ -9983,7 +10758,7 @@
         <f t="shared" si="10"/>
         <v>43</v>
       </c>
-      <c r="D210" t="s">
+      <c r="D210" s="15" t="s">
         <v>199</v>
       </c>
       <c r="E210">
@@ -10002,7 +10777,7 @@
         <f t="shared" si="10"/>
         <v>44</v>
       </c>
-      <c r="D211" t="s">
+      <c r="D211" s="15" t="s">
         <v>201</v>
       </c>
       <c r="E211">
@@ -10021,11 +10796,257 @@
         <f t="shared" si="10"/>
         <v>45</v>
       </c>
-      <c r="D212" t="s">
+      <c r="D212" s="15" t="s">
         <v>200</v>
       </c>
       <c r="E212">
         <v>387</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A213">
+        <f t="shared" si="11"/>
+        <v>212</v>
+      </c>
+      <c r="B213">
+        <v>21</v>
+      </c>
+      <c r="C213">
+        <v>1</v>
+      </c>
+      <c r="D213" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="E213">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A214">
+        <f t="shared" si="11"/>
+        <v>213</v>
+      </c>
+      <c r="B214">
+        <v>21</v>
+      </c>
+      <c r="C214">
+        <f>C213+1</f>
+        <v>2</v>
+      </c>
+      <c r="D214" s="15">
+        <v>1</v>
+      </c>
+      <c r="E214">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A215">
+        <f t="shared" si="11"/>
+        <v>214</v>
+      </c>
+      <c r="B215">
+        <v>21</v>
+      </c>
+      <c r="C215">
+        <f t="shared" ref="C215:C225" si="12">C214+1</f>
+        <v>3</v>
+      </c>
+      <c r="D215" s="15">
+        <v>2</v>
+      </c>
+      <c r="E215">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A216">
+        <f t="shared" si="11"/>
+        <v>215</v>
+      </c>
+      <c r="B216">
+        <v>21</v>
+      </c>
+      <c r="C216">
+        <f t="shared" si="12"/>
+        <v>4</v>
+      </c>
+      <c r="D216" s="15">
+        <v>3</v>
+      </c>
+      <c r="E216">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A217">
+        <f t="shared" si="11"/>
+        <v>216</v>
+      </c>
+      <c r="B217">
+        <v>21</v>
+      </c>
+      <c r="C217">
+        <f t="shared" si="12"/>
+        <v>5</v>
+      </c>
+      <c r="D217" s="15">
+        <v>4</v>
+      </c>
+      <c r="E217">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A218">
+        <f t="shared" si="11"/>
+        <v>217</v>
+      </c>
+      <c r="B218">
+        <v>21</v>
+      </c>
+      <c r="C218">
+        <f t="shared" si="12"/>
+        <v>6</v>
+      </c>
+      <c r="D218" s="15">
+        <v>5</v>
+      </c>
+      <c r="E218">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A219">
+        <f t="shared" si="11"/>
+        <v>218</v>
+      </c>
+      <c r="B219">
+        <v>21</v>
+      </c>
+      <c r="C219">
+        <f t="shared" si="12"/>
+        <v>7</v>
+      </c>
+      <c r="D219" s="15">
+        <v>6</v>
+      </c>
+      <c r="E219">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A220">
+        <f t="shared" si="11"/>
+        <v>219</v>
+      </c>
+      <c r="B220">
+        <v>21</v>
+      </c>
+      <c r="C220">
+        <f t="shared" si="12"/>
+        <v>8</v>
+      </c>
+      <c r="D220" s="15">
+        <v>7</v>
+      </c>
+      <c r="E220">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A221">
+        <f t="shared" si="11"/>
+        <v>220</v>
+      </c>
+      <c r="B221">
+        <v>21</v>
+      </c>
+      <c r="C221">
+        <f t="shared" si="12"/>
+        <v>9</v>
+      </c>
+      <c r="D221" s="15">
+        <v>8</v>
+      </c>
+      <c r="E221">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A222">
+        <f t="shared" si="11"/>
+        <v>221</v>
+      </c>
+      <c r="B222">
+        <v>21</v>
+      </c>
+      <c r="C222">
+        <f t="shared" si="12"/>
+        <v>10</v>
+      </c>
+      <c r="D222" s="15">
+        <v>9</v>
+      </c>
+      <c r="E222">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A223">
+        <f t="shared" si="11"/>
+        <v>222</v>
+      </c>
+      <c r="B223">
+        <v>21</v>
+      </c>
+      <c r="C223">
+        <f t="shared" si="12"/>
+        <v>11</v>
+      </c>
+      <c r="D223" s="15">
+        <v>10</v>
+      </c>
+      <c r="E223">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A224">
+        <f t="shared" si="11"/>
+        <v>223</v>
+      </c>
+      <c r="B224">
+        <v>21</v>
+      </c>
+      <c r="C224">
+        <f t="shared" si="12"/>
+        <v>12</v>
+      </c>
+      <c r="D224" s="15">
+        <v>11</v>
+      </c>
+      <c r="E224">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A225">
+        <f t="shared" si="11"/>
+        <v>224</v>
+      </c>
+      <c r="B225">
+        <v>21</v>
+      </c>
+      <c r="C225">
+        <f t="shared" si="12"/>
+        <v>13</v>
+      </c>
+      <c r="D225" s="15">
+        <v>12</v>
+      </c>
+      <c r="E225">
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data (Old Possum's Cats)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/code/projects/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F7900B-2BF9-6147-AC01-E1A6CE576E48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA45DFBE-0CA6-7345-9B2B-FD4ACB210FB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="15040" windowHeight="18980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="38400" windowHeight="20980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="210">
   <si>
     <t>book_id</t>
   </si>
@@ -661,7 +661,10 @@
     <t>Prologue</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t>Old Possum's Book of Practical Cats</t>
+  </si>
+  <si>
+    <t>T.S. Eliot</t>
   </si>
 </sst>
 </file>
@@ -716,7 +719,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -729,8 +732,6 @@
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -1076,7 +1077,6 @@
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" style="13"/>
     <col min="8" max="8" width="10.6640625" style="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.1640625" bestFit="1" customWidth="1"/>
@@ -1103,7 +1103,7 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="1" t="s">
         <v>64</v>
       </c>
       <c r="H1" s="10" t="s">
@@ -1142,7 +1142,7 @@
       <c r="F2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="13">
+      <c r="G2">
         <v>136</v>
       </c>
       <c r="H2" s="11">
@@ -1181,7 +1181,7 @@
       <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="13">
+      <c r="G3">
         <v>160</v>
       </c>
       <c r="H3" s="11">
@@ -1220,7 +1220,7 @@
       <c r="F4" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="13">
+      <c r="G4">
         <v>487</v>
       </c>
       <c r="H4" s="11">
@@ -1259,7 +1259,7 @@
       <c r="F5" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="13">
+      <c r="G5">
         <v>449</v>
       </c>
       <c r="H5" s="11">
@@ -1298,7 +1298,7 @@
       <c r="F6" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="13">
+      <c r="G6">
         <v>499</v>
       </c>
       <c r="H6" s="11">
@@ -1337,7 +1337,7 @@
       <c r="F7" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="13">
+      <c r="G7">
         <v>210</v>
       </c>
       <c r="H7" s="11">
@@ -1375,7 +1375,7 @@
       <c r="F8" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8">
         <v>266</v>
       </c>
       <c r="H8" s="11" t="s">
@@ -1413,7 +1413,7 @@
       <c r="F9" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="13">
+      <c r="G9">
         <v>261</v>
       </c>
       <c r="H9" s="11">
@@ -1451,7 +1451,7 @@
       <c r="F10" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="13">
+      <c r="G10">
         <v>310</v>
       </c>
       <c r="H10" s="11">
@@ -1489,7 +1489,7 @@
       <c r="F11" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11">
         <v>244</v>
       </c>
       <c r="H11" s="11">
@@ -1527,7 +1527,7 @@
       <c r="F12" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="13">
+      <c r="G12">
         <v>490</v>
       </c>
       <c r="H12" s="11">
@@ -1565,7 +1565,7 @@
       <c r="F13" t="s">
         <v>16</v>
       </c>
-      <c r="G13" s="13">
+      <c r="G13">
         <v>432</v>
       </c>
       <c r="H13" s="11">
@@ -1603,7 +1603,7 @@
       <c r="F14" t="s">
         <v>130</v>
       </c>
-      <c r="G14" s="13">
+      <c r="G14">
         <v>309</v>
       </c>
       <c r="H14" s="11">
@@ -1641,7 +1641,7 @@
       <c r="F15" t="s">
         <v>16</v>
       </c>
-      <c r="G15" s="13">
+      <c r="G15">
         <v>348</v>
       </c>
       <c r="H15" s="11">
@@ -1679,7 +1679,7 @@
       <c r="F16" t="s">
         <v>130</v>
       </c>
-      <c r="G16" s="13">
+      <c r="G16">
         <v>527</v>
       </c>
       <c r="H16" s="11">
@@ -1717,7 +1717,7 @@
       <c r="F17" t="s">
         <v>16</v>
       </c>
-      <c r="G17" s="13">
+      <c r="G17">
         <v>106</v>
       </c>
       <c r="H17" s="11">
@@ -1755,7 +1755,7 @@
       <c r="F18" t="s">
         <v>16</v>
       </c>
-      <c r="G18" s="13">
+      <c r="G18">
         <v>309</v>
       </c>
       <c r="H18" s="11">
@@ -1793,7 +1793,7 @@
       <c r="F19" t="s">
         <v>16</v>
       </c>
-      <c r="G19" s="13">
+      <c r="G19">
         <v>379</v>
       </c>
       <c r="H19" s="11">
@@ -1831,7 +1831,7 @@
       <c r="F20" t="s">
         <v>203</v>
       </c>
-      <c r="G20" s="13">
+      <c r="G20">
         <v>644</v>
       </c>
       <c r="H20" s="11">
@@ -1869,7 +1869,7 @@
       <c r="F21" t="s">
         <v>16</v>
       </c>
-      <c r="G21" s="13">
+      <c r="G21">
         <v>114</v>
       </c>
       <c r="H21" s="11">
@@ -1907,7 +1907,7 @@
       <c r="F22" t="s">
         <v>16</v>
       </c>
-      <c r="G22" s="13">
+      <c r="G22">
         <v>226</v>
       </c>
       <c r="H22" s="11">
@@ -1927,8 +1927,41 @@
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>208</v>
+      </c>
+      <c r="C23" t="s">
+        <v>209</v>
+      </c>
+      <c r="D23" t="s">
+        <v>144</v>
+      </c>
+      <c r="E23">
+        <v>1939</v>
+      </c>
+      <c r="F23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G23">
+        <v>56</v>
+      </c>
+      <c r="H23" s="11">
+        <v>5899</v>
+      </c>
       <c r="I23" t="s">
-        <v>208</v>
+        <v>104</v>
+      </c>
+      <c r="J23" t="s">
+        <v>81</v>
+      </c>
+      <c r="K23" s="7">
+        <v>46204</v>
+      </c>
+      <c r="L23" s="7">
+        <v>46204</v>
       </c>
     </row>
   </sheetData>
@@ -1938,7 +1971,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I230"/>
+  <dimension ref="A1:I231"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -6026,7 +6059,7 @@
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A195">
-        <f t="shared" ref="A195:A230" si="3">ROW() - 1</f>
+        <f t="shared" ref="A195:A231" si="3">ROW() - 1</f>
         <v>194</v>
       </c>
       <c r="B195">
@@ -6778,6 +6811,27 @@
       </c>
       <c r="F230" s="6">
         <v>1.8958333333333334E-2</v>
+      </c>
+    </row>
+    <row r="231" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A231">
+        <f t="shared" si="3"/>
+        <v>230</v>
+      </c>
+      <c r="B231">
+        <v>22</v>
+      </c>
+      <c r="C231" s="3">
+        <v>46204.552777777775</v>
+      </c>
+      <c r="D231">
+        <v>1</v>
+      </c>
+      <c r="E231">
+        <v>56</v>
+      </c>
+      <c r="F231" s="6">
+        <v>1.7372685185185185E-2</v>
       </c>
     </row>
   </sheetData>
@@ -6792,7 +6846,7 @@
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.5" style="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.5" style="13" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
   </cols>
@@ -6807,7 +6861,7 @@
       <c r="C1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -6825,7 +6879,7 @@
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="13" t="s">
         <v>37</v>
       </c>
       <c r="E2">
@@ -6843,7 +6897,7 @@
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="13" t="s">
         <v>18</v>
       </c>
       <c r="E3">
@@ -6861,7 +6915,7 @@
       <c r="C4">
         <v>3</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="13" t="s">
         <v>19</v>
       </c>
       <c r="E4">
@@ -6879,7 +6933,7 @@
       <c r="C5">
         <v>4</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="13" t="s">
         <v>20</v>
       </c>
       <c r="E5">
@@ -6897,7 +6951,7 @@
       <c r="C6">
         <v>5</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="13" t="s">
         <v>21</v>
       </c>
       <c r="E6">
@@ -6915,7 +6969,7 @@
       <c r="C7">
         <v>6</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="13" t="s">
         <v>22</v>
       </c>
       <c r="E7">
@@ -6933,7 +6987,7 @@
       <c r="C8">
         <v>7</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="13" t="s">
         <v>23</v>
       </c>
       <c r="E8">
@@ -6951,7 +7005,7 @@
       <c r="C9">
         <v>8</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="13" t="s">
         <v>24</v>
       </c>
       <c r="E9">
@@ -6969,7 +7023,7 @@
       <c r="C10">
         <v>9</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="13" t="s">
         <v>25</v>
       </c>
       <c r="E10">
@@ -6987,7 +7041,7 @@
       <c r="C11">
         <v>10</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="13" t="s">
         <v>26</v>
       </c>
       <c r="E11">
@@ -7005,7 +7059,7 @@
       <c r="C12">
         <v>11</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="13" t="s">
         <v>27</v>
       </c>
       <c r="E12">
@@ -7023,7 +7077,7 @@
       <c r="C13">
         <v>12</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="13" t="s">
         <v>28</v>
       </c>
       <c r="E13">
@@ -7041,7 +7095,7 @@
       <c r="C14">
         <v>13</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="13" t="s">
         <v>29</v>
       </c>
       <c r="E14">
@@ -7059,7 +7113,7 @@
       <c r="C15">
         <v>14</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="13" t="s">
         <v>30</v>
       </c>
       <c r="E15">
@@ -7077,7 +7131,7 @@
       <c r="C16">
         <v>15</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="13" t="s">
         <v>31</v>
       </c>
       <c r="E16">
@@ -7095,7 +7149,7 @@
       <c r="C17">
         <v>16</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="13" t="s">
         <v>32</v>
       </c>
       <c r="E17">
@@ -7113,7 +7167,7 @@
       <c r="C18">
         <v>17</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="13" t="s">
         <v>33</v>
       </c>
       <c r="E18">
@@ -7131,7 +7185,7 @@
       <c r="C19">
         <v>18</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="D19" s="13" t="s">
         <v>34</v>
       </c>
       <c r="E19">
@@ -7149,7 +7203,7 @@
       <c r="C20">
         <v>19</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E20">
@@ -7167,7 +7221,7 @@
       <c r="C21">
         <v>20</v>
       </c>
-      <c r="D21" s="15" t="s">
+      <c r="D21" s="13" t="s">
         <v>36</v>
       </c>
       <c r="E21">
@@ -7185,7 +7239,7 @@
       <c r="C22">
         <v>1</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="13" t="s">
         <v>39</v>
       </c>
       <c r="E22">
@@ -7203,7 +7257,7 @@
       <c r="C23">
         <v>2</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="13" t="s">
         <v>40</v>
       </c>
       <c r="E23">
@@ -7221,7 +7275,7 @@
       <c r="C24">
         <v>3</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="D24" s="13" t="s">
         <v>41</v>
       </c>
       <c r="E24">
@@ -7239,7 +7293,7 @@
       <c r="C25">
         <v>4</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="13" t="s">
         <v>42</v>
       </c>
       <c r="E25">
@@ -7257,7 +7311,7 @@
       <c r="C26">
         <v>5</v>
       </c>
-      <c r="D26" s="15" t="s">
+      <c r="D26" s="13" t="s">
         <v>43</v>
       </c>
       <c r="E26">
@@ -7275,7 +7329,7 @@
       <c r="C27">
         <v>6</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="13" t="s">
         <v>44</v>
       </c>
       <c r="E27">
@@ -7293,7 +7347,7 @@
       <c r="C28">
         <v>7</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="13" t="s">
         <v>45</v>
       </c>
       <c r="E28">
@@ -7311,7 +7365,7 @@
       <c r="C29">
         <v>8</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="13" t="s">
         <v>46</v>
       </c>
       <c r="E29">
@@ -7329,7 +7383,7 @@
       <c r="C30">
         <v>9</v>
       </c>
-      <c r="D30" s="15" t="s">
+      <c r="D30" s="13" t="s">
         <v>47</v>
       </c>
       <c r="E30">
@@ -7347,7 +7401,7 @@
       <c r="C31">
         <v>10</v>
       </c>
-      <c r="D31" s="15" t="s">
+      <c r="D31" s="13" t="s">
         <v>48</v>
       </c>
       <c r="E31">
@@ -7365,7 +7419,7 @@
       <c r="C32">
         <v>11</v>
       </c>
-      <c r="D32" s="15" t="s">
+      <c r="D32" s="13" t="s">
         <v>49</v>
       </c>
       <c r="E32">
@@ -7383,7 +7437,7 @@
       <c r="C33">
         <v>12</v>
       </c>
-      <c r="D33" s="15" t="s">
+      <c r="D33" s="13" t="s">
         <v>50</v>
       </c>
       <c r="E33">
@@ -7401,7 +7455,7 @@
       <c r="C34">
         <v>13</v>
       </c>
-      <c r="D34" s="15" t="s">
+      <c r="D34" s="13" t="s">
         <v>51</v>
       </c>
       <c r="E34">
@@ -7419,7 +7473,7 @@
       <c r="C35">
         <v>14</v>
       </c>
-      <c r="D35" s="15" t="s">
+      <c r="D35" s="13" t="s">
         <v>52</v>
       </c>
       <c r="E35">
@@ -7437,7 +7491,7 @@
       <c r="C36">
         <v>15</v>
       </c>
-      <c r="D36" s="15" t="s">
+      <c r="D36" s="13" t="s">
         <v>53</v>
       </c>
       <c r="E36">
@@ -7455,7 +7509,7 @@
       <c r="C37">
         <v>16</v>
       </c>
-      <c r="D37" s="15" t="s">
+      <c r="D37" s="13" t="s">
         <v>54</v>
       </c>
       <c r="E37">
@@ -7473,7 +7527,7 @@
       <c r="C38">
         <v>17</v>
       </c>
-      <c r="D38" s="15" t="s">
+      <c r="D38" s="13" t="s">
         <v>55</v>
       </c>
       <c r="E38">
@@ -7491,7 +7545,7 @@
       <c r="C39">
         <v>18</v>
       </c>
-      <c r="D39" s="15" t="s">
+      <c r="D39" s="13" t="s">
         <v>56</v>
       </c>
       <c r="E39">
@@ -7509,7 +7563,7 @@
       <c r="C40">
         <v>19</v>
       </c>
-      <c r="D40" s="15" t="s">
+      <c r="D40" s="13" t="s">
         <v>57</v>
       </c>
       <c r="E40">
@@ -7527,7 +7581,7 @@
       <c r="C41">
         <v>20</v>
       </c>
-      <c r="D41" s="15" t="s">
+      <c r="D41" s="13" t="s">
         <v>58</v>
       </c>
       <c r="E41">
@@ -7545,7 +7599,7 @@
       <c r="C42">
         <v>21</v>
       </c>
-      <c r="D42" s="15" t="s">
+      <c r="D42" s="13" t="s">
         <v>59</v>
       </c>
       <c r="E42">
@@ -7563,7 +7617,7 @@
       <c r="C43">
         <v>1</v>
       </c>
-      <c r="D43" s="15">
+      <c r="D43" s="13">
         <f>C43</f>
         <v>1</v>
       </c>
@@ -7582,7 +7636,7 @@
       <c r="C44">
         <v>2</v>
       </c>
-      <c r="D44" s="15">
+      <c r="D44" s="13">
         <f t="shared" ref="D44:D77" si="1">C44</f>
         <v>2</v>
       </c>
@@ -7601,7 +7655,7 @@
       <c r="C45">
         <v>3</v>
       </c>
-      <c r="D45" s="15">
+      <c r="D45" s="13">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -7620,7 +7674,7 @@
       <c r="C46">
         <v>4</v>
       </c>
-      <c r="D46" s="15">
+      <c r="D46" s="13">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
@@ -7639,7 +7693,7 @@
       <c r="C47">
         <v>5</v>
       </c>
-      <c r="D47" s="15">
+      <c r="D47" s="13">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
@@ -7658,7 +7712,7 @@
       <c r="C48">
         <v>6</v>
       </c>
-      <c r="D48" s="15">
+      <c r="D48" s="13">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
@@ -7677,7 +7731,7 @@
       <c r="C49">
         <v>7</v>
       </c>
-      <c r="D49" s="15">
+      <c r="D49" s="13">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -7696,7 +7750,7 @@
       <c r="C50">
         <v>8</v>
       </c>
-      <c r="D50" s="15">
+      <c r="D50" s="13">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -7715,7 +7769,7 @@
       <c r="C51">
         <v>9</v>
       </c>
-      <c r="D51" s="15">
+      <c r="D51" s="13">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
@@ -7734,7 +7788,7 @@
       <c r="C52">
         <v>10</v>
       </c>
-      <c r="D52" s="15">
+      <c r="D52" s="13">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
@@ -7753,7 +7807,7 @@
       <c r="C53">
         <v>11</v>
       </c>
-      <c r="D53" s="15">
+      <c r="D53" s="13">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
@@ -7772,7 +7826,7 @@
       <c r="C54">
         <v>12</v>
       </c>
-      <c r="D54" s="15">
+      <c r="D54" s="13">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
@@ -7791,7 +7845,7 @@
       <c r="C55">
         <v>13</v>
       </c>
-      <c r="D55" s="15">
+      <c r="D55" s="13">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
@@ -7810,7 +7864,7 @@
       <c r="C56">
         <v>14</v>
       </c>
-      <c r="D56" s="15">
+      <c r="D56" s="13">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
@@ -7829,7 +7883,7 @@
       <c r="C57">
         <v>15</v>
       </c>
-      <c r="D57" s="15">
+      <c r="D57" s="13">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
@@ -7848,7 +7902,7 @@
       <c r="C58">
         <v>16</v>
       </c>
-      <c r="D58" s="15">
+      <c r="D58" s="13">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
@@ -7867,7 +7921,7 @@
       <c r="C59">
         <v>17</v>
       </c>
-      <c r="D59" s="15">
+      <c r="D59" s="13">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
@@ -7886,7 +7940,7 @@
       <c r="C60">
         <v>18</v>
       </c>
-      <c r="D60" s="15">
+      <c r="D60" s="13">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
@@ -7905,7 +7959,7 @@
       <c r="C61">
         <v>19</v>
       </c>
-      <c r="D61" s="15">
+      <c r="D61" s="13">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
@@ -7924,7 +7978,7 @@
       <c r="C62">
         <v>20</v>
       </c>
-      <c r="D62" s="15">
+      <c r="D62" s="13">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
@@ -7943,7 +7997,7 @@
       <c r="C63">
         <v>21</v>
       </c>
-      <c r="D63" s="15">
+      <c r="D63" s="13">
         <f t="shared" si="1"/>
         <v>21</v>
       </c>
@@ -7962,7 +8016,7 @@
       <c r="C64">
         <v>22</v>
       </c>
-      <c r="D64" s="15">
+      <c r="D64" s="13">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
@@ -7981,7 +8035,7 @@
       <c r="C65">
         <v>23</v>
       </c>
-      <c r="D65" s="15">
+      <c r="D65" s="13">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
@@ -8000,7 +8054,7 @@
       <c r="C66">
         <v>24</v>
       </c>
-      <c r="D66" s="15">
+      <c r="D66" s="13">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
@@ -8019,7 +8073,7 @@
       <c r="C67">
         <v>25</v>
       </c>
-      <c r="D67" s="15">
+      <c r="D67" s="13">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
@@ -8038,7 +8092,7 @@
       <c r="C68">
         <v>1</v>
       </c>
-      <c r="D68" s="15">
+      <c r="D68" s="13">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
@@ -8057,7 +8111,7 @@
       <c r="C69">
         <v>2</v>
       </c>
-      <c r="D69" s="15">
+      <c r="D69" s="13">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
@@ -8076,7 +8130,7 @@
       <c r="C70">
         <v>3</v>
       </c>
-      <c r="D70" s="15">
+      <c r="D70" s="13">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -8095,7 +8149,7 @@
       <c r="C71">
         <v>4</v>
       </c>
-      <c r="D71" s="15">
+      <c r="D71" s="13">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
@@ -8114,7 +8168,7 @@
       <c r="C72">
         <v>5</v>
       </c>
-      <c r="D72" s="15">
+      <c r="D72" s="13">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
@@ -8133,7 +8187,7 @@
       <c r="C73">
         <v>6</v>
       </c>
-      <c r="D73" s="15">
+      <c r="D73" s="13">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
@@ -8152,7 +8206,7 @@
       <c r="C74">
         <v>7</v>
       </c>
-      <c r="D74" s="15">
+      <c r="D74" s="13">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -8171,7 +8225,7 @@
       <c r="C75">
         <v>8</v>
       </c>
-      <c r="D75" s="15">
+      <c r="D75" s="13">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -8190,7 +8244,7 @@
       <c r="C76">
         <v>9</v>
       </c>
-      <c r="D76" s="15">
+      <c r="D76" s="13">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
@@ -8209,7 +8263,7 @@
       <c r="C77">
         <v>10</v>
       </c>
-      <c r="D77" s="15">
+      <c r="D77" s="13">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
@@ -8228,7 +8282,7 @@
       <c r="C78">
         <v>11</v>
       </c>
-      <c r="D78" s="15" t="s">
+      <c r="D78" s="13" t="s">
         <v>84</v>
       </c>
       <c r="E78">
@@ -8246,7 +8300,7 @@
       <c r="C79">
         <v>1</v>
       </c>
-      <c r="D79" s="15" t="s">
+      <c r="D79" s="13" t="s">
         <v>88</v>
       </c>
       <c r="E79">
@@ -8264,7 +8318,7 @@
       <c r="C80">
         <v>2</v>
       </c>
-      <c r="D80" s="15" t="s">
+      <c r="D80" s="13" t="s">
         <v>89</v>
       </c>
       <c r="E80">
@@ -8283,7 +8337,7 @@
         <f>C80+1</f>
         <v>3</v>
       </c>
-      <c r="D81" s="15" t="s">
+      <c r="D81" s="13" t="s">
         <v>90</v>
       </c>
       <c r="E81">
@@ -8302,7 +8356,7 @@
         <f t="shared" ref="C82:C93" si="3">C81+1</f>
         <v>4</v>
       </c>
-      <c r="D82" s="15" t="s">
+      <c r="D82" s="13" t="s">
         <v>91</v>
       </c>
       <c r="E82">
@@ -8321,7 +8375,7 @@
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="D83" s="15" t="s">
+      <c r="D83" s="13" t="s">
         <v>92</v>
       </c>
       <c r="E83">
@@ -8340,7 +8394,7 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="D84" s="15" t="s">
+      <c r="D84" s="13" t="s">
         <v>93</v>
       </c>
       <c r="E84">
@@ -8359,7 +8413,7 @@
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
-      <c r="D85" s="15" t="s">
+      <c r="D85" s="13" t="s">
         <v>94</v>
       </c>
       <c r="E85">
@@ -8378,7 +8432,7 @@
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="D86" s="15" t="s">
+      <c r="D86" s="13" t="s">
         <v>95</v>
       </c>
       <c r="E86">
@@ -8397,7 +8451,7 @@
         <f t="shared" si="3"/>
         <v>9</v>
       </c>
-      <c r="D87" s="15" t="s">
+      <c r="D87" s="13" t="s">
         <v>96</v>
       </c>
       <c r="E87">
@@ -8416,7 +8470,7 @@
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="D88" s="15" t="s">
+      <c r="D88" s="13" t="s">
         <v>97</v>
       </c>
       <c r="E88">
@@ -8435,7 +8489,7 @@
         <f t="shared" si="3"/>
         <v>11</v>
       </c>
-      <c r="D89" s="15" t="s">
+      <c r="D89" s="13" t="s">
         <v>98</v>
       </c>
       <c r="E89">
@@ -8454,7 +8508,7 @@
         <f t="shared" si="3"/>
         <v>12</v>
       </c>
-      <c r="D90" s="15" t="s">
+      <c r="D90" s="13" t="s">
         <v>99</v>
       </c>
       <c r="E90">
@@ -8473,7 +8527,7 @@
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="D91" s="15" t="s">
+      <c r="D91" s="13" t="s">
         <v>100</v>
       </c>
       <c r="E91">
@@ -8492,7 +8546,7 @@
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="D92" s="15" t="s">
+      <c r="D92" s="13" t="s">
         <v>101</v>
       </c>
       <c r="E92">
@@ -8511,7 +8565,7 @@
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="D93" s="15" t="s">
+      <c r="D93" s="13" t="s">
         <v>102</v>
       </c>
       <c r="E93">
@@ -8529,7 +8583,7 @@
       <c r="C94">
         <v>1</v>
       </c>
-      <c r="D94" s="15">
+      <c r="D94" s="13">
         <f>C94</f>
         <v>1</v>
       </c>
@@ -8548,7 +8602,7 @@
       <c r="C95">
         <v>2</v>
       </c>
-      <c r="D95" s="15">
+      <c r="D95" s="13">
         <f t="shared" ref="D95:D112" si="4">C95</f>
         <v>2</v>
       </c>
@@ -8568,7 +8622,7 @@
         <f>C95+1</f>
         <v>3</v>
       </c>
-      <c r="D96" s="15">
+      <c r="D96" s="13">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
@@ -8588,7 +8642,7 @@
         <f t="shared" ref="C97:C112" si="5">C96+1</f>
         <v>4</v>
       </c>
-      <c r="D97" s="15">
+      <c r="D97" s="13">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
@@ -8608,7 +8662,7 @@
         <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="D98" s="15">
+      <c r="D98" s="13">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
@@ -8628,7 +8682,7 @@
         <f t="shared" si="5"/>
         <v>6</v>
       </c>
-      <c r="D99" s="15">
+      <c r="D99" s="13">
         <f t="shared" si="4"/>
         <v>6</v>
       </c>
@@ -8648,7 +8702,7 @@
         <f t="shared" si="5"/>
         <v>7</v>
       </c>
-      <c r="D100" s="15">
+      <c r="D100" s="13">
         <f t="shared" si="4"/>
         <v>7</v>
       </c>
@@ -8668,7 +8722,7 @@
         <f t="shared" si="5"/>
         <v>8</v>
       </c>
-      <c r="D101" s="15">
+      <c r="D101" s="13">
         <f t="shared" si="4"/>
         <v>8</v>
       </c>
@@ -8688,7 +8742,7 @@
         <f t="shared" si="5"/>
         <v>9</v>
       </c>
-      <c r="D102" s="15">
+      <c r="D102" s="13">
         <f t="shared" si="4"/>
         <v>9</v>
       </c>
@@ -8708,7 +8762,7 @@
         <f t="shared" si="5"/>
         <v>10</v>
       </c>
-      <c r="D103" s="15">
+      <c r="D103" s="13">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
@@ -8728,7 +8782,7 @@
         <f>C103+1</f>
         <v>11</v>
       </c>
-      <c r="D104" s="15">
+      <c r="D104" s="13">
         <f t="shared" si="4"/>
         <v>11</v>
       </c>
@@ -8748,7 +8802,7 @@
         <f t="shared" si="5"/>
         <v>12</v>
       </c>
-      <c r="D105" s="15">
+      <c r="D105" s="13">
         <f t="shared" si="4"/>
         <v>12</v>
       </c>
@@ -8768,7 +8822,7 @@
         <f t="shared" si="5"/>
         <v>13</v>
       </c>
-      <c r="D106" s="15">
+      <c r="D106" s="13">
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
@@ -8788,7 +8842,7 @@
         <f t="shared" si="5"/>
         <v>14</v>
       </c>
-      <c r="D107" s="15">
+      <c r="D107" s="13">
         <f t="shared" si="4"/>
         <v>14</v>
       </c>
@@ -8808,7 +8862,7 @@
         <f t="shared" si="5"/>
         <v>15</v>
       </c>
-      <c r="D108" s="15">
+      <c r="D108" s="13">
         <f t="shared" si="4"/>
         <v>15</v>
       </c>
@@ -8828,7 +8882,7 @@
         <f t="shared" si="5"/>
         <v>16</v>
       </c>
-      <c r="D109" s="15">
+      <c r="D109" s="13">
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
@@ -8848,7 +8902,7 @@
         <f>C109+1</f>
         <v>17</v>
       </c>
-      <c r="D110" s="15">
+      <c r="D110" s="13">
         <f t="shared" si="4"/>
         <v>17</v>
       </c>
@@ -8868,7 +8922,7 @@
         <f t="shared" si="5"/>
         <v>18</v>
       </c>
-      <c r="D111" s="15">
+      <c r="D111" s="13">
         <f t="shared" si="4"/>
         <v>18</v>
       </c>
@@ -8888,7 +8942,7 @@
         <f t="shared" si="5"/>
         <v>19</v>
       </c>
-      <c r="D112" s="15">
+      <c r="D112" s="13">
         <f t="shared" si="4"/>
         <v>19</v>
       </c>
@@ -8907,7 +8961,7 @@
       <c r="C113">
         <v>1</v>
       </c>
-      <c r="D113" s="15" t="s">
+      <c r="D113" s="13" t="s">
         <v>109</v>
       </c>
       <c r="E113">
@@ -8926,7 +8980,7 @@
         <f>C113+1</f>
         <v>2</v>
       </c>
-      <c r="D114" s="15" t="s">
+      <c r="D114" s="13" t="s">
         <v>110</v>
       </c>
       <c r="E114">
@@ -8945,7 +8999,7 @@
         <f t="shared" ref="C115:C131" si="6">C114+1</f>
         <v>3</v>
       </c>
-      <c r="D115" s="15" t="s">
+      <c r="D115" s="13" t="s">
         <v>29</v>
       </c>
       <c r="E115">
@@ -8964,7 +9018,7 @@
         <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="D116" s="15" t="s">
+      <c r="D116" s="13" t="s">
         <v>111</v>
       </c>
       <c r="E116">
@@ -8983,7 +9037,7 @@
         <f t="shared" si="6"/>
         <v>5</v>
       </c>
-      <c r="D117" s="15" t="s">
+      <c r="D117" s="13" t="s">
         <v>112</v>
       </c>
       <c r="E117">
@@ -9002,7 +9056,7 @@
         <f t="shared" si="6"/>
         <v>6</v>
       </c>
-      <c r="D118" s="15" t="s">
+      <c r="D118" s="13" t="s">
         <v>113</v>
       </c>
       <c r="E118">
@@ -9021,7 +9075,7 @@
         <f t="shared" si="6"/>
         <v>7</v>
       </c>
-      <c r="D119" s="15" t="s">
+      <c r="D119" s="13" t="s">
         <v>114</v>
       </c>
       <c r="E119">
@@ -9040,7 +9094,7 @@
         <f t="shared" si="6"/>
         <v>8</v>
       </c>
-      <c r="D120" s="15" t="s">
+      <c r="D120" s="13" t="s">
         <v>115</v>
       </c>
       <c r="E120">
@@ -9059,7 +9113,7 @@
         <f t="shared" si="6"/>
         <v>9</v>
       </c>
-      <c r="D121" s="15" t="s">
+      <c r="D121" s="13" t="s">
         <v>116</v>
       </c>
       <c r="E121">
@@ -9078,7 +9132,7 @@
         <f t="shared" si="6"/>
         <v>10</v>
       </c>
-      <c r="D122" s="15" t="s">
+      <c r="D122" s="13" t="s">
         <v>117</v>
       </c>
       <c r="E122">
@@ -9097,7 +9151,7 @@
         <f t="shared" si="6"/>
         <v>11</v>
       </c>
-      <c r="D123" s="15" t="s">
+      <c r="D123" s="13" t="s">
         <v>118</v>
       </c>
       <c r="E123">
@@ -9116,7 +9170,7 @@
         <f t="shared" si="6"/>
         <v>12</v>
       </c>
-      <c r="D124" s="15" t="s">
+      <c r="D124" s="13" t="s">
         <v>119</v>
       </c>
       <c r="E124">
@@ -9135,7 +9189,7 @@
         <f t="shared" si="6"/>
         <v>13</v>
       </c>
-      <c r="D125" s="15" t="s">
+      <c r="D125" s="13" t="s">
         <v>120</v>
       </c>
       <c r="E125">
@@ -9154,7 +9208,7 @@
         <f t="shared" si="6"/>
         <v>14</v>
       </c>
-      <c r="D126" s="15" t="s">
+      <c r="D126" s="13" t="s">
         <v>126</v>
       </c>
       <c r="E126">
@@ -9173,7 +9227,7 @@
         <f t="shared" si="6"/>
         <v>15</v>
       </c>
-      <c r="D127" s="15" t="s">
+      <c r="D127" s="13" t="s">
         <v>121</v>
       </c>
       <c r="E127">
@@ -9192,7 +9246,7 @@
         <f t="shared" si="6"/>
         <v>16</v>
       </c>
-      <c r="D128" s="15" t="s">
+      <c r="D128" s="13" t="s">
         <v>122</v>
       </c>
       <c r="E128">
@@ -9211,7 +9265,7 @@
         <f t="shared" si="6"/>
         <v>17</v>
       </c>
-      <c r="D129" s="15" t="s">
+      <c r="D129" s="13" t="s">
         <v>123</v>
       </c>
       <c r="E129">
@@ -9230,7 +9284,7 @@
         <f t="shared" si="6"/>
         <v>18</v>
       </c>
-      <c r="D130" s="15" t="s">
+      <c r="D130" s="13" t="s">
         <v>124</v>
       </c>
       <c r="E130">
@@ -9249,7 +9303,7 @@
         <f t="shared" si="6"/>
         <v>19</v>
       </c>
-      <c r="D131" s="15" t="s">
+      <c r="D131" s="13" t="s">
         <v>125</v>
       </c>
       <c r="E131">
@@ -9267,7 +9321,7 @@
       <c r="C132">
         <v>1</v>
       </c>
-      <c r="D132" s="15" t="s">
+      <c r="D132" s="13" t="s">
         <v>131</v>
       </c>
       <c r="E132">
@@ -9285,7 +9339,7 @@
       <c r="C133">
         <v>2</v>
       </c>
-      <c r="D133" s="15" t="s">
+      <c r="D133" s="13" t="s">
         <v>132</v>
       </c>
       <c r="E133">
@@ -9303,7 +9357,7 @@
       <c r="C134">
         <v>3</v>
       </c>
-      <c r="D134" s="15" t="s">
+      <c r="D134" s="13" t="s">
         <v>133</v>
       </c>
       <c r="E134">
@@ -9321,7 +9375,7 @@
       <c r="C135">
         <v>4</v>
       </c>
-      <c r="D135" s="15" t="s">
+      <c r="D135" s="13" t="s">
         <v>134</v>
       </c>
       <c r="E135">
@@ -9339,7 +9393,7 @@
       <c r="C136">
         <v>5</v>
       </c>
-      <c r="D136" s="15" t="s">
+      <c r="D136" s="13" t="s">
         <v>135</v>
       </c>
       <c r="E136">
@@ -9357,7 +9411,7 @@
       <c r="C137">
         <v>1</v>
       </c>
-      <c r="D137" s="15">
+      <c r="D137" s="13">
         <f>C137</f>
         <v>1</v>
       </c>
@@ -9377,7 +9431,7 @@
         <f>C137+1</f>
         <v>2</v>
       </c>
-      <c r="D138" s="15">
+      <c r="D138" s="13">
         <f t="shared" ref="D138:D159" si="8">C138</f>
         <v>2</v>
       </c>
@@ -9397,7 +9451,7 @@
         <f t="shared" ref="C139:C159" si="9">C138+1</f>
         <v>3</v>
       </c>
-      <c r="D139" s="15">
+      <c r="D139" s="13">
         <f t="shared" si="8"/>
         <v>3</v>
       </c>
@@ -9417,7 +9471,7 @@
         <f t="shared" si="9"/>
         <v>4</v>
       </c>
-      <c r="D140" s="15">
+      <c r="D140" s="13">
         <f t="shared" si="8"/>
         <v>4</v>
       </c>
@@ -9437,7 +9491,7 @@
         <f t="shared" si="9"/>
         <v>5</v>
       </c>
-      <c r="D141" s="15">
+      <c r="D141" s="13">
         <f t="shared" si="8"/>
         <v>5</v>
       </c>
@@ -9457,7 +9511,7 @@
         <f t="shared" si="9"/>
         <v>6</v>
       </c>
-      <c r="D142" s="15">
+      <c r="D142" s="13">
         <f t="shared" si="8"/>
         <v>6</v>
       </c>
@@ -9477,7 +9531,7 @@
         <f t="shared" si="9"/>
         <v>7</v>
       </c>
-      <c r="D143" s="15">
+      <c r="D143" s="13">
         <f t="shared" si="8"/>
         <v>7</v>
       </c>
@@ -9497,7 +9551,7 @@
         <f t="shared" si="9"/>
         <v>8</v>
       </c>
-      <c r="D144" s="15">
+      <c r="D144" s="13">
         <f t="shared" si="8"/>
         <v>8</v>
       </c>
@@ -9517,7 +9571,7 @@
         <f t="shared" si="9"/>
         <v>9</v>
       </c>
-      <c r="D145" s="15">
+      <c r="D145" s="13">
         <f t="shared" si="8"/>
         <v>9</v>
       </c>
@@ -9537,7 +9591,7 @@
         <f t="shared" si="9"/>
         <v>10</v>
       </c>
-      <c r="D146" s="15">
+      <c r="D146" s="13">
         <f t="shared" si="8"/>
         <v>10</v>
       </c>
@@ -9557,7 +9611,7 @@
         <f t="shared" si="9"/>
         <v>11</v>
       </c>
-      <c r="D147" s="15">
+      <c r="D147" s="13">
         <f t="shared" si="8"/>
         <v>11</v>
       </c>
@@ -9577,7 +9631,7 @@
         <f t="shared" si="9"/>
         <v>12</v>
       </c>
-      <c r="D148" s="15">
+      <c r="D148" s="13">
         <f t="shared" si="8"/>
         <v>12</v>
       </c>
@@ -9597,7 +9651,7 @@
         <f t="shared" si="9"/>
         <v>13</v>
       </c>
-      <c r="D149" s="15">
+      <c r="D149" s="13">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
@@ -9617,7 +9671,7 @@
         <f t="shared" si="9"/>
         <v>14</v>
       </c>
-      <c r="D150" s="15">
+      <c r="D150" s="13">
         <f t="shared" si="8"/>
         <v>14</v>
       </c>
@@ -9637,7 +9691,7 @@
         <f t="shared" si="9"/>
         <v>15</v>
       </c>
-      <c r="D151" s="15">
+      <c r="D151" s="13">
         <f t="shared" si="8"/>
         <v>15</v>
       </c>
@@ -9657,7 +9711,7 @@
         <f t="shared" si="9"/>
         <v>16</v>
       </c>
-      <c r="D152" s="15">
+      <c r="D152" s="13">
         <f t="shared" si="8"/>
         <v>16</v>
       </c>
@@ -9677,7 +9731,7 @@
         <f t="shared" si="9"/>
         <v>17</v>
       </c>
-      <c r="D153" s="15">
+      <c r="D153" s="13">
         <f t="shared" si="8"/>
         <v>17</v>
       </c>
@@ -9697,7 +9751,7 @@
         <f t="shared" si="9"/>
         <v>18</v>
       </c>
-      <c r="D154" s="15">
+      <c r="D154" s="13">
         <f t="shared" si="8"/>
         <v>18</v>
       </c>
@@ -9717,7 +9771,7 @@
         <f t="shared" si="9"/>
         <v>19</v>
       </c>
-      <c r="D155" s="15">
+      <c r="D155" s="13">
         <f t="shared" si="8"/>
         <v>19</v>
       </c>
@@ -9737,7 +9791,7 @@
         <f t="shared" si="9"/>
         <v>20</v>
       </c>
-      <c r="D156" s="15">
+      <c r="D156" s="13">
         <f t="shared" si="8"/>
         <v>20</v>
       </c>
@@ -9757,7 +9811,7 @@
         <f t="shared" si="9"/>
         <v>21</v>
       </c>
-      <c r="D157" s="15">
+      <c r="D157" s="13">
         <f t="shared" si="8"/>
         <v>21</v>
       </c>
@@ -9777,7 +9831,7 @@
         <f t="shared" si="9"/>
         <v>22</v>
       </c>
-      <c r="D158" s="15">
+      <c r="D158" s="13">
         <f t="shared" si="8"/>
         <v>22</v>
       </c>
@@ -9797,7 +9851,7 @@
         <f t="shared" si="9"/>
         <v>23</v>
       </c>
-      <c r="D159" s="15">
+      <c r="D159" s="13">
         <f t="shared" si="8"/>
         <v>23</v>
       </c>
@@ -9816,7 +9870,7 @@
       <c r="C160">
         <v>24</v>
       </c>
-      <c r="D160" s="15" t="s">
+      <c r="D160" s="13" t="s">
         <v>135</v>
       </c>
       <c r="E160">
@@ -9834,7 +9888,7 @@
       <c r="C161">
         <v>1</v>
       </c>
-      <c r="D161" s="15" t="s">
+      <c r="D161" s="13" t="s">
         <v>148</v>
       </c>
       <c r="E161">
@@ -9852,7 +9906,7 @@
       <c r="C162">
         <v>2</v>
       </c>
-      <c r="D162" s="15" t="s">
+      <c r="D162" s="13" t="s">
         <v>149</v>
       </c>
       <c r="E162">
@@ -9870,7 +9924,7 @@
       <c r="C163">
         <v>3</v>
       </c>
-      <c r="D163" s="15" t="s">
+      <c r="D163" s="13" t="s">
         <v>150</v>
       </c>
       <c r="E163">
@@ -9888,7 +9942,7 @@
       <c r="C164">
         <v>4</v>
       </c>
-      <c r="D164" s="15" t="s">
+      <c r="D164" s="13" t="s">
         <v>151</v>
       </c>
       <c r="E164">
@@ -9906,7 +9960,7 @@
       <c r="C165">
         <v>5</v>
       </c>
-      <c r="D165" s="15" t="s">
+      <c r="D165" s="13" t="s">
         <v>152</v>
       </c>
       <c r="E165">
@@ -9924,7 +9978,7 @@
       <c r="C166">
         <v>6</v>
       </c>
-      <c r="D166" s="15" t="s">
+      <c r="D166" s="13" t="s">
         <v>153</v>
       </c>
       <c r="E166">
@@ -9942,7 +9996,7 @@
       <c r="C167">
         <v>7</v>
       </c>
-      <c r="D167" s="15" t="s">
+      <c r="D167" s="13" t="s">
         <v>154</v>
       </c>
       <c r="E167">
@@ -9960,7 +10014,7 @@
       <c r="C168">
         <v>1</v>
       </c>
-      <c r="D168" s="15" t="s">
+      <c r="D168" s="13" t="s">
         <v>157</v>
       </c>
       <c r="E168">
@@ -9979,7 +10033,7 @@
         <f>C168+1</f>
         <v>2</v>
       </c>
-      <c r="D169" s="15" t="s">
+      <c r="D169" s="13" t="s">
         <v>158</v>
       </c>
       <c r="E169">
@@ -9998,7 +10052,7 @@
         <f t="shared" ref="C170:C212" si="10">C169+1</f>
         <v>3</v>
       </c>
-      <c r="D170" s="15" t="s">
+      <c r="D170" s="13" t="s">
         <v>159</v>
       </c>
       <c r="E170">
@@ -10017,7 +10071,7 @@
         <f t="shared" si="10"/>
         <v>4</v>
       </c>
-      <c r="D171" s="15" t="s">
+      <c r="D171" s="13" t="s">
         <v>160</v>
       </c>
       <c r="E171">
@@ -10036,7 +10090,7 @@
         <f t="shared" si="10"/>
         <v>5</v>
       </c>
-      <c r="D172" s="15" t="s">
+      <c r="D172" s="13" t="s">
         <v>161</v>
       </c>
       <c r="E172">
@@ -10055,7 +10109,7 @@
         <f t="shared" si="10"/>
         <v>6</v>
       </c>
-      <c r="D173" s="15" t="s">
+      <c r="D173" s="13" t="s">
         <v>162</v>
       </c>
       <c r="E173">
@@ -10074,7 +10128,7 @@
         <f t="shared" si="10"/>
         <v>7</v>
       </c>
-      <c r="D174" s="15" t="s">
+      <c r="D174" s="13" t="s">
         <v>163</v>
       </c>
       <c r="E174">
@@ -10093,7 +10147,7 @@
         <f t="shared" si="10"/>
         <v>8</v>
       </c>
-      <c r="D175" s="15" t="s">
+      <c r="D175" s="13" t="s">
         <v>164</v>
       </c>
       <c r="E175">
@@ -10112,7 +10166,7 @@
         <f t="shared" si="10"/>
         <v>9</v>
       </c>
-      <c r="D176" s="15" t="s">
+      <c r="D176" s="13" t="s">
         <v>165</v>
       </c>
       <c r="E176">
@@ -10131,7 +10185,7 @@
         <f t="shared" si="10"/>
         <v>10</v>
       </c>
-      <c r="D177" s="15" t="s">
+      <c r="D177" s="13" t="s">
         <v>166</v>
       </c>
       <c r="E177">
@@ -10150,7 +10204,7 @@
         <f t="shared" si="10"/>
         <v>11</v>
       </c>
-      <c r="D178" s="15" t="s">
+      <c r="D178" s="13" t="s">
         <v>167</v>
       </c>
       <c r="E178">
@@ -10169,7 +10223,7 @@
         <f t="shared" si="10"/>
         <v>12</v>
       </c>
-      <c r="D179" s="15" t="s">
+      <c r="D179" s="13" t="s">
         <v>168</v>
       </c>
       <c r="E179">
@@ -10188,7 +10242,7 @@
         <f t="shared" si="10"/>
         <v>13</v>
       </c>
-      <c r="D180" s="15" t="s">
+      <c r="D180" s="13" t="s">
         <v>169</v>
       </c>
       <c r="E180">
@@ -10207,7 +10261,7 @@
         <f t="shared" si="10"/>
         <v>14</v>
       </c>
-      <c r="D181" s="15" t="s">
+      <c r="D181" s="13" t="s">
         <v>170</v>
       </c>
       <c r="E181">
@@ -10226,7 +10280,7 @@
         <f t="shared" si="10"/>
         <v>15</v>
       </c>
-      <c r="D182" s="15" t="s">
+      <c r="D182" s="13" t="s">
         <v>171</v>
       </c>
       <c r="E182">
@@ -10245,7 +10299,7 @@
         <f t="shared" si="10"/>
         <v>16</v>
       </c>
-      <c r="D183" s="15" t="s">
+      <c r="D183" s="13" t="s">
         <v>172</v>
       </c>
       <c r="E183">
@@ -10264,7 +10318,7 @@
         <f t="shared" si="10"/>
         <v>17</v>
       </c>
-      <c r="D184" s="15" t="s">
+      <c r="D184" s="13" t="s">
         <v>173</v>
       </c>
       <c r="E184">
@@ -10283,7 +10337,7 @@
         <f t="shared" si="10"/>
         <v>18</v>
       </c>
-      <c r="D185" s="15" t="s">
+      <c r="D185" s="13" t="s">
         <v>174</v>
       </c>
       <c r="E185">
@@ -10302,7 +10356,7 @@
         <f t="shared" si="10"/>
         <v>19</v>
       </c>
-      <c r="D186" s="15" t="s">
+      <c r="D186" s="13" t="s">
         <v>175</v>
       </c>
       <c r="E186">
@@ -10321,7 +10375,7 @@
         <f t="shared" si="10"/>
         <v>20</v>
       </c>
-      <c r="D187" s="15" t="s">
+      <c r="D187" s="13" t="s">
         <v>176</v>
       </c>
       <c r="E187">
@@ -10340,7 +10394,7 @@
         <f t="shared" si="10"/>
         <v>21</v>
       </c>
-      <c r="D188" s="15" t="s">
+      <c r="D188" s="13" t="s">
         <v>178</v>
       </c>
       <c r="E188">
@@ -10359,7 +10413,7 @@
         <f t="shared" si="10"/>
         <v>22</v>
       </c>
-      <c r="D189" s="15" t="s">
+      <c r="D189" s="13" t="s">
         <v>177</v>
       </c>
       <c r="E189">
@@ -10378,7 +10432,7 @@
         <f t="shared" si="10"/>
         <v>23</v>
       </c>
-      <c r="D190" s="15" t="s">
+      <c r="D190" s="13" t="s">
         <v>179</v>
       </c>
       <c r="E190">
@@ -10397,7 +10451,7 @@
         <f t="shared" si="10"/>
         <v>24</v>
       </c>
-      <c r="D191" s="15" t="s">
+      <c r="D191" s="13" t="s">
         <v>180</v>
       </c>
       <c r="E191">
@@ -10416,7 +10470,7 @@
         <f t="shared" si="10"/>
         <v>25</v>
       </c>
-      <c r="D192" s="15" t="s">
+      <c r="D192" s="13" t="s">
         <v>181</v>
       </c>
       <c r="E192">
@@ -10435,7 +10489,7 @@
         <f t="shared" si="10"/>
         <v>26</v>
       </c>
-      <c r="D193" s="15" t="s">
+      <c r="D193" s="13" t="s">
         <v>182</v>
       </c>
       <c r="E193">
@@ -10454,7 +10508,7 @@
         <f t="shared" si="10"/>
         <v>27</v>
       </c>
-      <c r="D194" s="15" t="s">
+      <c r="D194" s="13" t="s">
         <v>183</v>
       </c>
       <c r="E194">
@@ -10473,7 +10527,7 @@
         <f t="shared" si="10"/>
         <v>28</v>
       </c>
-      <c r="D195" s="15" t="s">
+      <c r="D195" s="13" t="s">
         <v>184</v>
       </c>
       <c r="E195">
@@ -10492,7 +10546,7 @@
         <f t="shared" si="10"/>
         <v>29</v>
       </c>
-      <c r="D196" s="15" t="s">
+      <c r="D196" s="13" t="s">
         <v>185</v>
       </c>
       <c r="E196">
@@ -10511,7 +10565,7 @@
         <f t="shared" si="10"/>
         <v>30</v>
       </c>
-      <c r="D197" s="15" t="s">
+      <c r="D197" s="13" t="s">
         <v>186</v>
       </c>
       <c r="E197">
@@ -10530,7 +10584,7 @@
         <f t="shared" si="10"/>
         <v>31</v>
       </c>
-      <c r="D198" s="15" t="s">
+      <c r="D198" s="13" t="s">
         <v>187</v>
       </c>
       <c r="E198">
@@ -10549,7 +10603,7 @@
         <f t="shared" si="10"/>
         <v>32</v>
       </c>
-      <c r="D199" s="15" t="s">
+      <c r="D199" s="13" t="s">
         <v>188</v>
       </c>
       <c r="E199">
@@ -10568,7 +10622,7 @@
         <f t="shared" si="10"/>
         <v>33</v>
       </c>
-      <c r="D200" s="15" t="s">
+      <c r="D200" s="13" t="s">
         <v>189</v>
       </c>
       <c r="E200">
@@ -10587,7 +10641,7 @@
         <f t="shared" si="10"/>
         <v>34</v>
       </c>
-      <c r="D201" s="15" t="s">
+      <c r="D201" s="13" t="s">
         <v>190</v>
       </c>
       <c r="E201">
@@ -10606,7 +10660,7 @@
         <f t="shared" si="10"/>
         <v>35</v>
       </c>
-      <c r="D202" s="15" t="s">
+      <c r="D202" s="13" t="s">
         <v>191</v>
       </c>
       <c r="E202">
@@ -10625,7 +10679,7 @@
         <f t="shared" si="10"/>
         <v>36</v>
       </c>
-      <c r="D203" s="15" t="s">
+      <c r="D203" s="13" t="s">
         <v>192</v>
       </c>
       <c r="E203">
@@ -10644,7 +10698,7 @@
         <f t="shared" si="10"/>
         <v>37</v>
       </c>
-      <c r="D204" s="15" t="s">
+      <c r="D204" s="13" t="s">
         <v>193</v>
       </c>
       <c r="E204">
@@ -10663,7 +10717,7 @@
         <f t="shared" si="10"/>
         <v>38</v>
       </c>
-      <c r="D205" s="15" t="s">
+      <c r="D205" s="13" t="s">
         <v>194</v>
       </c>
       <c r="E205">
@@ -10682,7 +10736,7 @@
         <f t="shared" si="10"/>
         <v>39</v>
       </c>
-      <c r="D206" s="15" t="s">
+      <c r="D206" s="13" t="s">
         <v>195</v>
       </c>
       <c r="E206">
@@ -10701,7 +10755,7 @@
         <f t="shared" si="10"/>
         <v>40</v>
       </c>
-      <c r="D207" s="15" t="s">
+      <c r="D207" s="13" t="s">
         <v>196</v>
       </c>
       <c r="E207">
@@ -10720,7 +10774,7 @@
         <f t="shared" si="10"/>
         <v>41</v>
       </c>
-      <c r="D208" s="15" t="s">
+      <c r="D208" s="13" t="s">
         <v>197</v>
       </c>
       <c r="E208">
@@ -10739,7 +10793,7 @@
         <f t="shared" si="10"/>
         <v>42</v>
       </c>
-      <c r="D209" s="15" t="s">
+      <c r="D209" s="13" t="s">
         <v>198</v>
       </c>
       <c r="E209">
@@ -10758,7 +10812,7 @@
         <f t="shared" si="10"/>
         <v>43</v>
       </c>
-      <c r="D210" s="15" t="s">
+      <c r="D210" s="13" t="s">
         <v>199</v>
       </c>
       <c r="E210">
@@ -10777,7 +10831,7 @@
         <f t="shared" si="10"/>
         <v>44</v>
       </c>
-      <c r="D211" s="15" t="s">
+      <c r="D211" s="13" t="s">
         <v>201</v>
       </c>
       <c r="E211">
@@ -10796,7 +10850,7 @@
         <f t="shared" si="10"/>
         <v>45</v>
       </c>
-      <c r="D212" s="15" t="s">
+      <c r="D212" s="13" t="s">
         <v>200</v>
       </c>
       <c r="E212">
@@ -10814,7 +10868,7 @@
       <c r="C213">
         <v>1</v>
       </c>
-      <c r="D213" s="15" t="s">
+      <c r="D213" s="13" t="s">
         <v>207</v>
       </c>
       <c r="E213">
@@ -10833,7 +10887,7 @@
         <f>C213+1</f>
         <v>2</v>
       </c>
-      <c r="D214" s="15">
+      <c r="D214" s="13">
         <v>1</v>
       </c>
       <c r="E214">
@@ -10852,7 +10906,7 @@
         <f t="shared" ref="C215:C225" si="12">C214+1</f>
         <v>3</v>
       </c>
-      <c r="D215" s="15">
+      <c r="D215" s="13">
         <v>2</v>
       </c>
       <c r="E215">
@@ -10871,7 +10925,7 @@
         <f t="shared" si="12"/>
         <v>4</v>
       </c>
-      <c r="D216" s="15">
+      <c r="D216" s="13">
         <v>3</v>
       </c>
       <c r="E216">
@@ -10890,7 +10944,7 @@
         <f t="shared" si="12"/>
         <v>5</v>
       </c>
-      <c r="D217" s="15">
+      <c r="D217" s="13">
         <v>4</v>
       </c>
       <c r="E217">
@@ -10909,7 +10963,7 @@
         <f t="shared" si="12"/>
         <v>6</v>
       </c>
-      <c r="D218" s="15">
+      <c r="D218" s="13">
         <v>5</v>
       </c>
       <c r="E218">
@@ -10928,7 +10982,7 @@
         <f t="shared" si="12"/>
         <v>7</v>
       </c>
-      <c r="D219" s="15">
+      <c r="D219" s="13">
         <v>6</v>
       </c>
       <c r="E219">
@@ -10947,7 +11001,7 @@
         <f t="shared" si="12"/>
         <v>8</v>
       </c>
-      <c r="D220" s="15">
+      <c r="D220" s="13">
         <v>7</v>
       </c>
       <c r="E220">
@@ -10966,7 +11020,7 @@
         <f t="shared" si="12"/>
         <v>9</v>
       </c>
-      <c r="D221" s="15">
+      <c r="D221" s="13">
         <v>8</v>
       </c>
       <c r="E221">
@@ -10985,7 +11039,7 @@
         <f t="shared" si="12"/>
         <v>10</v>
       </c>
-      <c r="D222" s="15">
+      <c r="D222" s="13">
         <v>9</v>
       </c>
       <c r="E222">
@@ -11004,7 +11058,7 @@
         <f t="shared" si="12"/>
         <v>11</v>
       </c>
-      <c r="D223" s="15">
+      <c r="D223" s="13">
         <v>10</v>
       </c>
       <c r="E223">
@@ -11023,7 +11077,7 @@
         <f t="shared" si="12"/>
         <v>12</v>
       </c>
-      <c r="D224" s="15">
+      <c r="D224" s="13">
         <v>11</v>
       </c>
       <c r="E224">
@@ -11042,7 +11096,7 @@
         <f t="shared" si="12"/>
         <v>13</v>
       </c>
-      <c r="D225" s="15">
+      <c r="D225" s="13">
         <v>12</v>
       </c>
       <c r="E225">

</xml_diff>

<commit_message>
data (Songs of Innocence and of Experience)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/code/projects/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9EE02B8-57C9-7E4B-A31C-F4133E2FE74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7AE0CEC-F603-B042-91D7-065EF5B0B3D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="19220" windowHeight="20980" activeTab="1" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="19220" windowHeight="20980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="214">
   <si>
     <t>book_id</t>
   </si>
@@ -671,6 +671,12 @@
   </si>
   <si>
     <t>The Lord</t>
+  </si>
+  <si>
+    <t>Songs of Innocence and of Experience</t>
+  </si>
+  <si>
+    <t>William Blake</t>
   </si>
 </sst>
 </file>
@@ -1075,7 +1081,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -2007,6 +2013,44 @@
       </c>
       <c r="L24" s="7">
         <v>46206</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>212</v>
+      </c>
+      <c r="C25" t="s">
+        <v>213</v>
+      </c>
+      <c r="D25" t="s">
+        <v>144</v>
+      </c>
+      <c r="E25">
+        <v>1794</v>
+      </c>
+      <c r="F25" t="s">
+        <v>16</v>
+      </c>
+      <c r="G25">
+        <v>155</v>
+      </c>
+      <c r="H25" s="11">
+        <v>5379</v>
+      </c>
+      <c r="I25" t="s">
+        <v>104</v>
+      </c>
+      <c r="J25" t="s">
+        <v>76</v>
+      </c>
+      <c r="K25" s="7">
+        <v>46207</v>
+      </c>
+      <c r="L25" s="7">
+        <v>46209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data (Three Hainish Novels)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/code/projects/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F773D4F-DF79-574D-8A89-27B94C9AACBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268B24E8-9E93-E442-A2CE-A39858E0DE56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="680" windowWidth="15120" windowHeight="18980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="15420" windowHeight="18980" activeTab="2" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="221">
   <si>
     <t>book_id</t>
   </si>
@@ -683,6 +683,21 @@
   </si>
   <si>
     <t>Robert Coover</t>
+  </si>
+  <si>
+    <t>Three Hainish Novels</t>
+  </si>
+  <si>
+    <t>Ursula K. Le Guin</t>
+  </si>
+  <si>
+    <t>Rocannon's World</t>
+  </si>
+  <si>
+    <t>Planet of Exile</t>
+  </si>
+  <si>
+    <t>City of Illusions</t>
   </si>
 </sst>
 </file>
@@ -737,7 +752,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -751,8 +766,6 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1087,7 +1100,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -2097,6 +2110,44 @@
         <v>46212</v>
       </c>
     </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>216</v>
+      </c>
+      <c r="C27" t="s">
+        <v>217</v>
+      </c>
+      <c r="D27" t="s">
+        <v>17</v>
+      </c>
+      <c r="E27">
+        <v>1966</v>
+      </c>
+      <c r="F27" t="s">
+        <v>16</v>
+      </c>
+      <c r="G27">
+        <v>367</v>
+      </c>
+      <c r="H27" s="11">
+        <v>143071</v>
+      </c>
+      <c r="I27" t="s">
+        <v>104</v>
+      </c>
+      <c r="J27" t="s">
+        <v>67</v>
+      </c>
+      <c r="K27" s="7">
+        <v>46214</v>
+      </c>
+      <c r="L27" s="7">
+        <v>46220</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2104,7 +2155,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I250"/>
+  <dimension ref="A1:I274"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -6192,7 +6243,7 @@
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A195">
-        <f t="shared" ref="A195:A250" si="3">ROW() - 1</f>
+        <f t="shared" ref="A195:A258" si="3">ROW() - 1</f>
         <v>194</v>
       </c>
       <c r="B195">
@@ -7364,6 +7415,510 @@
       </c>
       <c r="F250" s="6">
         <v>1.7256944444444443E-2</v>
+      </c>
+    </row>
+    <row r="251" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A251">
+        <f t="shared" si="3"/>
+        <v>250</v>
+      </c>
+      <c r="B251">
+        <v>26</v>
+      </c>
+      <c r="C251" s="3">
+        <v>46214.40347222222</v>
+      </c>
+      <c r="D251">
+        <v>3</v>
+      </c>
+      <c r="E251">
+        <v>16</v>
+      </c>
+      <c r="F251" s="6">
+        <v>1.5277777777777777E-2</v>
+      </c>
+    </row>
+    <row r="252" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A252">
+        <f t="shared" si="3"/>
+        <v>251</v>
+      </c>
+      <c r="B252">
+        <v>26</v>
+      </c>
+      <c r="C252" s="3">
+        <v>46214.689583333333</v>
+      </c>
+      <c r="D252">
+        <v>16</v>
+      </c>
+      <c r="E252">
+        <v>28</v>
+      </c>
+      <c r="F252" s="6">
+        <v>1.1215277777777777E-2</v>
+      </c>
+    </row>
+    <row r="253" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A253">
+        <f t="shared" si="3"/>
+        <v>252</v>
+      </c>
+      <c r="B253">
+        <v>26</v>
+      </c>
+      <c r="C253" s="3">
+        <v>46215.865972222222</v>
+      </c>
+      <c r="D253">
+        <v>28</v>
+      </c>
+      <c r="E253">
+        <v>39</v>
+      </c>
+      <c r="F253" s="6">
+        <v>1.2291666666666666E-2</v>
+      </c>
+    </row>
+    <row r="254" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A254">
+        <f t="shared" si="3"/>
+        <v>253</v>
+      </c>
+      <c r="B254">
+        <v>26</v>
+      </c>
+      <c r="C254" s="3">
+        <v>46216.439583333333</v>
+      </c>
+      <c r="D254">
+        <v>39</v>
+      </c>
+      <c r="E254">
+        <v>49</v>
+      </c>
+      <c r="F254" s="6">
+        <v>9.7569444444444448E-3</v>
+      </c>
+    </row>
+    <row r="255" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A255">
+        <f t="shared" si="3"/>
+        <v>254</v>
+      </c>
+      <c r="B255">
+        <v>26</v>
+      </c>
+      <c r="C255" s="3">
+        <v>46216.479861111111</v>
+      </c>
+      <c r="D255">
+        <v>49</v>
+      </c>
+      <c r="E255">
+        <v>72</v>
+      </c>
+      <c r="F255" s="6">
+        <v>2.0185185185185184E-2</v>
+      </c>
+    </row>
+    <row r="256" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A256">
+        <f t="shared" si="3"/>
+        <v>255</v>
+      </c>
+      <c r="B256">
+        <v>26</v>
+      </c>
+      <c r="C256" s="3">
+        <v>46216.64166666667</v>
+      </c>
+      <c r="D256">
+        <v>72</v>
+      </c>
+      <c r="E256">
+        <v>92</v>
+      </c>
+      <c r="F256" s="6">
+        <v>1.9108796296296297E-2</v>
+      </c>
+    </row>
+    <row r="257" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A257">
+        <f t="shared" si="3"/>
+        <v>256</v>
+      </c>
+      <c r="B257">
+        <v>26</v>
+      </c>
+      <c r="C257" s="3">
+        <v>46216.775694444441</v>
+      </c>
+      <c r="D257">
+        <v>92</v>
+      </c>
+      <c r="E257">
+        <v>115</v>
+      </c>
+      <c r="F257" s="6">
+        <v>1.6597222222222222E-2</v>
+      </c>
+    </row>
+    <row r="258" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A258">
+        <f t="shared" si="3"/>
+        <v>257</v>
+      </c>
+      <c r="B258">
+        <v>26</v>
+      </c>
+      <c r="C258" s="3">
+        <v>46217.47152777778</v>
+      </c>
+      <c r="D258">
+        <v>115</v>
+      </c>
+      <c r="E258">
+        <v>132</v>
+      </c>
+      <c r="F258" s="6">
+        <v>1.7372685185185185E-2</v>
+      </c>
+    </row>
+    <row r="259" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A259">
+        <f t="shared" ref="A259:A274" si="4">ROW() - 1</f>
+        <v>258</v>
+      </c>
+      <c r="B259">
+        <v>26</v>
+      </c>
+      <c r="C259" s="3">
+        <v>46217.645833333336</v>
+      </c>
+      <c r="D259">
+        <v>132</v>
+      </c>
+      <c r="E259">
+        <v>139</v>
+      </c>
+      <c r="F259" s="6">
+        <v>7.3958333333333333E-3</v>
+      </c>
+    </row>
+    <row r="260" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A260">
+        <f t="shared" si="4"/>
+        <v>259</v>
+      </c>
+      <c r="B260">
+        <v>26</v>
+      </c>
+      <c r="C260" s="3">
+        <v>46217.665277777778</v>
+      </c>
+      <c r="D260">
+        <v>139</v>
+      </c>
+      <c r="E260">
+        <v>152</v>
+      </c>
+      <c r="F260" s="6">
+        <v>1.105324074074074E-2</v>
+      </c>
+    </row>
+    <row r="261" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A261">
+        <f t="shared" si="4"/>
+        <v>260</v>
+      </c>
+      <c r="B261">
+        <v>26</v>
+      </c>
+      <c r="C261" s="3">
+        <v>46217.793055555558</v>
+      </c>
+      <c r="D261">
+        <v>152</v>
+      </c>
+      <c r="E261">
+        <v>162</v>
+      </c>
+      <c r="F261" s="6">
+        <v>8.7152777777777784E-3</v>
+      </c>
+    </row>
+    <row r="262" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A262">
+        <f t="shared" si="4"/>
+        <v>261</v>
+      </c>
+      <c r="B262">
+        <v>26</v>
+      </c>
+      <c r="C262" s="3">
+        <v>46217.820138888892</v>
+      </c>
+      <c r="D262">
+        <v>162</v>
+      </c>
+      <c r="E262">
+        <v>178</v>
+      </c>
+      <c r="F262" s="6">
+        <v>1.4490740740740742E-2</v>
+      </c>
+    </row>
+    <row r="263" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A263">
+        <f t="shared" si="4"/>
+        <v>262</v>
+      </c>
+      <c r="B263">
+        <v>26</v>
+      </c>
+      <c r="C263" s="3">
+        <v>46217.897916666669</v>
+      </c>
+      <c r="D263">
+        <v>178</v>
+      </c>
+      <c r="E263">
+        <v>198</v>
+      </c>
+      <c r="F263" s="6">
+        <v>1.7314814814814814E-2</v>
+      </c>
+    </row>
+    <row r="264" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A264">
+        <f t="shared" si="4"/>
+        <v>263</v>
+      </c>
+      <c r="B264">
+        <v>26</v>
+      </c>
+      <c r="C264" s="3">
+        <v>46218.69027777778</v>
+      </c>
+      <c r="D264">
+        <v>198</v>
+      </c>
+      <c r="E264">
+        <v>215</v>
+      </c>
+      <c r="F264" s="6">
+        <v>1.0844907407407407E-2</v>
+      </c>
+    </row>
+    <row r="265" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A265">
+        <f t="shared" si="4"/>
+        <v>264</v>
+      </c>
+      <c r="B265">
+        <v>26</v>
+      </c>
+      <c r="C265" s="3">
+        <v>46219.750694444447</v>
+      </c>
+      <c r="D265">
+        <v>215</v>
+      </c>
+      <c r="E265">
+        <v>230</v>
+      </c>
+      <c r="F265" s="6">
+        <v>1.5057870370370371E-2</v>
+      </c>
+    </row>
+    <row r="266" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A266">
+        <f t="shared" si="4"/>
+        <v>265</v>
+      </c>
+      <c r="B266">
+        <v>26</v>
+      </c>
+      <c r="C266" s="3">
+        <v>46219.784722222219</v>
+      </c>
+      <c r="D266">
+        <v>230</v>
+      </c>
+      <c r="E266">
+        <v>248</v>
+      </c>
+      <c r="F266" s="6">
+        <v>1.457175925925926E-2</v>
+      </c>
+    </row>
+    <row r="267" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A267">
+        <f t="shared" si="4"/>
+        <v>266</v>
+      </c>
+      <c r="B267">
+        <v>26</v>
+      </c>
+      <c r="C267" s="3">
+        <v>46219.878472222219</v>
+      </c>
+      <c r="D267">
+        <v>248</v>
+      </c>
+      <c r="E267">
+        <v>262</v>
+      </c>
+      <c r="F267" s="6">
+        <v>1.3321759259259259E-2</v>
+      </c>
+    </row>
+    <row r="268" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A268">
+        <f t="shared" si="4"/>
+        <v>267</v>
+      </c>
+      <c r="B268">
+        <v>26</v>
+      </c>
+      <c r="C268" s="3">
+        <v>46220.428472222222</v>
+      </c>
+      <c r="D268">
+        <v>262</v>
+      </c>
+      <c r="E268">
+        <v>276</v>
+      </c>
+      <c r="F268" s="6">
+        <v>1.2673611111111111E-2</v>
+      </c>
+    </row>
+    <row r="269" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A269">
+        <f t="shared" si="4"/>
+        <v>268</v>
+      </c>
+      <c r="B269">
+        <v>26</v>
+      </c>
+      <c r="C269" s="3">
+        <v>46220.449305555558</v>
+      </c>
+      <c r="D269">
+        <v>276</v>
+      </c>
+      <c r="E269">
+        <v>291</v>
+      </c>
+      <c r="F269" s="6">
+        <v>1.21875E-2</v>
+      </c>
+    </row>
+    <row r="270" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A270">
+        <f t="shared" si="4"/>
+        <v>269</v>
+      </c>
+      <c r="B270">
+        <v>26</v>
+      </c>
+      <c r="C270" s="3">
+        <v>46220.535416666666</v>
+      </c>
+      <c r="D270">
+        <v>291</v>
+      </c>
+      <c r="E270">
+        <v>307</v>
+      </c>
+      <c r="F270" s="6">
+        <v>1.4456018518518519E-2</v>
+      </c>
+    </row>
+    <row r="271" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A271">
+        <f t="shared" si="4"/>
+        <v>270</v>
+      </c>
+      <c r="B271">
+        <v>26</v>
+      </c>
+      <c r="C271" s="3">
+        <v>46220.647916666669</v>
+      </c>
+      <c r="D271">
+        <v>307</v>
+      </c>
+      <c r="E271">
+        <v>320</v>
+      </c>
+      <c r="F271" s="6">
+        <v>1.0416666666666666E-2</v>
+      </c>
+    </row>
+    <row r="272" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A272">
+        <f t="shared" si="4"/>
+        <v>271</v>
+      </c>
+      <c r="B272">
+        <v>26</v>
+      </c>
+      <c r="C272" s="3">
+        <v>46220.681944444441</v>
+      </c>
+      <c r="D272">
+        <v>320</v>
+      </c>
+      <c r="E272">
+        <v>339</v>
+      </c>
+      <c r="F272" s="6">
+        <v>1.4363425925925925E-2</v>
+      </c>
+    </row>
+    <row r="273" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A273">
+        <f t="shared" si="4"/>
+        <v>272</v>
+      </c>
+      <c r="B273">
+        <v>26</v>
+      </c>
+      <c r="C273" s="3">
+        <v>46220.715277777781</v>
+      </c>
+      <c r="D273">
+        <v>339</v>
+      </c>
+      <c r="E273">
+        <v>356</v>
+      </c>
+      <c r="F273" s="6">
+        <v>1.3125E-2</v>
+      </c>
+    </row>
+    <row r="274" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A274">
+        <f t="shared" si="4"/>
+        <v>273</v>
+      </c>
+      <c r="B274">
+        <v>26</v>
+      </c>
+      <c r="C274" s="3">
+        <v>46220.740277777775</v>
+      </c>
+      <c r="D274">
+        <v>356</v>
+      </c>
+      <c r="E274">
+        <v>370</v>
+      </c>
+      <c r="F274" s="6">
+        <v>1.0717592592592593E-2</v>
       </c>
     </row>
   </sheetData>
@@ -7373,12 +7928,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CC89663-E888-2445-AD16-77803353ADBB}">
-  <dimension ref="A1:E233"/>
+  <dimension ref="A1:E236"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.5" style="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
   </cols>
@@ -7393,7 +7948,7 @@
       <c r="C1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="1" t="s">
         <v>13</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -7411,7 +7966,7 @@
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" t="s">
         <v>37</v>
       </c>
       <c r="E2">
@@ -7429,7 +7984,7 @@
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" t="s">
         <v>18</v>
       </c>
       <c r="E3">
@@ -7447,7 +8002,7 @@
       <c r="C4">
         <v>3</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" t="s">
         <v>19</v>
       </c>
       <c r="E4">
@@ -7465,7 +8020,7 @@
       <c r="C5">
         <v>4</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" t="s">
         <v>20</v>
       </c>
       <c r="E5">
@@ -7483,7 +8038,7 @@
       <c r="C6">
         <v>5</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" t="s">
         <v>21</v>
       </c>
       <c r="E6">
@@ -7501,7 +8056,7 @@
       <c r="C7">
         <v>6</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" t="s">
         <v>22</v>
       </c>
       <c r="E7">
@@ -7519,7 +8074,7 @@
       <c r="C8">
         <v>7</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" t="s">
         <v>23</v>
       </c>
       <c r="E8">
@@ -7537,7 +8092,7 @@
       <c r="C9">
         <v>8</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" t="s">
         <v>24</v>
       </c>
       <c r="E9">
@@ -7555,7 +8110,7 @@
       <c r="C10">
         <v>9</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D10" t="s">
         <v>25</v>
       </c>
       <c r="E10">
@@ -7573,7 +8128,7 @@
       <c r="C11">
         <v>10</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" t="s">
         <v>26</v>
       </c>
       <c r="E11">
@@ -7591,7 +8146,7 @@
       <c r="C12">
         <v>11</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" t="s">
         <v>27</v>
       </c>
       <c r="E12">
@@ -7609,7 +8164,7 @@
       <c r="C13">
         <v>12</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" t="s">
         <v>28</v>
       </c>
       <c r="E13">
@@ -7627,7 +8182,7 @@
       <c r="C14">
         <v>13</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" t="s">
         <v>29</v>
       </c>
       <c r="E14">
@@ -7645,7 +8200,7 @@
       <c r="C15">
         <v>14</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D15" t="s">
         <v>30</v>
       </c>
       <c r="E15">
@@ -7663,7 +8218,7 @@
       <c r="C16">
         <v>15</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="D16" t="s">
         <v>31</v>
       </c>
       <c r="E16">
@@ -7681,7 +8236,7 @@
       <c r="C17">
         <v>16</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="D17" t="s">
         <v>32</v>
       </c>
       <c r="E17">
@@ -7699,7 +8254,7 @@
       <c r="C18">
         <v>17</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" t="s">
         <v>33</v>
       </c>
       <c r="E18">
@@ -7717,7 +8272,7 @@
       <c r="C19">
         <v>18</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="D19" t="s">
         <v>34</v>
       </c>
       <c r="E19">
@@ -7735,7 +8290,7 @@
       <c r="C20">
         <v>19</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" t="s">
         <v>35</v>
       </c>
       <c r="E20">
@@ -7753,7 +8308,7 @@
       <c r="C21">
         <v>20</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" t="s">
         <v>36</v>
       </c>
       <c r="E21">
@@ -7771,7 +8326,7 @@
       <c r="C22">
         <v>1</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="D22" t="s">
         <v>39</v>
       </c>
       <c r="E22">
@@ -7789,7 +8344,7 @@
       <c r="C23">
         <v>2</v>
       </c>
-      <c r="D23" s="14" t="s">
+      <c r="D23" t="s">
         <v>40</v>
       </c>
       <c r="E23">
@@ -7807,7 +8362,7 @@
       <c r="C24">
         <v>3</v>
       </c>
-      <c r="D24" s="14" t="s">
+      <c r="D24" t="s">
         <v>41</v>
       </c>
       <c r="E24">
@@ -7825,7 +8380,7 @@
       <c r="C25">
         <v>4</v>
       </c>
-      <c r="D25" s="14" t="s">
+      <c r="D25" t="s">
         <v>42</v>
       </c>
       <c r="E25">
@@ -7843,7 +8398,7 @@
       <c r="C26">
         <v>5</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="D26" t="s">
         <v>43</v>
       </c>
       <c r="E26">
@@ -7861,7 +8416,7 @@
       <c r="C27">
         <v>6</v>
       </c>
-      <c r="D27" s="14" t="s">
+      <c r="D27" t="s">
         <v>44</v>
       </c>
       <c r="E27">
@@ -7879,7 +8434,7 @@
       <c r="C28">
         <v>7</v>
       </c>
-      <c r="D28" s="14" t="s">
+      <c r="D28" t="s">
         <v>45</v>
       </c>
       <c r="E28">
@@ -7897,7 +8452,7 @@
       <c r="C29">
         <v>8</v>
       </c>
-      <c r="D29" s="14" t="s">
+      <c r="D29" t="s">
         <v>46</v>
       </c>
       <c r="E29">
@@ -7915,7 +8470,7 @@
       <c r="C30">
         <v>9</v>
       </c>
-      <c r="D30" s="14" t="s">
+      <c r="D30" t="s">
         <v>47</v>
       </c>
       <c r="E30">
@@ -7933,7 +8488,7 @@
       <c r="C31">
         <v>10</v>
       </c>
-      <c r="D31" s="14" t="s">
+      <c r="D31" t="s">
         <v>48</v>
       </c>
       <c r="E31">
@@ -7951,7 +8506,7 @@
       <c r="C32">
         <v>11</v>
       </c>
-      <c r="D32" s="14" t="s">
+      <c r="D32" t="s">
         <v>49</v>
       </c>
       <c r="E32">
@@ -7969,7 +8524,7 @@
       <c r="C33">
         <v>12</v>
       </c>
-      <c r="D33" s="14" t="s">
+      <c r="D33" t="s">
         <v>50</v>
       </c>
       <c r="E33">
@@ -7987,7 +8542,7 @@
       <c r="C34">
         <v>13</v>
       </c>
-      <c r="D34" s="14" t="s">
+      <c r="D34" t="s">
         <v>51</v>
       </c>
       <c r="E34">
@@ -8005,7 +8560,7 @@
       <c r="C35">
         <v>14</v>
       </c>
-      <c r="D35" s="14" t="s">
+      <c r="D35" t="s">
         <v>52</v>
       </c>
       <c r="E35">
@@ -8023,7 +8578,7 @@
       <c r="C36">
         <v>15</v>
       </c>
-      <c r="D36" s="14" t="s">
+      <c r="D36" t="s">
         <v>53</v>
       </c>
       <c r="E36">
@@ -8041,7 +8596,7 @@
       <c r="C37">
         <v>16</v>
       </c>
-      <c r="D37" s="14" t="s">
+      <c r="D37" t="s">
         <v>54</v>
       </c>
       <c r="E37">
@@ -8059,7 +8614,7 @@
       <c r="C38">
         <v>17</v>
       </c>
-      <c r="D38" s="14" t="s">
+      <c r="D38" t="s">
         <v>55</v>
       </c>
       <c r="E38">
@@ -8077,7 +8632,7 @@
       <c r="C39">
         <v>18</v>
       </c>
-      <c r="D39" s="14" t="s">
+      <c r="D39" t="s">
         <v>56</v>
       </c>
       <c r="E39">
@@ -8095,7 +8650,7 @@
       <c r="C40">
         <v>19</v>
       </c>
-      <c r="D40" s="14" t="s">
+      <c r="D40" t="s">
         <v>57</v>
       </c>
       <c r="E40">
@@ -8113,7 +8668,7 @@
       <c r="C41">
         <v>20</v>
       </c>
-      <c r="D41" s="14" t="s">
+      <c r="D41" t="s">
         <v>58</v>
       </c>
       <c r="E41">
@@ -8131,7 +8686,7 @@
       <c r="C42">
         <v>21</v>
       </c>
-      <c r="D42" s="14" t="s">
+      <c r="D42" t="s">
         <v>59</v>
       </c>
       <c r="E42">
@@ -8149,7 +8704,7 @@
       <c r="C43">
         <v>1</v>
       </c>
-      <c r="D43" s="14">
+      <c r="D43">
         <f>C43</f>
         <v>1</v>
       </c>
@@ -8168,7 +8723,7 @@
       <c r="C44">
         <v>2</v>
       </c>
-      <c r="D44" s="14">
+      <c r="D44">
         <f t="shared" ref="D44:D77" si="1">C44</f>
         <v>2</v>
       </c>
@@ -8187,7 +8742,7 @@
       <c r="C45">
         <v>3</v>
       </c>
-      <c r="D45" s="14">
+      <c r="D45">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -8206,7 +8761,7 @@
       <c r="C46">
         <v>4</v>
       </c>
-      <c r="D46" s="14">
+      <c r="D46">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
@@ -8225,7 +8780,7 @@
       <c r="C47">
         <v>5</v>
       </c>
-      <c r="D47" s="14">
+      <c r="D47">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
@@ -8244,7 +8799,7 @@
       <c r="C48">
         <v>6</v>
       </c>
-      <c r="D48" s="14">
+      <c r="D48">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
@@ -8263,7 +8818,7 @@
       <c r="C49">
         <v>7</v>
       </c>
-      <c r="D49" s="14">
+      <c r="D49">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -8282,7 +8837,7 @@
       <c r="C50">
         <v>8</v>
       </c>
-      <c r="D50" s="14">
+      <c r="D50">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -8301,7 +8856,7 @@
       <c r="C51">
         <v>9</v>
       </c>
-      <c r="D51" s="14">
+      <c r="D51">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
@@ -8320,7 +8875,7 @@
       <c r="C52">
         <v>10</v>
       </c>
-      <c r="D52" s="14">
+      <c r="D52">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
@@ -8339,7 +8894,7 @@
       <c r="C53">
         <v>11</v>
       </c>
-      <c r="D53" s="14">
+      <c r="D53">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
@@ -8358,7 +8913,7 @@
       <c r="C54">
         <v>12</v>
       </c>
-      <c r="D54" s="14">
+      <c r="D54">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
@@ -8377,7 +8932,7 @@
       <c r="C55">
         <v>13</v>
       </c>
-      <c r="D55" s="14">
+      <c r="D55">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
@@ -8396,7 +8951,7 @@
       <c r="C56">
         <v>14</v>
       </c>
-      <c r="D56" s="14">
+      <c r="D56">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
@@ -8415,7 +8970,7 @@
       <c r="C57">
         <v>15</v>
       </c>
-      <c r="D57" s="14">
+      <c r="D57">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
@@ -8434,7 +8989,7 @@
       <c r="C58">
         <v>16</v>
       </c>
-      <c r="D58" s="14">
+      <c r="D58">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
@@ -8453,7 +9008,7 @@
       <c r="C59">
         <v>17</v>
       </c>
-      <c r="D59" s="14">
+      <c r="D59">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
@@ -8472,7 +9027,7 @@
       <c r="C60">
         <v>18</v>
       </c>
-      <c r="D60" s="14">
+      <c r="D60">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
@@ -8491,7 +9046,7 @@
       <c r="C61">
         <v>19</v>
       </c>
-      <c r="D61" s="14">
+      <c r="D61">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
@@ -8510,7 +9065,7 @@
       <c r="C62">
         <v>20</v>
       </c>
-      <c r="D62" s="14">
+      <c r="D62">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
@@ -8529,7 +9084,7 @@
       <c r="C63">
         <v>21</v>
       </c>
-      <c r="D63" s="14">
+      <c r="D63">
         <f t="shared" si="1"/>
         <v>21</v>
       </c>
@@ -8548,7 +9103,7 @@
       <c r="C64">
         <v>22</v>
       </c>
-      <c r="D64" s="14">
+      <c r="D64">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
@@ -8567,7 +9122,7 @@
       <c r="C65">
         <v>23</v>
       </c>
-      <c r="D65" s="14">
+      <c r="D65">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
@@ -8586,7 +9141,7 @@
       <c r="C66">
         <v>24</v>
       </c>
-      <c r="D66" s="14">
+      <c r="D66">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
@@ -8605,7 +9160,7 @@
       <c r="C67">
         <v>25</v>
       </c>
-      <c r="D67" s="14">
+      <c r="D67">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
@@ -8624,7 +9179,7 @@
       <c r="C68">
         <v>1</v>
       </c>
-      <c r="D68" s="14">
+      <c r="D68">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
@@ -8643,7 +9198,7 @@
       <c r="C69">
         <v>2</v>
       </c>
-      <c r="D69" s="14">
+      <c r="D69">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
@@ -8662,7 +9217,7 @@
       <c r="C70">
         <v>3</v>
       </c>
-      <c r="D70" s="14">
+      <c r="D70">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -8681,7 +9236,7 @@
       <c r="C71">
         <v>4</v>
       </c>
-      <c r="D71" s="14">
+      <c r="D71">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
@@ -8700,7 +9255,7 @@
       <c r="C72">
         <v>5</v>
       </c>
-      <c r="D72" s="14">
+      <c r="D72">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
@@ -8719,7 +9274,7 @@
       <c r="C73">
         <v>6</v>
       </c>
-      <c r="D73" s="14">
+      <c r="D73">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
@@ -8738,7 +9293,7 @@
       <c r="C74">
         <v>7</v>
       </c>
-      <c r="D74" s="14">
+      <c r="D74">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -8757,7 +9312,7 @@
       <c r="C75">
         <v>8</v>
       </c>
-      <c r="D75" s="14">
+      <c r="D75">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -8776,7 +9331,7 @@
       <c r="C76">
         <v>9</v>
       </c>
-      <c r="D76" s="14">
+      <c r="D76">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
@@ -8795,7 +9350,7 @@
       <c r="C77">
         <v>10</v>
       </c>
-      <c r="D77" s="14">
+      <c r="D77">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
@@ -8814,7 +9369,7 @@
       <c r="C78">
         <v>11</v>
       </c>
-      <c r="D78" s="14" t="s">
+      <c r="D78" t="s">
         <v>84</v>
       </c>
       <c r="E78">
@@ -8832,7 +9387,7 @@
       <c r="C79">
         <v>1</v>
       </c>
-      <c r="D79" s="14" t="s">
+      <c r="D79" t="s">
         <v>88</v>
       </c>
       <c r="E79">
@@ -8850,7 +9405,7 @@
       <c r="C80">
         <v>2</v>
       </c>
-      <c r="D80" s="14" t="s">
+      <c r="D80" t="s">
         <v>89</v>
       </c>
       <c r="E80">
@@ -8869,7 +9424,7 @@
         <f>C80+1</f>
         <v>3</v>
       </c>
-      <c r="D81" s="14" t="s">
+      <c r="D81" t="s">
         <v>90</v>
       </c>
       <c r="E81">
@@ -8888,7 +9443,7 @@
         <f t="shared" ref="C82:C93" si="3">C81+1</f>
         <v>4</v>
       </c>
-      <c r="D82" s="14" t="s">
+      <c r="D82" t="s">
         <v>91</v>
       </c>
       <c r="E82">
@@ -8907,7 +9462,7 @@
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="D83" s="14" t="s">
+      <c r="D83" t="s">
         <v>92</v>
       </c>
       <c r="E83">
@@ -8926,7 +9481,7 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="D84" s="14" t="s">
+      <c r="D84" t="s">
         <v>93</v>
       </c>
       <c r="E84">
@@ -8945,7 +9500,7 @@
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
-      <c r="D85" s="14" t="s">
+      <c r="D85" t="s">
         <v>94</v>
       </c>
       <c r="E85">
@@ -8964,7 +9519,7 @@
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="D86" s="14" t="s">
+      <c r="D86" t="s">
         <v>95</v>
       </c>
       <c r="E86">
@@ -8983,7 +9538,7 @@
         <f t="shared" si="3"/>
         <v>9</v>
       </c>
-      <c r="D87" s="14" t="s">
+      <c r="D87" t="s">
         <v>96</v>
       </c>
       <c r="E87">
@@ -9002,7 +9557,7 @@
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="D88" s="14" t="s">
+      <c r="D88" t="s">
         <v>97</v>
       </c>
       <c r="E88">
@@ -9021,7 +9576,7 @@
         <f t="shared" si="3"/>
         <v>11</v>
       </c>
-      <c r="D89" s="14" t="s">
+      <c r="D89" t="s">
         <v>98</v>
       </c>
       <c r="E89">
@@ -9040,7 +9595,7 @@
         <f t="shared" si="3"/>
         <v>12</v>
       </c>
-      <c r="D90" s="14" t="s">
+      <c r="D90" t="s">
         <v>99</v>
       </c>
       <c r="E90">
@@ -9059,7 +9614,7 @@
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="D91" s="14" t="s">
+      <c r="D91" t="s">
         <v>100</v>
       </c>
       <c r="E91">
@@ -9078,7 +9633,7 @@
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="D92" s="14" t="s">
+      <c r="D92" t="s">
         <v>101</v>
       </c>
       <c r="E92">
@@ -9097,7 +9652,7 @@
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="D93" s="14" t="s">
+      <c r="D93" t="s">
         <v>102</v>
       </c>
       <c r="E93">
@@ -9115,7 +9670,7 @@
       <c r="C94">
         <v>1</v>
       </c>
-      <c r="D94" s="14">
+      <c r="D94">
         <f>C94</f>
         <v>1</v>
       </c>
@@ -9134,7 +9689,7 @@
       <c r="C95">
         <v>2</v>
       </c>
-      <c r="D95" s="14">
+      <c r="D95">
         <f t="shared" ref="D95:D112" si="4">C95</f>
         <v>2</v>
       </c>
@@ -9154,7 +9709,7 @@
         <f>C95+1</f>
         <v>3</v>
       </c>
-      <c r="D96" s="14">
+      <c r="D96">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
@@ -9174,7 +9729,7 @@
         <f t="shared" ref="C97:C112" si="5">C96+1</f>
         <v>4</v>
       </c>
-      <c r="D97" s="14">
+      <c r="D97">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
@@ -9194,7 +9749,7 @@
         <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="D98" s="14">
+      <c r="D98">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
@@ -9214,7 +9769,7 @@
         <f t="shared" si="5"/>
         <v>6</v>
       </c>
-      <c r="D99" s="14">
+      <c r="D99">
         <f t="shared" si="4"/>
         <v>6</v>
       </c>
@@ -9234,7 +9789,7 @@
         <f t="shared" si="5"/>
         <v>7</v>
       </c>
-      <c r="D100" s="14">
+      <c r="D100">
         <f t="shared" si="4"/>
         <v>7</v>
       </c>
@@ -9254,7 +9809,7 @@
         <f t="shared" si="5"/>
         <v>8</v>
       </c>
-      <c r="D101" s="14">
+      <c r="D101">
         <f t="shared" si="4"/>
         <v>8</v>
       </c>
@@ -9274,7 +9829,7 @@
         <f t="shared" si="5"/>
         <v>9</v>
       </c>
-      <c r="D102" s="14">
+      <c r="D102">
         <f t="shared" si="4"/>
         <v>9</v>
       </c>
@@ -9294,7 +9849,7 @@
         <f t="shared" si="5"/>
         <v>10</v>
       </c>
-      <c r="D103" s="14">
+      <c r="D103">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
@@ -9314,7 +9869,7 @@
         <f>C103+1</f>
         <v>11</v>
       </c>
-      <c r="D104" s="14">
+      <c r="D104">
         <f t="shared" si="4"/>
         <v>11</v>
       </c>
@@ -9334,7 +9889,7 @@
         <f t="shared" si="5"/>
         <v>12</v>
       </c>
-      <c r="D105" s="14">
+      <c r="D105">
         <f t="shared" si="4"/>
         <v>12</v>
       </c>
@@ -9354,7 +9909,7 @@
         <f t="shared" si="5"/>
         <v>13</v>
       </c>
-      <c r="D106" s="14">
+      <c r="D106">
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
@@ -9374,7 +9929,7 @@
         <f t="shared" si="5"/>
         <v>14</v>
       </c>
-      <c r="D107" s="14">
+      <c r="D107">
         <f t="shared" si="4"/>
         <v>14</v>
       </c>
@@ -9394,7 +9949,7 @@
         <f t="shared" si="5"/>
         <v>15</v>
       </c>
-      <c r="D108" s="14">
+      <c r="D108">
         <f t="shared" si="4"/>
         <v>15</v>
       </c>
@@ -9414,7 +9969,7 @@
         <f t="shared" si="5"/>
         <v>16</v>
       </c>
-      <c r="D109" s="14">
+      <c r="D109">
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
@@ -9434,7 +9989,7 @@
         <f>C109+1</f>
         <v>17</v>
       </c>
-      <c r="D110" s="14">
+      <c r="D110">
         <f t="shared" si="4"/>
         <v>17</v>
       </c>
@@ -9454,7 +10009,7 @@
         <f t="shared" si="5"/>
         <v>18</v>
       </c>
-      <c r="D111" s="14">
+      <c r="D111">
         <f t="shared" si="4"/>
         <v>18</v>
       </c>
@@ -9474,7 +10029,7 @@
         <f t="shared" si="5"/>
         <v>19</v>
       </c>
-      <c r="D112" s="14">
+      <c r="D112">
         <f t="shared" si="4"/>
         <v>19</v>
       </c>
@@ -9493,7 +10048,7 @@
       <c r="C113">
         <v>1</v>
       </c>
-      <c r="D113" s="14" t="s">
+      <c r="D113" t="s">
         <v>109</v>
       </c>
       <c r="E113">
@@ -9512,7 +10067,7 @@
         <f>C113+1</f>
         <v>2</v>
       </c>
-      <c r="D114" s="14" t="s">
+      <c r="D114" t="s">
         <v>110</v>
       </c>
       <c r="E114">
@@ -9531,7 +10086,7 @@
         <f t="shared" ref="C115:C131" si="6">C114+1</f>
         <v>3</v>
       </c>
-      <c r="D115" s="14" t="s">
+      <c r="D115" t="s">
         <v>29</v>
       </c>
       <c r="E115">
@@ -9550,7 +10105,7 @@
         <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="D116" s="14" t="s">
+      <c r="D116" t="s">
         <v>111</v>
       </c>
       <c r="E116">
@@ -9569,7 +10124,7 @@
         <f t="shared" si="6"/>
         <v>5</v>
       </c>
-      <c r="D117" s="14" t="s">
+      <c r="D117" t="s">
         <v>112</v>
       </c>
       <c r="E117">
@@ -9588,7 +10143,7 @@
         <f t="shared" si="6"/>
         <v>6</v>
       </c>
-      <c r="D118" s="14" t="s">
+      <c r="D118" t="s">
         <v>113</v>
       </c>
       <c r="E118">
@@ -9607,7 +10162,7 @@
         <f t="shared" si="6"/>
         <v>7</v>
       </c>
-      <c r="D119" s="14" t="s">
+      <c r="D119" t="s">
         <v>114</v>
       </c>
       <c r="E119">
@@ -9626,7 +10181,7 @@
         <f t="shared" si="6"/>
         <v>8</v>
       </c>
-      <c r="D120" s="14" t="s">
+      <c r="D120" t="s">
         <v>115</v>
       </c>
       <c r="E120">
@@ -9645,7 +10200,7 @@
         <f t="shared" si="6"/>
         <v>9</v>
       </c>
-      <c r="D121" s="14" t="s">
+      <c r="D121" t="s">
         <v>116</v>
       </c>
       <c r="E121">
@@ -9664,7 +10219,7 @@
         <f t="shared" si="6"/>
         <v>10</v>
       </c>
-      <c r="D122" s="14" t="s">
+      <c r="D122" t="s">
         <v>117</v>
       </c>
       <c r="E122">
@@ -9683,7 +10238,7 @@
         <f t="shared" si="6"/>
         <v>11</v>
       </c>
-      <c r="D123" s="14" t="s">
+      <c r="D123" t="s">
         <v>118</v>
       </c>
       <c r="E123">
@@ -9702,7 +10257,7 @@
         <f t="shared" si="6"/>
         <v>12</v>
       </c>
-      <c r="D124" s="14" t="s">
+      <c r="D124" t="s">
         <v>119</v>
       </c>
       <c r="E124">
@@ -9721,7 +10276,7 @@
         <f t="shared" si="6"/>
         <v>13</v>
       </c>
-      <c r="D125" s="14" t="s">
+      <c r="D125" t="s">
         <v>120</v>
       </c>
       <c r="E125">
@@ -9740,7 +10295,7 @@
         <f t="shared" si="6"/>
         <v>14</v>
       </c>
-      <c r="D126" s="14" t="s">
+      <c r="D126" t="s">
         <v>126</v>
       </c>
       <c r="E126">
@@ -9759,7 +10314,7 @@
         <f t="shared" si="6"/>
         <v>15</v>
       </c>
-      <c r="D127" s="14" t="s">
+      <c r="D127" t="s">
         <v>121</v>
       </c>
       <c r="E127">
@@ -9778,7 +10333,7 @@
         <f t="shared" si="6"/>
         <v>16</v>
       </c>
-      <c r="D128" s="14" t="s">
+      <c r="D128" t="s">
         <v>122</v>
       </c>
       <c r="E128">
@@ -9797,7 +10352,7 @@
         <f t="shared" si="6"/>
         <v>17</v>
       </c>
-      <c r="D129" s="14" t="s">
+      <c r="D129" t="s">
         <v>123</v>
       </c>
       <c r="E129">
@@ -9816,7 +10371,7 @@
         <f t="shared" si="6"/>
         <v>18</v>
       </c>
-      <c r="D130" s="14" t="s">
+      <c r="D130" t="s">
         <v>124</v>
       </c>
       <c r="E130">
@@ -9835,7 +10390,7 @@
         <f t="shared" si="6"/>
         <v>19</v>
       </c>
-      <c r="D131" s="14" t="s">
+      <c r="D131" t="s">
         <v>125</v>
       </c>
       <c r="E131">
@@ -9853,7 +10408,7 @@
       <c r="C132">
         <v>1</v>
       </c>
-      <c r="D132" s="14" t="s">
+      <c r="D132" t="s">
         <v>131</v>
       </c>
       <c r="E132">
@@ -9871,7 +10426,7 @@
       <c r="C133">
         <v>2</v>
       </c>
-      <c r="D133" s="14" t="s">
+      <c r="D133" t="s">
         <v>132</v>
       </c>
       <c r="E133">
@@ -9889,7 +10444,7 @@
       <c r="C134">
         <v>3</v>
       </c>
-      <c r="D134" s="14" t="s">
+      <c r="D134" t="s">
         <v>133</v>
       </c>
       <c r="E134">
@@ -9907,7 +10462,7 @@
       <c r="C135">
         <v>4</v>
       </c>
-      <c r="D135" s="14" t="s">
+      <c r="D135" t="s">
         <v>134</v>
       </c>
       <c r="E135">
@@ -9925,7 +10480,7 @@
       <c r="C136">
         <v>5</v>
       </c>
-      <c r="D136" s="14" t="s">
+      <c r="D136" t="s">
         <v>135</v>
       </c>
       <c r="E136">
@@ -9943,7 +10498,7 @@
       <c r="C137">
         <v>1</v>
       </c>
-      <c r="D137" s="14">
+      <c r="D137">
         <f>C137</f>
         <v>1</v>
       </c>
@@ -9963,7 +10518,7 @@
         <f>C137+1</f>
         <v>2</v>
       </c>
-      <c r="D138" s="14">
+      <c r="D138">
         <f t="shared" ref="D138:D159" si="8">C138</f>
         <v>2</v>
       </c>
@@ -9983,7 +10538,7 @@
         <f t="shared" ref="C139:C159" si="9">C138+1</f>
         <v>3</v>
       </c>
-      <c r="D139" s="14">
+      <c r="D139">
         <f t="shared" si="8"/>
         <v>3</v>
       </c>
@@ -10003,7 +10558,7 @@
         <f t="shared" si="9"/>
         <v>4</v>
       </c>
-      <c r="D140" s="14">
+      <c r="D140">
         <f t="shared" si="8"/>
         <v>4</v>
       </c>
@@ -10023,7 +10578,7 @@
         <f t="shared" si="9"/>
         <v>5</v>
       </c>
-      <c r="D141" s="14">
+      <c r="D141">
         <f t="shared" si="8"/>
         <v>5</v>
       </c>
@@ -10043,7 +10598,7 @@
         <f t="shared" si="9"/>
         <v>6</v>
       </c>
-      <c r="D142" s="14">
+      <c r="D142">
         <f t="shared" si="8"/>
         <v>6</v>
       </c>
@@ -10063,7 +10618,7 @@
         <f t="shared" si="9"/>
         <v>7</v>
       </c>
-      <c r="D143" s="14">
+      <c r="D143">
         <f t="shared" si="8"/>
         <v>7</v>
       </c>
@@ -10083,7 +10638,7 @@
         <f t="shared" si="9"/>
         <v>8</v>
       </c>
-      <c r="D144" s="14">
+      <c r="D144">
         <f t="shared" si="8"/>
         <v>8</v>
       </c>
@@ -10103,7 +10658,7 @@
         <f t="shared" si="9"/>
         <v>9</v>
       </c>
-      <c r="D145" s="14">
+      <c r="D145">
         <f t="shared" si="8"/>
         <v>9</v>
       </c>
@@ -10123,7 +10678,7 @@
         <f t="shared" si="9"/>
         <v>10</v>
       </c>
-      <c r="D146" s="14">
+      <c r="D146">
         <f t="shared" si="8"/>
         <v>10</v>
       </c>
@@ -10143,7 +10698,7 @@
         <f t="shared" si="9"/>
         <v>11</v>
       </c>
-      <c r="D147" s="14">
+      <c r="D147">
         <f t="shared" si="8"/>
         <v>11</v>
       </c>
@@ -10163,7 +10718,7 @@
         <f t="shared" si="9"/>
         <v>12</v>
       </c>
-      <c r="D148" s="14">
+      <c r="D148">
         <f t="shared" si="8"/>
         <v>12</v>
       </c>
@@ -10183,7 +10738,7 @@
         <f t="shared" si="9"/>
         <v>13</v>
       </c>
-      <c r="D149" s="14">
+      <c r="D149">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
@@ -10203,7 +10758,7 @@
         <f t="shared" si="9"/>
         <v>14</v>
       </c>
-      <c r="D150" s="14">
+      <c r="D150">
         <f t="shared" si="8"/>
         <v>14</v>
       </c>
@@ -10223,7 +10778,7 @@
         <f t="shared" si="9"/>
         <v>15</v>
       </c>
-      <c r="D151" s="14">
+      <c r="D151">
         <f t="shared" si="8"/>
         <v>15</v>
       </c>
@@ -10243,7 +10798,7 @@
         <f t="shared" si="9"/>
         <v>16</v>
       </c>
-      <c r="D152" s="14">
+      <c r="D152">
         <f t="shared" si="8"/>
         <v>16</v>
       </c>
@@ -10263,7 +10818,7 @@
         <f t="shared" si="9"/>
         <v>17</v>
       </c>
-      <c r="D153" s="14">
+      <c r="D153">
         <f t="shared" si="8"/>
         <v>17</v>
       </c>
@@ -10283,7 +10838,7 @@
         <f t="shared" si="9"/>
         <v>18</v>
       </c>
-      <c r="D154" s="14">
+      <c r="D154">
         <f t="shared" si="8"/>
         <v>18</v>
       </c>
@@ -10303,7 +10858,7 @@
         <f t="shared" si="9"/>
         <v>19</v>
       </c>
-      <c r="D155" s="14">
+      <c r="D155">
         <f t="shared" si="8"/>
         <v>19</v>
       </c>
@@ -10323,7 +10878,7 @@
         <f t="shared" si="9"/>
         <v>20</v>
       </c>
-      <c r="D156" s="14">
+      <c r="D156">
         <f t="shared" si="8"/>
         <v>20</v>
       </c>
@@ -10343,7 +10898,7 @@
         <f t="shared" si="9"/>
         <v>21</v>
       </c>
-      <c r="D157" s="14">
+      <c r="D157">
         <f t="shared" si="8"/>
         <v>21</v>
       </c>
@@ -10363,7 +10918,7 @@
         <f t="shared" si="9"/>
         <v>22</v>
       </c>
-      <c r="D158" s="14">
+      <c r="D158">
         <f t="shared" si="8"/>
         <v>22</v>
       </c>
@@ -10383,7 +10938,7 @@
         <f t="shared" si="9"/>
         <v>23</v>
       </c>
-      <c r="D159" s="14">
+      <c r="D159">
         <f t="shared" si="8"/>
         <v>23</v>
       </c>
@@ -10402,7 +10957,7 @@
       <c r="C160">
         <v>24</v>
       </c>
-      <c r="D160" s="14" t="s">
+      <c r="D160" t="s">
         <v>135</v>
       </c>
       <c r="E160">
@@ -10420,7 +10975,7 @@
       <c r="C161">
         <v>1</v>
       </c>
-      <c r="D161" s="14" t="s">
+      <c r="D161" t="s">
         <v>148</v>
       </c>
       <c r="E161">
@@ -10438,7 +10993,7 @@
       <c r="C162">
         <v>2</v>
       </c>
-      <c r="D162" s="14" t="s">
+      <c r="D162" t="s">
         <v>149</v>
       </c>
       <c r="E162">
@@ -10456,7 +11011,7 @@
       <c r="C163">
         <v>3</v>
       </c>
-      <c r="D163" s="14" t="s">
+      <c r="D163" t="s">
         <v>150</v>
       </c>
       <c r="E163">
@@ -10474,7 +11029,7 @@
       <c r="C164">
         <v>4</v>
       </c>
-      <c r="D164" s="14" t="s">
+      <c r="D164" t="s">
         <v>151</v>
       </c>
       <c r="E164">
@@ -10492,7 +11047,7 @@
       <c r="C165">
         <v>5</v>
       </c>
-      <c r="D165" s="14" t="s">
+      <c r="D165" t="s">
         <v>152</v>
       </c>
       <c r="E165">
@@ -10510,7 +11065,7 @@
       <c r="C166">
         <v>6</v>
       </c>
-      <c r="D166" s="14" t="s">
+      <c r="D166" t="s">
         <v>153</v>
       </c>
       <c r="E166">
@@ -10528,7 +11083,7 @@
       <c r="C167">
         <v>7</v>
       </c>
-      <c r="D167" s="14" t="s">
+      <c r="D167" t="s">
         <v>154</v>
       </c>
       <c r="E167">
@@ -10546,7 +11101,7 @@
       <c r="C168">
         <v>1</v>
       </c>
-      <c r="D168" s="14" t="s">
+      <c r="D168" t="s">
         <v>157</v>
       </c>
       <c r="E168">
@@ -10565,7 +11120,7 @@
         <f>C168+1</f>
         <v>2</v>
       </c>
-      <c r="D169" s="14" t="s">
+      <c r="D169" t="s">
         <v>158</v>
       </c>
       <c r="E169">
@@ -10584,7 +11139,7 @@
         <f t="shared" ref="C170:C212" si="10">C169+1</f>
         <v>3</v>
       </c>
-      <c r="D170" s="14" t="s">
+      <c r="D170" t="s">
         <v>159</v>
       </c>
       <c r="E170">
@@ -10603,7 +11158,7 @@
         <f t="shared" si="10"/>
         <v>4</v>
       </c>
-      <c r="D171" s="14" t="s">
+      <c r="D171" t="s">
         <v>160</v>
       </c>
       <c r="E171">
@@ -10622,7 +11177,7 @@
         <f t="shared" si="10"/>
         <v>5</v>
       </c>
-      <c r="D172" s="14" t="s">
+      <c r="D172" t="s">
         <v>161</v>
       </c>
       <c r="E172">
@@ -10641,7 +11196,7 @@
         <f t="shared" si="10"/>
         <v>6</v>
       </c>
-      <c r="D173" s="14" t="s">
+      <c r="D173" t="s">
         <v>162</v>
       </c>
       <c r="E173">
@@ -10660,7 +11215,7 @@
         <f t="shared" si="10"/>
         <v>7</v>
       </c>
-      <c r="D174" s="14" t="s">
+      <c r="D174" t="s">
         <v>163</v>
       </c>
       <c r="E174">
@@ -10679,7 +11234,7 @@
         <f t="shared" si="10"/>
         <v>8</v>
       </c>
-      <c r="D175" s="14" t="s">
+      <c r="D175" t="s">
         <v>164</v>
       </c>
       <c r="E175">
@@ -10698,7 +11253,7 @@
         <f t="shared" si="10"/>
         <v>9</v>
       </c>
-      <c r="D176" s="14" t="s">
+      <c r="D176" t="s">
         <v>165</v>
       </c>
       <c r="E176">
@@ -10717,7 +11272,7 @@
         <f t="shared" si="10"/>
         <v>10</v>
       </c>
-      <c r="D177" s="14" t="s">
+      <c r="D177" t="s">
         <v>166</v>
       </c>
       <c r="E177">
@@ -10736,7 +11291,7 @@
         <f t="shared" si="10"/>
         <v>11</v>
       </c>
-      <c r="D178" s="14" t="s">
+      <c r="D178" t="s">
         <v>167</v>
       </c>
       <c r="E178">
@@ -10755,7 +11310,7 @@
         <f t="shared" si="10"/>
         <v>12</v>
       </c>
-      <c r="D179" s="14" t="s">
+      <c r="D179" t="s">
         <v>168</v>
       </c>
       <c r="E179">
@@ -10774,7 +11329,7 @@
         <f t="shared" si="10"/>
         <v>13</v>
       </c>
-      <c r="D180" s="14" t="s">
+      <c r="D180" t="s">
         <v>169</v>
       </c>
       <c r="E180">
@@ -10793,7 +11348,7 @@
         <f t="shared" si="10"/>
         <v>14</v>
       </c>
-      <c r="D181" s="14" t="s">
+      <c r="D181" t="s">
         <v>170</v>
       </c>
       <c r="E181">
@@ -10812,7 +11367,7 @@
         <f t="shared" si="10"/>
         <v>15</v>
       </c>
-      <c r="D182" s="14" t="s">
+      <c r="D182" t="s">
         <v>171</v>
       </c>
       <c r="E182">
@@ -10831,7 +11386,7 @@
         <f t="shared" si="10"/>
         <v>16</v>
       </c>
-      <c r="D183" s="14" t="s">
+      <c r="D183" t="s">
         <v>172</v>
       </c>
       <c r="E183">
@@ -10850,7 +11405,7 @@
         <f t="shared" si="10"/>
         <v>17</v>
       </c>
-      <c r="D184" s="14" t="s">
+      <c r="D184" t="s">
         <v>173</v>
       </c>
       <c r="E184">
@@ -10869,7 +11424,7 @@
         <f t="shared" si="10"/>
         <v>18</v>
       </c>
-      <c r="D185" s="14" t="s">
+      <c r="D185" t="s">
         <v>174</v>
       </c>
       <c r="E185">
@@ -10888,7 +11443,7 @@
         <f t="shared" si="10"/>
         <v>19</v>
       </c>
-      <c r="D186" s="14" t="s">
+      <c r="D186" t="s">
         <v>175</v>
       </c>
       <c r="E186">
@@ -10907,7 +11462,7 @@
         <f t="shared" si="10"/>
         <v>20</v>
       </c>
-      <c r="D187" s="14" t="s">
+      <c r="D187" t="s">
         <v>176</v>
       </c>
       <c r="E187">
@@ -10926,7 +11481,7 @@
         <f t="shared" si="10"/>
         <v>21</v>
       </c>
-      <c r="D188" s="14" t="s">
+      <c r="D188" t="s">
         <v>178</v>
       </c>
       <c r="E188">
@@ -10945,7 +11500,7 @@
         <f t="shared" si="10"/>
         <v>22</v>
       </c>
-      <c r="D189" s="14" t="s">
+      <c r="D189" t="s">
         <v>177</v>
       </c>
       <c r="E189">
@@ -10964,7 +11519,7 @@
         <f t="shared" si="10"/>
         <v>23</v>
       </c>
-      <c r="D190" s="14" t="s">
+      <c r="D190" t="s">
         <v>179</v>
       </c>
       <c r="E190">
@@ -10983,7 +11538,7 @@
         <f t="shared" si="10"/>
         <v>24</v>
       </c>
-      <c r="D191" s="14" t="s">
+      <c r="D191" t="s">
         <v>180</v>
       </c>
       <c r="E191">
@@ -11002,7 +11557,7 @@
         <f t="shared" si="10"/>
         <v>25</v>
       </c>
-      <c r="D192" s="14" t="s">
+      <c r="D192" t="s">
         <v>181</v>
       </c>
       <c r="E192">
@@ -11021,7 +11576,7 @@
         <f t="shared" si="10"/>
         <v>26</v>
       </c>
-      <c r="D193" s="14" t="s">
+      <c r="D193" t="s">
         <v>182</v>
       </c>
       <c r="E193">
@@ -11040,7 +11595,7 @@
         <f t="shared" si="10"/>
         <v>27</v>
       </c>
-      <c r="D194" s="14" t="s">
+      <c r="D194" t="s">
         <v>183</v>
       </c>
       <c r="E194">
@@ -11049,7 +11604,7 @@
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A195">
-        <f t="shared" ref="A195:A233" si="11" xml:space="preserve"> ROW() -1</f>
+        <f t="shared" ref="A195:A236" si="11" xml:space="preserve"> ROW() -1</f>
         <v>194</v>
       </c>
       <c r="B195">
@@ -11059,7 +11614,7 @@
         <f t="shared" si="10"/>
         <v>28</v>
       </c>
-      <c r="D195" s="14" t="s">
+      <c r="D195" t="s">
         <v>184</v>
       </c>
       <c r="E195">
@@ -11078,7 +11633,7 @@
         <f t="shared" si="10"/>
         <v>29</v>
       </c>
-      <c r="D196" s="14" t="s">
+      <c r="D196" t="s">
         <v>185</v>
       </c>
       <c r="E196">
@@ -11097,7 +11652,7 @@
         <f t="shared" si="10"/>
         <v>30</v>
       </c>
-      <c r="D197" s="14" t="s">
+      <c r="D197" t="s">
         <v>186</v>
       </c>
       <c r="E197">
@@ -11116,7 +11671,7 @@
         <f t="shared" si="10"/>
         <v>31</v>
       </c>
-      <c r="D198" s="14" t="s">
+      <c r="D198" t="s">
         <v>187</v>
       </c>
       <c r="E198">
@@ -11135,7 +11690,7 @@
         <f t="shared" si="10"/>
         <v>32</v>
       </c>
-      <c r="D199" s="14" t="s">
+      <c r="D199" t="s">
         <v>188</v>
       </c>
       <c r="E199">
@@ -11154,7 +11709,7 @@
         <f t="shared" si="10"/>
         <v>33</v>
       </c>
-      <c r="D200" s="14" t="s">
+      <c r="D200" t="s">
         <v>189</v>
       </c>
       <c r="E200">
@@ -11173,7 +11728,7 @@
         <f t="shared" si="10"/>
         <v>34</v>
       </c>
-      <c r="D201" s="14" t="s">
+      <c r="D201" t="s">
         <v>190</v>
       </c>
       <c r="E201">
@@ -11192,7 +11747,7 @@
         <f t="shared" si="10"/>
         <v>35</v>
       </c>
-      <c r="D202" s="14" t="s">
+      <c r="D202" t="s">
         <v>191</v>
       </c>
       <c r="E202">
@@ -11211,7 +11766,7 @@
         <f t="shared" si="10"/>
         <v>36</v>
       </c>
-      <c r="D203" s="14" t="s">
+      <c r="D203" t="s">
         <v>192</v>
       </c>
       <c r="E203">
@@ -11230,7 +11785,7 @@
         <f t="shared" si="10"/>
         <v>37</v>
       </c>
-      <c r="D204" s="14" t="s">
+      <c r="D204" t="s">
         <v>193</v>
       </c>
       <c r="E204">
@@ -11249,7 +11804,7 @@
         <f t="shared" si="10"/>
         <v>38</v>
       </c>
-      <c r="D205" s="14" t="s">
+      <c r="D205" t="s">
         <v>194</v>
       </c>
       <c r="E205">
@@ -11268,7 +11823,7 @@
         <f t="shared" si="10"/>
         <v>39</v>
       </c>
-      <c r="D206" s="14" t="s">
+      <c r="D206" t="s">
         <v>195</v>
       </c>
       <c r="E206">
@@ -11287,7 +11842,7 @@
         <f t="shared" si="10"/>
         <v>40</v>
       </c>
-      <c r="D207" s="14" t="s">
+      <c r="D207" t="s">
         <v>196</v>
       </c>
       <c r="E207">
@@ -11306,7 +11861,7 @@
         <f t="shared" si="10"/>
         <v>41</v>
       </c>
-      <c r="D208" s="14" t="s">
+      <c r="D208" t="s">
         <v>197</v>
       </c>
       <c r="E208">
@@ -11325,7 +11880,7 @@
         <f t="shared" si="10"/>
         <v>42</v>
       </c>
-      <c r="D209" s="14" t="s">
+      <c r="D209" t="s">
         <v>198</v>
       </c>
       <c r="E209">
@@ -11344,7 +11899,7 @@
         <f t="shared" si="10"/>
         <v>43</v>
       </c>
-      <c r="D210" s="14" t="s">
+      <c r="D210" t="s">
         <v>199</v>
       </c>
       <c r="E210">
@@ -11363,7 +11918,7 @@
         <f t="shared" si="10"/>
         <v>44</v>
       </c>
-      <c r="D211" s="14" t="s">
+      <c r="D211" t="s">
         <v>201</v>
       </c>
       <c r="E211">
@@ -11382,7 +11937,7 @@
         <f t="shared" si="10"/>
         <v>45</v>
       </c>
-      <c r="D212" s="14" t="s">
+      <c r="D212" t="s">
         <v>200</v>
       </c>
       <c r="E212">
@@ -11400,7 +11955,7 @@
       <c r="C213">
         <v>1</v>
       </c>
-      <c r="D213" s="14" t="s">
+      <c r="D213" t="s">
         <v>207</v>
       </c>
       <c r="E213">
@@ -11419,7 +11974,7 @@
         <f>C213+1</f>
         <v>2</v>
       </c>
-      <c r="D214" s="14">
+      <c r="D214">
         <v>1</v>
       </c>
       <c r="E214">
@@ -11438,7 +11993,7 @@
         <f t="shared" ref="C215:C225" si="12">C214+1</f>
         <v>3</v>
       </c>
-      <c r="D215" s="14">
+      <c r="D215">
         <v>2</v>
       </c>
       <c r="E215">
@@ -11457,7 +12012,7 @@
         <f t="shared" si="12"/>
         <v>4</v>
       </c>
-      <c r="D216" s="14">
+      <c r="D216">
         <v>3</v>
       </c>
       <c r="E216">
@@ -11476,7 +12031,7 @@
         <f t="shared" si="12"/>
         <v>5</v>
       </c>
-      <c r="D217" s="14">
+      <c r="D217">
         <v>4</v>
       </c>
       <c r="E217">
@@ -11495,7 +12050,7 @@
         <f t="shared" si="12"/>
         <v>6</v>
       </c>
-      <c r="D218" s="14">
+      <c r="D218">
         <v>5</v>
       </c>
       <c r="E218">
@@ -11514,7 +12069,7 @@
         <f t="shared" si="12"/>
         <v>7</v>
       </c>
-      <c r="D219" s="14">
+      <c r="D219">
         <v>6</v>
       </c>
       <c r="E219">
@@ -11533,7 +12088,7 @@
         <f t="shared" si="12"/>
         <v>8</v>
       </c>
-      <c r="D220" s="14">
+      <c r="D220">
         <v>7</v>
       </c>
       <c r="E220">
@@ -11552,7 +12107,7 @@
         <f t="shared" si="12"/>
         <v>9</v>
       </c>
-      <c r="D221" s="14">
+      <c r="D221">
         <v>8</v>
       </c>
       <c r="E221">
@@ -11571,7 +12126,7 @@
         <f t="shared" si="12"/>
         <v>10</v>
       </c>
-      <c r="D222" s="14">
+      <c r="D222">
         <v>9</v>
       </c>
       <c r="E222">
@@ -11590,7 +12145,7 @@
         <f t="shared" si="12"/>
         <v>11</v>
       </c>
-      <c r="D223" s="14">
+      <c r="D223">
         <v>10</v>
       </c>
       <c r="E223">
@@ -11609,7 +12164,7 @@
         <f t="shared" si="12"/>
         <v>12</v>
       </c>
-      <c r="D224" s="14">
+      <c r="D224">
         <v>11</v>
       </c>
       <c r="E224">
@@ -11628,7 +12183,7 @@
         <f t="shared" si="12"/>
         <v>13</v>
       </c>
-      <c r="D225" s="14">
+      <c r="D225">
         <v>12</v>
       </c>
       <c r="E225">
@@ -11646,7 +12201,7 @@
       <c r="C226">
         <v>1</v>
       </c>
-      <c r="D226" s="14">
+      <c r="D226">
         <f>C226</f>
         <v>1</v>
       </c>
@@ -11666,7 +12221,7 @@
         <f>C226+1</f>
         <v>2</v>
       </c>
-      <c r="D227" s="14">
+      <c r="D227">
         <f t="shared" ref="D227:D233" si="13">C227</f>
         <v>2</v>
       </c>
@@ -11686,7 +12241,7 @@
         <f t="shared" ref="C228:C233" si="14">C227+1</f>
         <v>3</v>
       </c>
-      <c r="D228" s="14">
+      <c r="D228">
         <f t="shared" si="13"/>
         <v>3</v>
       </c>
@@ -11706,7 +12261,7 @@
         <f t="shared" si="14"/>
         <v>4</v>
       </c>
-      <c r="D229" s="14">
+      <c r="D229">
         <f t="shared" si="13"/>
         <v>4</v>
       </c>
@@ -11726,7 +12281,7 @@
         <f t="shared" si="14"/>
         <v>5</v>
       </c>
-      <c r="D230" s="14">
+      <c r="D230">
         <f t="shared" si="13"/>
         <v>5</v>
       </c>
@@ -11746,7 +12301,7 @@
         <f t="shared" si="14"/>
         <v>6</v>
       </c>
-      <c r="D231" s="14">
+      <c r="D231">
         <f t="shared" si="13"/>
         <v>6</v>
       </c>
@@ -11766,7 +12321,7 @@
         <f t="shared" si="14"/>
         <v>7</v>
       </c>
-      <c r="D232" s="14">
+      <c r="D232">
         <f t="shared" si="13"/>
         <v>7</v>
       </c>
@@ -11786,12 +12341,66 @@
         <f t="shared" si="14"/>
         <v>8</v>
       </c>
-      <c r="D233" s="14">
+      <c r="D233">
         <f t="shared" si="13"/>
         <v>8</v>
       </c>
       <c r="E233">
         <v>242</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A234">
+        <f t="shared" si="11"/>
+        <v>233</v>
+      </c>
+      <c r="B234">
+        <v>26</v>
+      </c>
+      <c r="C234">
+        <v>1</v>
+      </c>
+      <c r="D234" t="s">
+        <v>218</v>
+      </c>
+      <c r="E234">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A235">
+        <f t="shared" si="11"/>
+        <v>234</v>
+      </c>
+      <c r="B235">
+        <v>26</v>
+      </c>
+      <c r="C235">
+        <v>2</v>
+      </c>
+      <c r="D235" t="s">
+        <v>219</v>
+      </c>
+      <c r="E235">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A236">
+        <f t="shared" si="11"/>
+        <v>235</v>
+      </c>
+      <c r="B236">
+        <v>26</v>
+      </c>
+      <c r="C236">
+        <v>3</v>
+      </c>
+      <c r="D236" t="s">
+        <v>220</v>
+      </c>
+      <c r="E236">
+        <v>370</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data (Too Loud a Solitude & Crazy Genie)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/code/projects/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268B24E8-9E93-E442-A2CE-A39858E0DE56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48FAF91B-4635-C74F-A7BF-0F728429C49D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="15420" windowHeight="18980" activeTab="2" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="11880" yWindow="760" windowWidth="15440" windowHeight="19000" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="225">
   <si>
     <t>book_id</t>
   </si>
@@ -698,6 +698,18 @@
   </si>
   <si>
     <t>City of Illusions</t>
+  </si>
+  <si>
+    <t>Too Loud a Solitude</t>
+  </si>
+  <si>
+    <t>Crazy Genie</t>
+  </si>
+  <si>
+    <t>Bohumil Hrabal</t>
+  </si>
+  <si>
+    <t>Ines Cagnati</t>
   </si>
 </sst>
 </file>
@@ -1100,7 +1112,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -2148,6 +2160,82 @@
         <v>46220</v>
       </c>
     </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>221</v>
+      </c>
+      <c r="C28" t="s">
+        <v>223</v>
+      </c>
+      <c r="D28" t="s">
+        <v>62</v>
+      </c>
+      <c r="E28">
+        <v>1976</v>
+      </c>
+      <c r="F28" t="s">
+        <v>16</v>
+      </c>
+      <c r="G28">
+        <v>112</v>
+      </c>
+      <c r="H28" s="11">
+        <v>27148</v>
+      </c>
+      <c r="I28" t="s">
+        <v>104</v>
+      </c>
+      <c r="J28" t="s">
+        <v>67</v>
+      </c>
+      <c r="K28" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L28" s="7">
+        <v>46224</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>222</v>
+      </c>
+      <c r="C29" t="s">
+        <v>224</v>
+      </c>
+      <c r="D29" t="s">
+        <v>62</v>
+      </c>
+      <c r="E29">
+        <v>1976</v>
+      </c>
+      <c r="F29" t="s">
+        <v>16</v>
+      </c>
+      <c r="G29">
+        <v>151</v>
+      </c>
+      <c r="H29" s="11">
+        <v>38354</v>
+      </c>
+      <c r="I29" t="s">
+        <v>105</v>
+      </c>
+      <c r="J29" t="s">
+        <v>67</v>
+      </c>
+      <c r="K29" s="7">
+        <v>46224</v>
+      </c>
+      <c r="L29" s="7">
+        <v>46226</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2155,7 +2243,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I274"/>
+  <dimension ref="A1:I283"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -7587,7 +7675,7 @@
     </row>
     <row r="259" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A259">
-        <f t="shared" ref="A259:A274" si="4">ROW() - 1</f>
+        <f t="shared" ref="A259:A283" si="4">ROW() - 1</f>
         <v>258</v>
       </c>
       <c r="B259">
@@ -7919,6 +8007,195 @@
       </c>
       <c r="F274" s="6">
         <v>1.0717592592592593E-2</v>
+      </c>
+    </row>
+    <row r="275" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A275">
+        <f t="shared" si="4"/>
+        <v>274</v>
+      </c>
+      <c r="B275">
+        <v>27</v>
+      </c>
+      <c r="C275" s="3">
+        <v>46223.706250000003</v>
+      </c>
+      <c r="D275" t="s">
+        <v>63</v>
+      </c>
+      <c r="E275" t="s">
+        <v>63</v>
+      </c>
+      <c r="F275" s="6">
+        <v>2.0057870370370372E-2</v>
+      </c>
+    </row>
+    <row r="276" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A276">
+        <f t="shared" si="4"/>
+        <v>275</v>
+      </c>
+      <c r="B276">
+        <v>27</v>
+      </c>
+      <c r="C276" s="3">
+        <v>46223.802083333336</v>
+      </c>
+      <c r="D276" t="s">
+        <v>63</v>
+      </c>
+      <c r="E276" t="s">
+        <v>63</v>
+      </c>
+      <c r="F276" s="6">
+        <v>1.7627314814814814E-2</v>
+      </c>
+    </row>
+    <row r="277" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A277">
+        <f t="shared" si="4"/>
+        <v>276</v>
+      </c>
+      <c r="B277">
+        <v>27</v>
+      </c>
+      <c r="C277" s="3">
+        <v>46224.401388888888</v>
+      </c>
+      <c r="D277" t="s">
+        <v>63</v>
+      </c>
+      <c r="E277" t="s">
+        <v>63</v>
+      </c>
+      <c r="F277" s="6">
+        <v>1.40625E-2</v>
+      </c>
+    </row>
+    <row r="278" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A278">
+        <f t="shared" si="4"/>
+        <v>277</v>
+      </c>
+      <c r="B278">
+        <v>27</v>
+      </c>
+      <c r="C278" s="3">
+        <v>46224.45</v>
+      </c>
+      <c r="D278" t="s">
+        <v>63</v>
+      </c>
+      <c r="E278" t="s">
+        <v>63</v>
+      </c>
+      <c r="F278" s="6">
+        <v>6.6087962962962966E-3</v>
+      </c>
+    </row>
+    <row r="279" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A279">
+        <f t="shared" si="4"/>
+        <v>278</v>
+      </c>
+      <c r="B279">
+        <v>28</v>
+      </c>
+      <c r="C279" s="3">
+        <v>46224.921527777777</v>
+      </c>
+      <c r="D279">
+        <v>1</v>
+      </c>
+      <c r="E279">
+        <v>20</v>
+      </c>
+      <c r="F279" s="6">
+        <v>1.0034722222222223E-2</v>
+      </c>
+    </row>
+    <row r="280" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A280">
+        <f t="shared" si="4"/>
+        <v>279</v>
+      </c>
+      <c r="B280">
+        <v>28</v>
+      </c>
+      <c r="C280" s="3">
+        <v>46225.704861111109</v>
+      </c>
+      <c r="D280">
+        <v>20</v>
+      </c>
+      <c r="E280">
+        <v>50</v>
+      </c>
+      <c r="F280" s="6">
+        <v>1.4363425925925925E-2</v>
+      </c>
+    </row>
+    <row r="281" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A281">
+        <f t="shared" si="4"/>
+        <v>280</v>
+      </c>
+      <c r="B281">
+        <v>28</v>
+      </c>
+      <c r="C281" s="3">
+        <v>46225.784722222219</v>
+      </c>
+      <c r="D281">
+        <v>50</v>
+      </c>
+      <c r="E281">
+        <v>72</v>
+      </c>
+      <c r="F281" s="6">
+        <v>1.1666666666666667E-2</v>
+      </c>
+    </row>
+    <row r="282" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A282">
+        <f t="shared" si="4"/>
+        <v>281</v>
+      </c>
+      <c r="B282">
+        <v>28</v>
+      </c>
+      <c r="C282" s="3">
+        <v>46225.885416666664</v>
+      </c>
+      <c r="D282">
+        <v>72</v>
+      </c>
+      <c r="E282">
+        <v>99</v>
+      </c>
+      <c r="F282" s="6">
+        <v>1.2789351851851852E-2</v>
+      </c>
+    </row>
+    <row r="283" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A283">
+        <f t="shared" si="4"/>
+        <v>282</v>
+      </c>
+      <c r="B283">
+        <v>28</v>
+      </c>
+      <c r="C283" s="3">
+        <v>46226.615277777775</v>
+      </c>
+      <c r="D283">
+        <v>99</v>
+      </c>
+      <c r="E283">
+        <v>152</v>
+      </c>
+      <c r="F283" s="6">
+        <v>2.3842592592592592E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>